<commit_message>
Highlight missing Exec Names in red and fill with N/A
https://claude.ai/code/session_01917JoB1LXoWCAoYuucjGiV
</commit_message>
<xml_diff>
--- a/Womens_HRT_Hormones_Only_New_cleaned_updated.xlsx
+++ b/Womens_HRT_Hormones_Only_New_cleaned_updated.xlsx
@@ -26,12 +26,18 @@
       <scheme val="minor"/>
     </font>
   </fonts>
-  <fills count="2">
+  <fills count="3">
     <fill>
       <patternFill/>
     </fill>
     <fill>
       <patternFill patternType="gray125"/>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00FF0000"/>
+        <bgColor rgb="00FF0000"/>
+      </patternFill>
     </fill>
   </fills>
   <borders count="1">
@@ -46,8 +52,9 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="1">
+  <cellXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -562,7 +569,6 @@
           <t>data-only</t>
         </is>
       </c>
-      <c r="C2" t="inlineStr"/>
       <c r="D2" t="inlineStr">
         <is>
           <t>Pure-play hormone/TRT/HRT or longevity practice</t>
@@ -613,8 +619,6 @@
           <t>President</t>
         </is>
       </c>
-      <c r="N2" t="inlineStr"/>
-      <c r="O2" t="inlineStr"/>
       <c r="P2" t="n">
         <v>5</v>
       </c>
@@ -650,7 +654,6 @@
           <t>Core hormone/longevity practice — 3 hormone service signals, prescriber-led</t>
         </is>
       </c>
-      <c r="AA2" t="inlineStr"/>
     </row>
     <row r="3">
       <c r="A3" t="n">
@@ -661,7 +664,6 @@
           <t>data-only</t>
         </is>
       </c>
-      <c r="C3" t="inlineStr"/>
       <c r="D3" t="inlineStr">
         <is>
           <t>Pure-play hormone/TRT/HRT or longevity practice</t>
@@ -712,7 +714,6 @@
           <t>Owner</t>
         </is>
       </c>
-      <c r="N3" t="inlineStr"/>
       <c r="O3" t="inlineStr">
         <is>
           <t>https://www.linkedin.com/company/ocsportsandwellnessca/</t>
@@ -753,7 +754,6 @@
           <t>Core hormone/longevity practice — 3 hormone service signals, prescriber-led</t>
         </is>
       </c>
-      <c r="AA3" t="inlineStr"/>
     </row>
     <row r="4">
       <c r="A4" t="n">
@@ -764,7 +764,6 @@
           <t>data-only</t>
         </is>
       </c>
-      <c r="C4" t="inlineStr"/>
       <c r="D4" t="inlineStr">
         <is>
           <t>Pure-play hormone/TRT/HRT or longevity practice</t>
@@ -810,8 +809,6 @@
           <t>Antoinette Jackson-Sekunda</t>
         </is>
       </c>
-      <c r="M4" t="inlineStr"/>
-      <c r="N4" t="inlineStr"/>
       <c r="O4" t="inlineStr">
         <is>
           <t>https://www.linkedin.com/company/bff-medical-wellness-clinic/</t>
@@ -829,7 +826,6 @@
       <c r="S4" t="n">
         <v>3</v>
       </c>
-      <c r="T4" t="inlineStr"/>
       <c r="U4" t="n">
         <v>240000</v>
       </c>
@@ -850,7 +846,6 @@
           <t>Mixed practice — hormone services present alongside 0 aesthetic and 0 weight-loss signals</t>
         </is>
       </c>
-      <c r="AA4" t="inlineStr"/>
     </row>
     <row r="5">
       <c r="A5" t="n">
@@ -861,7 +856,6 @@
           <t>data-only</t>
         </is>
       </c>
-      <c r="C5" t="inlineStr"/>
       <c r="D5" t="inlineStr">
         <is>
           <t>Pure-play hormone/TRT/HRT or longevity practice</t>
@@ -912,8 +906,6 @@
           <t>Founder,</t>
         </is>
       </c>
-      <c r="N5" t="inlineStr"/>
-      <c r="O5" t="inlineStr"/>
       <c r="P5" t="n">
         <v>4.6</v>
       </c>
@@ -926,7 +918,6 @@
       <c r="S5" t="n">
         <v>1</v>
       </c>
-      <c r="T5" t="inlineStr"/>
       <c r="U5" t="n">
         <v>720000</v>
       </c>
@@ -947,7 +938,6 @@
           <t>Core hormone/longevity practice — 4 hormone service signals, prescriber-led</t>
         </is>
       </c>
-      <c r="AA5" t="inlineStr"/>
     </row>
     <row r="6">
       <c r="A6" t="n">
@@ -958,7 +948,6 @@
           <t>data-only</t>
         </is>
       </c>
-      <c r="C6" t="inlineStr"/>
       <c r="D6" t="inlineStr">
         <is>
           <t>Pure-play hormone/TRT/HRT or longevity practice</t>
@@ -1004,9 +993,6 @@
           <t>Chris Potter</t>
         </is>
       </c>
-      <c r="M6" t="inlineStr"/>
-      <c r="N6" t="inlineStr"/>
-      <c r="O6" t="inlineStr"/>
       <c r="P6" t="n">
         <v>5</v>
       </c>
@@ -1019,7 +1005,6 @@
       <c r="S6" t="n">
         <v>5</v>
       </c>
-      <c r="T6" t="inlineStr"/>
       <c r="U6" t="n">
         <v>144000</v>
       </c>
@@ -1055,7 +1040,6 @@
           <t>data-only</t>
         </is>
       </c>
-      <c r="C7" t="inlineStr"/>
       <c r="D7" t="inlineStr">
         <is>
           <t>Pure-play hormone/TRT/HRT or longevity practice</t>
@@ -1101,9 +1085,6 @@
           <t>Kathryn Houston</t>
         </is>
       </c>
-      <c r="M7" t="inlineStr"/>
-      <c r="N7" t="inlineStr"/>
-      <c r="O7" t="inlineStr"/>
       <c r="P7" t="n">
         <v>4.9</v>
       </c>
@@ -1116,7 +1097,6 @@
       <c r="S7" t="n">
         <v>3</v>
       </c>
-      <c r="T7" t="inlineStr"/>
       <c r="U7" t="n">
         <v>288000</v>
       </c>
@@ -1152,7 +1132,6 @@
           <t>data-only</t>
         </is>
       </c>
-      <c r="C8" t="inlineStr"/>
       <c r="D8" t="inlineStr">
         <is>
           <t>Pure-play hormone/TRT/HRT or longevity practice</t>
@@ -1208,7 +1187,6 @@
           <t>beautymd.us@gmail.com</t>
         </is>
       </c>
-      <c r="O8" t="inlineStr"/>
       <c r="P8" t="n">
         <v>5</v>
       </c>
@@ -1221,7 +1199,6 @@
       <c r="S8" t="n">
         <v>1</v>
       </c>
-      <c r="T8" t="inlineStr"/>
       <c r="U8" t="n">
         <v>144000</v>
       </c>
@@ -1242,7 +1219,6 @@
           <t>Solid hormone line (TRT/HRT focus in name/type) but mixed with other services</t>
         </is>
       </c>
-      <c r="AA8" t="inlineStr"/>
     </row>
     <row r="9">
       <c r="A9" t="n">
@@ -1253,7 +1229,6 @@
           <t>data-only</t>
         </is>
       </c>
-      <c r="C9" t="inlineStr"/>
       <c r="D9" t="inlineStr">
         <is>
           <t>Pure-play hormone/TRT/HRT or longevity practice</t>
@@ -1284,7 +1259,6 @@
           <t>elevateherhealth.com</t>
         </is>
       </c>
-      <c r="J9" t="inlineStr"/>
       <c r="K9" t="inlineStr">
         <is>
           <t>508 Brinkerhoff Ave</t>
@@ -1305,7 +1279,6 @@
           <t>sam@elevateherhealth.com</t>
         </is>
       </c>
-      <c r="O9" t="inlineStr"/>
       <c r="P9" t="n">
         <v>5</v>
       </c>
@@ -1318,7 +1291,6 @@
       <c r="S9" t="n">
         <v>15</v>
       </c>
-      <c r="T9" t="inlineStr"/>
       <c r="U9" t="n">
         <v>144000</v>
       </c>
@@ -1339,7 +1311,6 @@
           <t>Some hormone presence but not the clear focus</t>
         </is>
       </c>
-      <c r="AA9" t="inlineStr"/>
     </row>
     <row r="10">
       <c r="A10" t="n">
@@ -1350,7 +1321,6 @@
           <t>data-only</t>
         </is>
       </c>
-      <c r="C10" t="inlineStr"/>
       <c r="D10" t="inlineStr">
         <is>
           <t>Pure-play hormone/TRT/HRT or longevity practice</t>
@@ -1446,7 +1416,6 @@
           <t>Some hormone presence but not the clear focus</t>
         </is>
       </c>
-      <c r="AA10" t="inlineStr"/>
     </row>
     <row r="11">
       <c r="A11" t="n">
@@ -1457,7 +1426,6 @@
           <t>data-only</t>
         </is>
       </c>
-      <c r="C11" t="inlineStr"/>
       <c r="D11" t="inlineStr">
         <is>
           <t>Pure-play hormone/TRT/HRT or longevity practice</t>
@@ -1508,7 +1476,6 @@
           <t>Owner</t>
         </is>
       </c>
-      <c r="N11" t="inlineStr"/>
       <c r="O11" t="inlineStr">
         <is>
           <t>https://www.linkedin.com/company/akasha-center-for-integrative-medicine/</t>
@@ -1549,7 +1516,6 @@
           <t>Some hormone presence but not the clear focus</t>
         </is>
       </c>
-      <c r="AA11" t="inlineStr"/>
     </row>
     <row r="12">
       <c r="A12" t="n">
@@ -1560,7 +1526,6 @@
           <t>data-only</t>
         </is>
       </c>
-      <c r="C12" t="inlineStr"/>
       <c r="D12" t="inlineStr">
         <is>
           <t>Pure-play hormone/TRT/HRT or longevity practice</t>
@@ -1656,7 +1621,6 @@
           <t>Some hormone presence but not the clear focus</t>
         </is>
       </c>
-      <c r="AA12" t="inlineStr"/>
     </row>
     <row r="13">
       <c r="A13" t="n">
@@ -1667,7 +1631,6 @@
           <t>data-only</t>
         </is>
       </c>
-      <c r="C13" t="inlineStr"/>
       <c r="D13" t="inlineStr">
         <is>
           <t>Pure-play hormone/TRT/HRT or longevity practice</t>
@@ -1763,7 +1726,6 @@
           <t>Some hormone presence but not the clear focus</t>
         </is>
       </c>
-      <c r="AA13" t="inlineStr"/>
     </row>
     <row r="14">
       <c r="A14" t="n">
@@ -1774,7 +1736,6 @@
           <t>data-only</t>
         </is>
       </c>
-      <c r="C14" t="inlineStr"/>
       <c r="D14" t="inlineStr">
         <is>
           <t>Pure-play hormone/TRT/HRT or longevity practice</t>
@@ -1820,9 +1781,6 @@
           <t>Yasmine Perdue</t>
         </is>
       </c>
-      <c r="M14" t="inlineStr"/>
-      <c r="N14" t="inlineStr"/>
-      <c r="O14" t="inlineStr"/>
       <c r="P14" t="n">
         <v>5</v>
       </c>
@@ -1835,7 +1793,6 @@
       <c r="S14" t="n">
         <v>1</v>
       </c>
-      <c r="T14" t="inlineStr"/>
       <c r="U14" t="n">
         <v>144000</v>
       </c>
@@ -1856,7 +1813,6 @@
           <t>Core hormone/longevity practice — 3 hormone service signals, prescriber-led</t>
         </is>
       </c>
-      <c r="AA14" t="inlineStr"/>
     </row>
     <row r="15">
       <c r="A15" t="n">
@@ -1867,7 +1823,6 @@
           <t>data-only</t>
         </is>
       </c>
-      <c r="C15" t="inlineStr"/>
       <c r="D15" t="inlineStr">
         <is>
           <t>Pure-play hormone/TRT/HRT or longevity practice</t>
@@ -1908,10 +1863,11 @@
           <t>8127 Mulberry Ave Ste 108</t>
         </is>
       </c>
-      <c r="L15" t="inlineStr"/>
-      <c r="M15" t="inlineStr"/>
-      <c r="N15" t="inlineStr"/>
-      <c r="O15" t="inlineStr"/>
+      <c r="L15" s="1" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
       <c r="P15" t="n">
         <v>4.9</v>
       </c>
@@ -1924,7 +1880,6 @@
       <c r="S15" t="n">
         <v>1</v>
       </c>
-      <c r="T15" t="inlineStr"/>
       <c r="U15" t="n">
         <v>144000</v>
       </c>
@@ -1945,7 +1900,6 @@
           <t>Some hormone presence but not the clear focus</t>
         </is>
       </c>
-      <c r="AA15" t="inlineStr"/>
     </row>
     <row r="16">
       <c r="A16" t="n">
@@ -1956,7 +1910,6 @@
           <t>data-only</t>
         </is>
       </c>
-      <c r="C16" t="inlineStr"/>
       <c r="D16" t="inlineStr">
         <is>
           <t>Pure-play hormone/TRT/HRT or longevity practice</t>
@@ -2029,7 +1982,6 @@
       <c r="S16" t="n">
         <v>1</v>
       </c>
-      <c r="T16" t="inlineStr"/>
       <c r="U16" t="n">
         <v>144000</v>
       </c>
@@ -2050,7 +2002,6 @@
           <t>Some hormone presence but not the clear focus</t>
         </is>
       </c>
-      <c r="AA16" t="inlineStr"/>
     </row>
     <row r="17">
       <c r="A17" t="n">
@@ -2061,7 +2012,6 @@
           <t>data-only</t>
         </is>
       </c>
-      <c r="C17" t="inlineStr"/>
       <c r="D17" t="inlineStr">
         <is>
           <t>Pure-play hormone/TRT/HRT or longevity practice</t>
@@ -2107,9 +2057,6 @@
           <t>Sharone Utter</t>
         </is>
       </c>
-      <c r="M17" t="inlineStr"/>
-      <c r="N17" t="inlineStr"/>
-      <c r="O17" t="inlineStr"/>
       <c r="P17" t="n">
         <v>4.8</v>
       </c>
@@ -2122,7 +2069,6 @@
       <c r="S17" t="n">
         <v>1</v>
       </c>
-      <c r="T17" t="inlineStr"/>
       <c r="U17" t="n">
         <v>144000</v>
       </c>
@@ -2143,7 +2089,6 @@
           <t>Some hormone presence but not the clear focus</t>
         </is>
       </c>
-      <c r="AA17" t="inlineStr"/>
     </row>
     <row r="18">
       <c r="A18" t="n">
@@ -2154,7 +2099,6 @@
           <t>data-only</t>
         </is>
       </c>
-      <c r="C18" t="inlineStr"/>
       <c r="D18" t="inlineStr">
         <is>
           <t>Pure-play hormone/TRT/HRT or longevity practice</t>
@@ -2200,9 +2144,6 @@
           <t>Marc Kaufman</t>
         </is>
       </c>
-      <c r="M18" t="inlineStr"/>
-      <c r="N18" t="inlineStr"/>
-      <c r="O18" t="inlineStr"/>
       <c r="P18" t="n">
         <v>5</v>
       </c>
@@ -2215,7 +2156,6 @@
       <c r="S18" t="n">
         <v>1</v>
       </c>
-      <c r="T18" t="inlineStr"/>
       <c r="U18" t="n">
         <v>195000</v>
       </c>
@@ -2251,7 +2191,6 @@
           <t>data-only</t>
         </is>
       </c>
-      <c r="C19" t="inlineStr"/>
       <c r="D19" t="inlineStr">
         <is>
           <t>Pure-play hormone/TRT/HRT or longevity practice</t>
@@ -2297,9 +2236,6 @@
           <t>Van Nguyen</t>
         </is>
       </c>
-      <c r="M19" t="inlineStr"/>
-      <c r="N19" t="inlineStr"/>
-      <c r="O19" t="inlineStr"/>
       <c r="P19" t="n">
         <v>4.8</v>
       </c>
@@ -2312,7 +2248,6 @@
       <c r="S19" t="n">
         <v>1</v>
       </c>
-      <c r="T19" t="inlineStr"/>
       <c r="U19" t="n">
         <v>86400</v>
       </c>
@@ -2348,7 +2283,6 @@
           <t>data-only</t>
         </is>
       </c>
-      <c r="C20" t="inlineStr"/>
       <c r="D20" t="inlineStr">
         <is>
           <t>Pure-play hormone/TRT/HRT or longevity practice</t>
@@ -2389,10 +2323,11 @@
           <t>14115 S Dixie Hwy SUITE H, Palmetto Bay, FL 33176, USA</t>
         </is>
       </c>
-      <c r="L20" t="inlineStr"/>
-      <c r="M20" t="inlineStr"/>
-      <c r="N20" t="inlineStr"/>
-      <c r="O20" t="inlineStr"/>
+      <c r="L20" s="1" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
       <c r="P20" t="n">
         <v>5</v>
       </c>
@@ -2405,7 +2340,6 @@
       <c r="S20" t="n">
         <v>1</v>
       </c>
-      <c r="T20" t="inlineStr"/>
       <c r="U20" t="n">
         <v>95400</v>
       </c>
@@ -2441,7 +2375,6 @@
           <t>data-only</t>
         </is>
       </c>
-      <c r="C21" t="inlineStr"/>
       <c r="D21" t="inlineStr">
         <is>
           <t>Pure-play hormone/TRT/HRT or longevity practice</t>
@@ -2487,9 +2420,6 @@
           <t>Yazan Abdullah</t>
         </is>
       </c>
-      <c r="M21" t="inlineStr"/>
-      <c r="N21" t="inlineStr"/>
-      <c r="O21" t="inlineStr"/>
       <c r="P21" t="n">
         <v>4.8</v>
       </c>
@@ -2502,7 +2432,6 @@
       <c r="S21" t="n">
         <v>1</v>
       </c>
-      <c r="T21" t="inlineStr"/>
       <c r="U21" t="n">
         <v>144000</v>
       </c>
@@ -2523,7 +2452,6 @@
           <t>Some hormone presence but not the clear focus</t>
         </is>
       </c>
-      <c r="AA21" t="inlineStr"/>
     </row>
     <row r="22">
       <c r="A22" t="n">
@@ -2534,7 +2462,6 @@
           <t>data-only</t>
         </is>
       </c>
-      <c r="C22" t="inlineStr"/>
       <c r="D22" t="inlineStr">
         <is>
           <t>Pure-play hormone/TRT/HRT or longevity practice</t>
@@ -2580,9 +2507,6 @@
           <t>Ojen Masrour</t>
         </is>
       </c>
-      <c r="M22" t="inlineStr"/>
-      <c r="N22" t="inlineStr"/>
-      <c r="O22" t="inlineStr"/>
       <c r="P22" t="n">
         <v>4.2</v>
       </c>
@@ -2595,7 +2519,6 @@
       <c r="S22" t="n">
         <v>1</v>
       </c>
-      <c r="T22" t="inlineStr"/>
       <c r="U22" t="n">
         <v>111600</v>
       </c>
@@ -2616,7 +2539,6 @@
           <t>Some hormone presence but not the clear focus</t>
         </is>
       </c>
-      <c r="AA22" t="inlineStr"/>
     </row>
     <row r="23">
       <c r="A23" t="n">
@@ -2627,7 +2549,6 @@
           <t>data-only</t>
         </is>
       </c>
-      <c r="C23" t="inlineStr"/>
       <c r="D23" t="inlineStr">
         <is>
           <t>Pure-play hormone/TRT/HRT or longevity practice</t>
@@ -2673,9 +2594,6 @@
           <t>Melissa Kemp</t>
         </is>
       </c>
-      <c r="M23" t="inlineStr"/>
-      <c r="N23" t="inlineStr"/>
-      <c r="O23" t="inlineStr"/>
       <c r="P23" t="n">
         <v>5</v>
       </c>
@@ -2688,7 +2606,6 @@
       <c r="S23" t="n">
         <v>1</v>
       </c>
-      <c r="T23" t="inlineStr"/>
       <c r="U23" t="n">
         <v>144000</v>
       </c>
@@ -2724,7 +2641,6 @@
           <t>data-only</t>
         </is>
       </c>
-      <c r="C24" t="inlineStr"/>
       <c r="D24" t="inlineStr">
         <is>
           <t>Pure-play hormone/TRT/HRT or longevity practice</t>
@@ -2770,9 +2686,6 @@
           <t>Thom Lobe</t>
         </is>
       </c>
-      <c r="M24" t="inlineStr"/>
-      <c r="N24" t="inlineStr"/>
-      <c r="O24" t="inlineStr"/>
       <c r="P24" t="n">
         <v>4.5</v>
       </c>
@@ -2785,7 +2698,6 @@
       <c r="S24" t="n">
         <v>1</v>
       </c>
-      <c r="T24" t="inlineStr"/>
       <c r="U24" t="n">
         <v>108000</v>
       </c>
@@ -2806,7 +2718,6 @@
           <t>Some hormone presence but not the clear focus</t>
         </is>
       </c>
-      <c r="AA24" t="inlineStr"/>
     </row>
     <row r="25">
       <c r="A25" t="n">
@@ -2817,7 +2728,6 @@
           <t>data-only</t>
         </is>
       </c>
-      <c r="C25" t="inlineStr"/>
       <c r="D25" t="inlineStr">
         <is>
           <t>Pure-play hormone/TRT/HRT or longevity practice</t>
@@ -2863,9 +2773,6 @@
           <t>Devon Casida</t>
         </is>
       </c>
-      <c r="M25" t="inlineStr"/>
-      <c r="N25" t="inlineStr"/>
-      <c r="O25" t="inlineStr"/>
       <c r="P25" t="n">
         <v>5</v>
       </c>
@@ -2878,7 +2785,6 @@
       <c r="S25" t="n">
         <v>1</v>
       </c>
-      <c r="T25" t="inlineStr"/>
       <c r="U25" t="n">
         <v>216000</v>
       </c>
@@ -2914,7 +2820,6 @@
           <t>data-only</t>
         </is>
       </c>
-      <c r="C26" t="inlineStr"/>
       <c r="D26" t="inlineStr">
         <is>
           <t>Pure-play hormone/TRT/HRT or longevity practice</t>
@@ -2960,9 +2865,6 @@
           <t>Jennifer Davis</t>
         </is>
       </c>
-      <c r="M26" t="inlineStr"/>
-      <c r="N26" t="inlineStr"/>
-      <c r="O26" t="inlineStr"/>
       <c r="P26" t="n">
         <v>4.9</v>
       </c>
@@ -2975,7 +2877,6 @@
       <c r="S26" t="n">
         <v>1</v>
       </c>
-      <c r="T26" t="inlineStr"/>
       <c r="U26" t="n">
         <v>240000</v>
       </c>
@@ -3011,7 +2912,6 @@
           <t>data-only</t>
         </is>
       </c>
-      <c r="C27" t="inlineStr"/>
       <c r="D27" t="inlineStr">
         <is>
           <t>Pure-play hormone/TRT/HRT or longevity practice</t>
@@ -3057,9 +2957,6 @@
           <t>Matthew Risner</t>
         </is>
       </c>
-      <c r="M27" t="inlineStr"/>
-      <c r="N27" t="inlineStr"/>
-      <c r="O27" t="inlineStr"/>
       <c r="P27" t="n">
         <v>5</v>
       </c>
@@ -3072,7 +2969,6 @@
       <c r="S27" t="n">
         <v>1</v>
       </c>
-      <c r="T27" t="inlineStr"/>
       <c r="U27" t="n">
         <v>240000</v>
       </c>
@@ -3108,7 +3004,6 @@
           <t>data-only</t>
         </is>
       </c>
-      <c r="C28" t="inlineStr"/>
       <c r="D28" t="inlineStr">
         <is>
           <t>Pure-play hormone/TRT/HRT or longevity practice</t>
@@ -3154,9 +3049,6 @@
           <t>Joseph Aiello</t>
         </is>
       </c>
-      <c r="M28" t="inlineStr"/>
-      <c r="N28" t="inlineStr"/>
-      <c r="O28" t="inlineStr"/>
       <c r="P28" t="n">
         <v>4.9</v>
       </c>
@@ -3192,7 +3084,6 @@
           <t>Some hormone presence but not the clear focus</t>
         </is>
       </c>
-      <c r="AA28" t="inlineStr"/>
     </row>
     <row r="29">
       <c r="A29" t="n">
@@ -3253,9 +3144,6 @@
           <t>Pamela Gaudry</t>
         </is>
       </c>
-      <c r="M29" t="inlineStr"/>
-      <c r="N29" t="inlineStr"/>
-      <c r="O29" t="inlineStr"/>
       <c r="P29" t="n">
         <v>4.7</v>
       </c>
@@ -3268,7 +3156,6 @@
       <c r="S29" t="n">
         <v>2</v>
       </c>
-      <c r="T29" t="inlineStr"/>
       <c r="U29" t="n">
         <v>489000</v>
       </c>
@@ -3304,7 +3191,6 @@
           <t>data-only</t>
         </is>
       </c>
-      <c r="C30" t="inlineStr"/>
       <c r="D30" t="inlineStr">
         <is>
           <t>Pure-play hormone/TRT/HRT or longevity practice</t>
@@ -3350,9 +3236,6 @@
           <t>Cally Smith</t>
         </is>
       </c>
-      <c r="M30" t="inlineStr"/>
-      <c r="N30" t="inlineStr"/>
-      <c r="O30" t="inlineStr"/>
       <c r="P30" t="n">
         <v>5</v>
       </c>
@@ -3365,7 +3248,6 @@
       <c r="S30" t="n">
         <v>1</v>
       </c>
-      <c r="T30" t="inlineStr"/>
       <c r="U30" t="n">
         <v>240000</v>
       </c>
@@ -3446,10 +3328,11 @@
           <t>3405 Dallas Hwy Suite 200, Marietta, GA 30064, USA</t>
         </is>
       </c>
-      <c r="L31" t="inlineStr"/>
-      <c r="M31" t="inlineStr"/>
-      <c r="N31" t="inlineStr"/>
-      <c r="O31" t="inlineStr"/>
+      <c r="L31" s="1" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
       <c r="P31" t="n">
         <v>4.8</v>
       </c>
@@ -3500,7 +3383,6 @@
           <t>data-only</t>
         </is>
       </c>
-      <c r="C32" t="inlineStr"/>
       <c r="D32" t="inlineStr">
         <is>
           <t>Pure-play hormone/TRT/HRT or longevity practice</t>
@@ -3546,9 +3428,6 @@
           <t>Vahe Melikyan</t>
         </is>
       </c>
-      <c r="M32" t="inlineStr"/>
-      <c r="N32" t="inlineStr"/>
-      <c r="O32" t="inlineStr"/>
       <c r="P32" t="n">
         <v>5</v>
       </c>
@@ -3599,7 +3478,6 @@
           <t>data-only</t>
         </is>
       </c>
-      <c r="C33" t="inlineStr"/>
       <c r="D33" t="inlineStr">
         <is>
           <t>Pure-play hormone/TRT/HRT or longevity practice</t>
@@ -3645,9 +3523,6 @@
           <t>Reem Sharhan</t>
         </is>
       </c>
-      <c r="M33" t="inlineStr"/>
-      <c r="N33" t="inlineStr"/>
-      <c r="O33" t="inlineStr"/>
       <c r="P33" t="n">
         <v>5</v>
       </c>
@@ -3660,7 +3535,6 @@
       <c r="S33" t="n">
         <v>1</v>
       </c>
-      <c r="T33" t="inlineStr"/>
       <c r="U33" t="n">
         <v>150000</v>
       </c>
@@ -3696,7 +3570,6 @@
           <t>data-only</t>
         </is>
       </c>
-      <c r="C34" t="inlineStr"/>
       <c r="D34" t="inlineStr">
         <is>
           <t>Pure-play hormone/TRT/HRT or longevity practice</t>
@@ -3737,10 +3610,11 @@
           <t>90 W Main St, Victor, NY 14564, USA</t>
         </is>
       </c>
-      <c r="L34" t="inlineStr"/>
-      <c r="M34" t="inlineStr"/>
-      <c r="N34" t="inlineStr"/>
-      <c r="O34" t="inlineStr"/>
+      <c r="L34" s="1" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
       <c r="P34" t="n">
         <v>5</v>
       </c>
@@ -3753,7 +3627,6 @@
       <c r="S34" t="n">
         <v>1</v>
       </c>
-      <c r="T34" t="inlineStr"/>
       <c r="U34" t="n">
         <v>120600</v>
       </c>
@@ -3789,7 +3662,6 @@
           <t>data-only</t>
         </is>
       </c>
-      <c r="C35" t="inlineStr"/>
       <c r="D35" t="inlineStr">
         <is>
           <t>Pure-play hormone/TRT/HRT or longevity practice</t>
@@ -3815,7 +3687,6 @@
           <t>Garland</t>
         </is>
       </c>
-      <c r="I35" t="inlineStr"/>
       <c r="J35" t="inlineStr">
         <is>
           <t>(469) 461-7044</t>
@@ -3826,10 +3697,11 @@
           <t>1529 E Interstate 30 #108, Garland, TX 75043, USA</t>
         </is>
       </c>
-      <c r="L35" t="inlineStr"/>
-      <c r="M35" t="inlineStr"/>
-      <c r="N35" t="inlineStr"/>
-      <c r="O35" t="inlineStr"/>
+      <c r="L35" s="1" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
       <c r="P35" t="n">
         <v>5</v>
       </c>
@@ -3842,7 +3714,6 @@
       <c r="S35" t="n">
         <v>1</v>
       </c>
-      <c r="T35" t="inlineStr"/>
       <c r="U35" t="n">
         <v>144000</v>
       </c>
@@ -3928,9 +3799,6 @@
           <t>Heather Bartos</t>
         </is>
       </c>
-      <c r="M36" t="inlineStr"/>
-      <c r="N36" t="inlineStr"/>
-      <c r="O36" t="inlineStr"/>
       <c r="P36" t="n">
         <v>4.5</v>
       </c>
@@ -3943,7 +3811,6 @@
       <c r="S36" t="n">
         <v>1</v>
       </c>
-      <c r="T36" t="inlineStr"/>
       <c r="U36" t="n">
         <v>240000</v>
       </c>
@@ -4029,9 +3896,6 @@
           <t>John Gomes</t>
         </is>
       </c>
-      <c r="M37" t="inlineStr"/>
-      <c r="N37" t="inlineStr"/>
-      <c r="O37" t="inlineStr"/>
       <c r="P37" t="n">
         <v>4.9</v>
       </c>
@@ -4132,9 +3996,6 @@
           <t>Jennifer Wright-Bennion</t>
         </is>
       </c>
-      <c r="M38" t="inlineStr"/>
-      <c r="N38" t="inlineStr"/>
-      <c r="O38" t="inlineStr"/>
       <c r="P38" t="n">
         <v>4</v>
       </c>
@@ -4147,7 +4008,6 @@
       <c r="S38" t="n">
         <v>4</v>
       </c>
-      <c r="T38" t="inlineStr"/>
       <c r="U38" t="n">
         <v>240000</v>
       </c>
@@ -4233,9 +4093,6 @@
           <t>Larissa Fomitcheva</t>
         </is>
       </c>
-      <c r="M39" t="inlineStr"/>
-      <c r="N39" t="inlineStr"/>
-      <c r="O39" t="inlineStr"/>
       <c r="P39" t="n">
         <v>4.7</v>
       </c>
@@ -4248,7 +4105,6 @@
       <c r="S39" t="n">
         <v>1</v>
       </c>
-      <c r="T39" t="inlineStr"/>
       <c r="U39" t="n">
         <v>720000</v>
       </c>
@@ -4269,7 +4125,6 @@
           <t>No hormone, aesthetic, or weight-loss signals detected — may need manual review</t>
         </is>
       </c>
-      <c r="AA39" t="inlineStr"/>
     </row>
     <row r="40">
       <c r="A40" t="n">
@@ -4330,9 +4185,6 @@
           <t>Kourtney Sims</t>
         </is>
       </c>
-      <c r="M40" t="inlineStr"/>
-      <c r="N40" t="inlineStr"/>
-      <c r="O40" t="inlineStr"/>
       <c r="P40" t="n">
         <v>4.8</v>
       </c>
@@ -4345,7 +4197,6 @@
       <c r="S40" t="n">
         <v>2</v>
       </c>
-      <c r="T40" t="inlineStr"/>
       <c r="U40" t="n">
         <v>240000</v>
       </c>
@@ -4441,7 +4292,6 @@
           <t>anna.barbieri@annabarbieri-md.com</t>
         </is>
       </c>
-      <c r="O41" t="inlineStr"/>
       <c r="P41" t="n">
         <v>4.9</v>
       </c>
@@ -4454,7 +4304,6 @@
       <c r="S41" t="n">
         <v>1</v>
       </c>
-      <c r="T41" t="inlineStr"/>
       <c r="U41" t="n">
         <v>720000</v>
       </c>
@@ -4475,7 +4324,6 @@
           <t>No hormone, aesthetic, or weight-loss signals detected — may need manual review</t>
         </is>
       </c>
-      <c r="AA41" t="inlineStr"/>
     </row>
     <row r="42">
       <c r="A42" t="n">
@@ -4511,7 +4359,6 @@
           <t>NY</t>
         </is>
       </c>
-      <c r="H42" t="inlineStr"/>
       <c r="I42" t="inlineStr">
         <is>
           <t>http://www.trustwomenshealthcare.com/</t>
@@ -4532,9 +4379,6 @@
           <t>Peggy Margetson</t>
         </is>
       </c>
-      <c r="M42" t="inlineStr"/>
-      <c r="N42" t="inlineStr"/>
-      <c r="O42" t="inlineStr"/>
       <c r="P42" t="n">
         <v>4.5</v>
       </c>
@@ -4547,7 +4391,6 @@
       <c r="S42" t="n">
         <v>1</v>
       </c>
-      <c r="T42" t="inlineStr"/>
       <c r="U42" t="n">
         <v>240000</v>
       </c>
@@ -4633,9 +4476,6 @@
           <t>Kate</t>
         </is>
       </c>
-      <c r="M43" t="inlineStr"/>
-      <c r="N43" t="inlineStr"/>
-      <c r="O43" t="inlineStr"/>
       <c r="P43" t="n">
         <v>4.8</v>
       </c>
@@ -4648,7 +4488,6 @@
       <c r="S43" t="n">
         <v>1</v>
       </c>
-      <c r="T43" t="inlineStr"/>
       <c r="U43" t="n">
         <v>174000</v>
       </c>
@@ -4734,9 +4573,6 @@
           <t>Carolyn Moyers</t>
         </is>
       </c>
-      <c r="M44" t="inlineStr"/>
-      <c r="N44" t="inlineStr"/>
-      <c r="O44" t="inlineStr"/>
       <c r="P44" t="n">
         <v>4.9</v>
       </c>
@@ -4749,7 +4585,6 @@
       <c r="S44" t="n">
         <v>1</v>
       </c>
-      <c r="T44" t="inlineStr"/>
       <c r="U44" t="n">
         <v>240000</v>
       </c>
@@ -4830,10 +4665,11 @@
           <t>2460 N Interstate 35 E Rd Suite 165, Waxahachie, TX 75165, USA</t>
         </is>
       </c>
-      <c r="L45" t="inlineStr"/>
-      <c r="M45" t="inlineStr"/>
-      <c r="N45" t="inlineStr"/>
-      <c r="O45" t="inlineStr"/>
+      <c r="L45" s="1" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
       <c r="P45" t="n">
         <v>4.8</v>
       </c>
@@ -4929,10 +4765,11 @@
           <t>207 E 94th St 5th floor, New York, NY 10128, USA</t>
         </is>
       </c>
-      <c r="L46" t="inlineStr"/>
-      <c r="M46" t="inlineStr"/>
-      <c r="N46" t="inlineStr"/>
-      <c r="O46" t="inlineStr"/>
+      <c r="L46" s="1" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
       <c r="P46" t="n">
         <v>4.9</v>
       </c>
@@ -4945,7 +4782,6 @@
       <c r="S46" t="n">
         <v>3</v>
       </c>
-      <c r="T46" t="inlineStr"/>
       <c r="U46" t="n">
         <v>1680000</v>
       </c>
@@ -5031,9 +4867,6 @@
           <t>Laquita Martinez</t>
         </is>
       </c>
-      <c r="M47" t="inlineStr"/>
-      <c r="N47" t="inlineStr"/>
-      <c r="O47" t="inlineStr"/>
       <c r="P47" t="n">
         <v>4.6</v>
       </c>
@@ -5046,7 +4879,6 @@
       <c r="S47" t="n">
         <v>2</v>
       </c>
-      <c r="T47" t="inlineStr"/>
       <c r="U47" t="n">
         <v>720000</v>
       </c>
@@ -5127,10 +4959,11 @@
           <t>3237 Blue Ridge Rd, Raleigh, NC 27612, USA</t>
         </is>
       </c>
-      <c r="L48" t="inlineStr"/>
-      <c r="M48" t="inlineStr"/>
-      <c r="N48" t="inlineStr"/>
-      <c r="O48" t="inlineStr"/>
+      <c r="L48" s="1" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
       <c r="P48" t="n">
         <v>4.8</v>
       </c>
@@ -5143,7 +4976,6 @@
       <c r="S48" t="n">
         <v>11</v>
       </c>
-      <c r="T48" t="inlineStr"/>
       <c r="U48" t="n">
         <v>480000</v>
       </c>
@@ -5229,9 +5061,6 @@
           <t>Ann Cha</t>
         </is>
       </c>
-      <c r="M49" t="inlineStr"/>
-      <c r="N49" t="inlineStr"/>
-      <c r="O49" t="inlineStr"/>
       <c r="P49" t="n">
         <v>4.7</v>
       </c>
@@ -5244,7 +5073,6 @@
       <c r="S49" t="n">
         <v>4</v>
       </c>
-      <c r="T49" t="inlineStr"/>
       <c r="U49" t="n">
         <v>480000</v>
       </c>
@@ -5340,7 +5168,6 @@
           <t>nlamberty@aawomenshealth.com</t>
         </is>
       </c>
-      <c r="O50" t="inlineStr"/>
       <c r="P50" t="n">
         <v>4.2</v>
       </c>
@@ -5376,7 +5203,6 @@
           <t>No hormone, aesthetic, or weight-loss signals detected — may need manual review</t>
         </is>
       </c>
-      <c r="AA50" t="inlineStr"/>
     </row>
     <row r="51">
       <c r="A51" t="n">
@@ -5437,9 +5263,6 @@
           <t>Angela Hudson</t>
         </is>
       </c>
-      <c r="M51" t="inlineStr"/>
-      <c r="N51" t="inlineStr"/>
-      <c r="O51" t="inlineStr"/>
       <c r="P51" t="n">
         <v>4.9</v>
       </c>
@@ -5452,7 +5275,6 @@
       <c r="S51" t="n">
         <v>1</v>
       </c>
-      <c r="T51" t="inlineStr"/>
       <c r="U51" t="n">
         <v>240000</v>
       </c>
@@ -5533,10 +5355,11 @@
           <t>9940 Talbert Ave #303, Fountain Valley, CA 92708, USA</t>
         </is>
       </c>
-      <c r="L52" t="inlineStr"/>
-      <c r="M52" t="inlineStr"/>
-      <c r="N52" t="inlineStr"/>
-      <c r="O52" t="inlineStr"/>
+      <c r="L52" s="1" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
       <c r="P52" t="n">
         <v>4.4</v>
       </c>
@@ -5549,7 +5372,6 @@
       <c r="S52" t="n">
         <v>1</v>
       </c>
-      <c r="T52" t="inlineStr"/>
       <c r="U52" t="n">
         <v>561000</v>
       </c>
@@ -5630,10 +5452,11 @@
           <t>227 Riverstone Dr, Canton, GA 30114, USA</t>
         </is>
       </c>
-      <c r="L53" t="inlineStr"/>
-      <c r="M53" t="inlineStr"/>
-      <c r="N53" t="inlineStr"/>
-      <c r="O53" t="inlineStr"/>
+      <c r="L53" s="1" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
       <c r="P53" t="n">
         <v>4.6</v>
       </c>
@@ -5646,7 +5469,6 @@
       <c r="S53" t="n">
         <v>1</v>
       </c>
-      <c r="T53" t="inlineStr"/>
       <c r="U53" t="n">
         <v>240000</v>
       </c>
@@ -5732,9 +5554,6 @@
           <t>Drew Howard</t>
         </is>
       </c>
-      <c r="M54" t="inlineStr"/>
-      <c r="N54" t="inlineStr"/>
-      <c r="O54" t="inlineStr"/>
       <c r="P54" t="n">
         <v>4.8</v>
       </c>
@@ -5747,7 +5566,6 @@
       <c r="S54" t="n">
         <v>1</v>
       </c>
-      <c r="T54" t="inlineStr"/>
       <c r="U54" t="n">
         <v>240000</v>
       </c>
@@ -5828,10 +5646,11 @@
           <t>381 Deerfield Rd, Boone, NC 28607, USA</t>
         </is>
       </c>
-      <c r="L55" t="inlineStr"/>
-      <c r="M55" t="inlineStr"/>
-      <c r="N55" t="inlineStr"/>
-      <c r="O55" t="inlineStr"/>
+      <c r="L55" s="1" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
       <c r="P55" t="n">
         <v>4</v>
       </c>
@@ -5844,7 +5663,6 @@
       <c r="S55" t="n">
         <v>1</v>
       </c>
-      <c r="T55" t="inlineStr"/>
       <c r="U55" t="n">
         <v>240000</v>
       </c>
@@ -5925,10 +5743,11 @@
           <t>5161 Soquel Dr Ste C Floor 2, Soquel, CA 95073, USA</t>
         </is>
       </c>
-      <c r="L56" t="inlineStr"/>
-      <c r="M56" t="inlineStr"/>
-      <c r="N56" t="inlineStr"/>
-      <c r="O56" t="inlineStr"/>
+      <c r="L56" s="1" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
       <c r="P56" t="n">
         <v>5</v>
       </c>
@@ -5941,7 +5760,6 @@
       <c r="S56" t="n">
         <v>1</v>
       </c>
-      <c r="T56" t="inlineStr"/>
       <c r="U56" t="n">
         <v>240000</v>
       </c>
@@ -6022,10 +5840,11 @@
           <t>1875 Old Alabama Rd STE 210, Roswell, GA 30076, USA</t>
         </is>
       </c>
-      <c r="L57" t="inlineStr"/>
-      <c r="M57" t="inlineStr"/>
-      <c r="N57" t="inlineStr"/>
-      <c r="O57" t="inlineStr"/>
+      <c r="L57" s="1" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
       <c r="P57" t="n">
         <v>4.4</v>
       </c>
@@ -6038,7 +5857,6 @@
       <c r="S57" t="n">
         <v>2</v>
       </c>
-      <c r="T57" t="inlineStr"/>
       <c r="U57" t="n">
         <v>240000</v>
       </c>
@@ -6104,7 +5922,6 @@
           <t>San Antonio</t>
         </is>
       </c>
-      <c r="I58" t="inlineStr"/>
       <c r="J58" t="inlineStr">
         <is>
           <t>(210) 614-7993</t>
@@ -6115,10 +5932,11 @@
           <t>8257 Fredericksburg Rd, San Antonio, TX 78229, USA</t>
         </is>
       </c>
-      <c r="L58" t="inlineStr"/>
-      <c r="M58" t="inlineStr"/>
-      <c r="N58" t="inlineStr"/>
-      <c r="O58" t="inlineStr"/>
+      <c r="L58" s="1" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
       <c r="P58" t="n">
         <v>4.9</v>
       </c>
@@ -6131,7 +5949,6 @@
       <c r="S58" t="n">
         <v>1</v>
       </c>
-      <c r="T58" t="inlineStr"/>
       <c r="U58" t="n">
         <v>240000</v>
       </c>

</xml_diff>

<commit_message>
Split Exec Name into Exec First Name and Exec Last Name columns
https://claude.ai/code/session_01917JoB1LXoWCAoYuucjGiV
</commit_message>
<xml_diff>
--- a/Womens_HRT_Hormones_Only_New_cleaned_updated.xlsx
+++ b/Womens_HRT_Hormones_Only_New_cleaned_updated.xlsx
@@ -420,7 +420,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AA58"/>
+  <dimension ref="A1:AB58"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -481,80 +481,85 @@
       </c>
       <c r="L1" t="inlineStr">
         <is>
-          <t>Exec Name</t>
+          <t>Exec First Name</t>
         </is>
       </c>
       <c r="M1" t="inlineStr">
         <is>
+          <t>Exec Last Name</t>
+        </is>
+      </c>
+      <c r="N1" t="inlineStr">
+        <is>
           <t>Exec Title</t>
         </is>
       </c>
-      <c r="N1" t="inlineStr">
+      <c r="O1" t="inlineStr">
         <is>
           <t>Exec Email</t>
         </is>
       </c>
-      <c r="O1" t="inlineStr">
+      <c r="P1" t="inlineStr">
         <is>
           <t>Exec LinkedIn</t>
         </is>
       </c>
-      <c r="P1" t="inlineStr">
+      <c r="Q1" t="inlineStr">
         <is>
           <t>Google Rating</t>
         </is>
       </c>
-      <c r="Q1" t="inlineStr">
+      <c r="R1" t="inlineStr">
         <is>
           <t>Reviews</t>
         </is>
       </c>
-      <c r="R1" t="inlineStr">
+      <c r="S1" t="inlineStr">
         <is>
           <t># Physicians</t>
         </is>
       </c>
-      <c r="S1" t="inlineStr">
+      <c r="T1" t="inlineStr">
         <is>
           <t># Locations</t>
         </is>
       </c>
-      <c r="T1" t="inlineStr">
+      <c r="U1" t="inlineStr">
         <is>
           <t>Years Operating</t>
         </is>
       </c>
-      <c r="U1" t="inlineStr">
+      <c r="V1" t="inlineStr">
         <is>
           <t>Est Rev Low</t>
         </is>
       </c>
-      <c r="V1" t="inlineStr">
+      <c r="W1" t="inlineStr">
         <is>
           <t>Est Rev High</t>
         </is>
       </c>
-      <c r="W1" t="inlineStr">
+      <c r="X1" t="inlineStr">
         <is>
           <t>Est EBITDA Low</t>
         </is>
       </c>
-      <c r="X1" t="inlineStr">
+      <c r="Y1" t="inlineStr">
         <is>
           <t>Est EBITDA High</t>
         </is>
       </c>
-      <c r="Y1" t="inlineStr">
+      <c r="Z1" t="inlineStr">
         <is>
           <t>ClinicIQ Score</t>
         </is>
       </c>
-      <c r="Z1" t="inlineStr">
+      <c r="AA1" t="inlineStr">
         <is>
           <t>Original Focus Reason</t>
         </is>
       </c>
-      <c r="AA1" t="inlineStr">
+      <c r="AB1" t="inlineStr">
         <is>
           <t>Google Maps</t>
         </is>
@@ -611,45 +616,50 @@
       </c>
       <c r="L2" t="inlineStr">
         <is>
-          <t>Karie Mcmurray</t>
+          <t>Karie</t>
         </is>
       </c>
       <c r="M2" t="inlineStr">
         <is>
+          <t>Mcmurray</t>
+        </is>
+      </c>
+      <c r="N2" t="inlineStr">
+        <is>
           <t>President</t>
         </is>
       </c>
-      <c r="P2" t="n">
+      <c r="Q2" t="n">
         <v>5</v>
       </c>
-      <c r="Q2" t="n">
+      <c r="R2" t="n">
         <v>506</v>
-      </c>
-      <c r="R2" t="n">
-        <v>2</v>
       </c>
       <c r="S2" t="n">
         <v>2</v>
       </c>
       <c r="T2" t="n">
+        <v>2</v>
+      </c>
+      <c r="U2" t="n">
         <v>35</v>
       </c>
-      <c r="U2" t="n">
+      <c r="V2" t="n">
         <v>288000</v>
       </c>
-      <c r="V2" t="n">
+      <c r="W2" t="n">
         <v>1260000</v>
       </c>
-      <c r="W2" t="n">
+      <c r="X2" t="n">
         <v>43200</v>
       </c>
-      <c r="X2" t="n">
+      <c r="Y2" t="n">
         <v>252000</v>
       </c>
-      <c r="Y2" t="n">
+      <c r="Z2" t="n">
         <v>77.59999999999999</v>
       </c>
-      <c r="Z2" t="inlineStr">
+      <c r="AA2" t="inlineStr">
         <is>
           <t>Core hormone/longevity practice — 3 hormone service signals, prescriber-led</t>
         </is>
@@ -706,50 +716,55 @@
       </c>
       <c r="L3" t="inlineStr">
         <is>
-          <t>Francine Giardino</t>
+          <t>Francine</t>
         </is>
       </c>
       <c r="M3" t="inlineStr">
         <is>
+          <t>Giardino</t>
+        </is>
+      </c>
+      <c r="N3" t="inlineStr">
+        <is>
           <t>Owner</t>
         </is>
       </c>
-      <c r="O3" t="inlineStr">
+      <c r="P3" t="inlineStr">
         <is>
           <t>https://www.linkedin.com/company/ocsportsandwellnessca/</t>
         </is>
       </c>
-      <c r="P3" t="n">
+      <c r="Q3" t="n">
         <v>4.9</v>
       </c>
-      <c r="Q3" t="n">
+      <c r="R3" t="n">
         <v>110</v>
       </c>
-      <c r="R3" t="n">
+      <c r="S3" t="n">
         <v>4</v>
       </c>
-      <c r="S3" t="n">
+      <c r="T3" t="n">
         <v>1</v>
       </c>
-      <c r="T3" t="n">
+      <c r="U3" t="n">
         <v>27</v>
       </c>
-      <c r="U3" t="n">
+      <c r="V3" t="n">
         <v>792000</v>
       </c>
-      <c r="V3" t="n">
+      <c r="W3" t="n">
         <v>3240000</v>
       </c>
-      <c r="W3" t="n">
+      <c r="X3" t="n">
         <v>118800</v>
       </c>
-      <c r="X3" t="n">
+      <c r="Y3" t="n">
         <v>648000</v>
       </c>
-      <c r="Y3" t="n">
+      <c r="Z3" t="n">
         <v>53.2</v>
       </c>
-      <c r="Z3" t="inlineStr">
+      <c r="AA3" t="inlineStr">
         <is>
           <t>Core hormone/longevity practice — 3 hormone service signals, prescriber-led</t>
         </is>
@@ -806,42 +821,47 @@
       </c>
       <c r="L4" t="inlineStr">
         <is>
-          <t>Antoinette Jackson-Sekunda</t>
-        </is>
-      </c>
-      <c r="O4" t="inlineStr">
+          <t>Antoinette</t>
+        </is>
+      </c>
+      <c r="M4" t="inlineStr">
+        <is>
+          <t>Jackson-Sekunda</t>
+        </is>
+      </c>
+      <c r="P4" t="inlineStr">
         <is>
           <t>https://www.linkedin.com/company/bff-medical-wellness-clinic/</t>
         </is>
       </c>
-      <c r="P4" t="n">
+      <c r="Q4" t="n">
         <v>4.8</v>
       </c>
-      <c r="Q4" t="n">
+      <c r="R4" t="n">
         <v>196</v>
       </c>
-      <c r="R4" t="n">
+      <c r="S4" t="n">
         <v>0</v>
       </c>
-      <c r="S4" t="n">
+      <c r="T4" t="n">
         <v>3</v>
       </c>
-      <c r="U4" t="n">
+      <c r="V4" t="n">
         <v>240000</v>
       </c>
-      <c r="V4" t="n">
+      <c r="W4" t="n">
         <v>810000</v>
       </c>
-      <c r="W4" t="n">
+      <c r="X4" t="n">
         <v>36000</v>
       </c>
-      <c r="X4" t="n">
+      <c r="Y4" t="n">
         <v>162000</v>
       </c>
-      <c r="Y4" t="n">
+      <c r="Z4" t="n">
         <v>52.4</v>
       </c>
-      <c r="Z4" t="inlineStr">
+      <c r="AA4" t="inlineStr">
         <is>
           <t>Mixed practice — hormone services present alongside 0 aesthetic and 0 weight-loss signals</t>
         </is>
@@ -898,42 +918,47 @@
       </c>
       <c r="L5" t="inlineStr">
         <is>
-          <t>Lamia Gabal</t>
+          <t>Lamia</t>
         </is>
       </c>
       <c r="M5" t="inlineStr">
         <is>
+          <t>Gabal</t>
+        </is>
+      </c>
+      <c r="N5" t="inlineStr">
+        <is>
           <t>Founder,</t>
         </is>
       </c>
-      <c r="P5" t="n">
+      <c r="Q5" t="n">
         <v>4.6</v>
       </c>
-      <c r="Q5" t="n">
+      <c r="R5" t="n">
         <v>420</v>
       </c>
-      <c r="R5" t="n">
+      <c r="S5" t="n">
         <v>3</v>
       </c>
-      <c r="S5" t="n">
+      <c r="T5" t="n">
         <v>1</v>
       </c>
-      <c r="U5" t="n">
+      <c r="V5" t="n">
         <v>720000</v>
       </c>
-      <c r="V5" t="n">
+      <c r="W5" t="n">
         <v>2430000</v>
       </c>
-      <c r="W5" t="n">
+      <c r="X5" t="n">
         <v>108000</v>
       </c>
-      <c r="X5" t="n">
+      <c r="Y5" t="n">
         <v>486000</v>
       </c>
-      <c r="Y5" t="n">
+      <c r="Z5" t="n">
         <v>50.8</v>
       </c>
-      <c r="Z5" t="inlineStr">
+      <c r="AA5" t="inlineStr">
         <is>
           <t>Core hormone/longevity practice — 4 hormone service signals, prescriber-led</t>
         </is>
@@ -990,42 +1015,47 @@
       </c>
       <c r="L6" t="inlineStr">
         <is>
-          <t>Chris Potter</t>
-        </is>
-      </c>
-      <c r="P6" t="n">
+          <t>Chris</t>
+        </is>
+      </c>
+      <c r="M6" t="inlineStr">
+        <is>
+          <t>Potter</t>
+        </is>
+      </c>
+      <c r="Q6" t="n">
         <v>5</v>
       </c>
-      <c r="Q6" t="n">
+      <c r="R6" t="n">
         <v>22</v>
       </c>
-      <c r="R6" t="n">
+      <c r="S6" t="n">
         <v>0</v>
       </c>
-      <c r="S6" t="n">
+      <c r="T6" t="n">
         <v>5</v>
       </c>
-      <c r="U6" t="n">
+      <c r="V6" t="n">
         <v>144000</v>
       </c>
-      <c r="V6" t="n">
+      <c r="W6" t="n">
         <v>630000</v>
       </c>
-      <c r="W6" t="n">
+      <c r="X6" t="n">
         <v>21600</v>
       </c>
-      <c r="X6" t="n">
+      <c r="Y6" t="n">
         <v>126000</v>
       </c>
-      <c r="Y6" t="n">
+      <c r="Z6" t="n">
         <v>48.7</v>
       </c>
-      <c r="Z6" t="inlineStr">
+      <c r="AA6" t="inlineStr">
         <is>
           <t>Solid hormone line (TRT/HRT focus in name/type) but mixed with other services</t>
         </is>
       </c>
-      <c r="AA6" t="inlineStr">
+      <c r="AB6" t="inlineStr">
         <is>
           <t>https://maps.google.com/?cid=11054917828088815494</t>
         </is>
@@ -1082,42 +1112,47 @@
       </c>
       <c r="L7" t="inlineStr">
         <is>
-          <t>Kathryn Houston</t>
-        </is>
-      </c>
-      <c r="P7" t="n">
+          <t>Kathryn</t>
+        </is>
+      </c>
+      <c r="M7" t="inlineStr">
+        <is>
+          <t>Houston</t>
+        </is>
+      </c>
+      <c r="Q7" t="n">
         <v>4.9</v>
       </c>
-      <c r="Q7" t="n">
+      <c r="R7" t="n">
         <v>64</v>
       </c>
-      <c r="R7" t="n">
+      <c r="S7" t="n">
         <v>2</v>
       </c>
-      <c r="S7" t="n">
+      <c r="T7" t="n">
         <v>3</v>
       </c>
-      <c r="U7" t="n">
+      <c r="V7" t="n">
         <v>288000</v>
       </c>
-      <c r="V7" t="n">
+      <c r="W7" t="n">
         <v>1260000</v>
       </c>
-      <c r="W7" t="n">
+      <c r="X7" t="n">
         <v>43200</v>
       </c>
-      <c r="X7" t="n">
+      <c r="Y7" t="n">
         <v>252000</v>
       </c>
-      <c r="Y7" t="n">
+      <c r="Z7" t="n">
         <v>41.2</v>
       </c>
-      <c r="Z7" t="inlineStr">
+      <c r="AA7" t="inlineStr">
         <is>
           <t>Some hormone presence but not the clear focus</t>
         </is>
       </c>
-      <c r="AA7" t="inlineStr">
+      <c r="AB7" t="inlineStr">
         <is>
           <t>https://maps.google.com/?cid=12133140771630574727</t>
         </is>
@@ -1174,47 +1209,52 @@
       </c>
       <c r="L8" t="inlineStr">
         <is>
-          <t>Rosa Cataldo</t>
+          <t>Rosa</t>
         </is>
       </c>
       <c r="M8" t="inlineStr">
         <is>
+          <t>Cataldo</t>
+        </is>
+      </c>
+      <c r="N8" t="inlineStr">
+        <is>
           <t>Founder</t>
         </is>
       </c>
-      <c r="N8" t="inlineStr">
+      <c r="O8" t="inlineStr">
         <is>
           <t>beautymd.us@gmail.com</t>
         </is>
       </c>
-      <c r="P8" t="n">
+      <c r="Q8" t="n">
         <v>5</v>
       </c>
-      <c r="Q8" t="n">
+      <c r="R8" t="n">
         <v>188</v>
       </c>
-      <c r="R8" t="n">
+      <c r="S8" t="n">
         <v>0</v>
       </c>
-      <c r="S8" t="n">
+      <c r="T8" t="n">
         <v>1</v>
       </c>
-      <c r="U8" t="n">
+      <c r="V8" t="n">
         <v>144000</v>
       </c>
-      <c r="V8" t="n">
+      <c r="W8" t="n">
         <v>630000</v>
       </c>
-      <c r="W8" t="n">
+      <c r="X8" t="n">
         <v>21600</v>
       </c>
-      <c r="X8" t="n">
+      <c r="Y8" t="n">
         <v>126000</v>
       </c>
-      <c r="Y8" t="n">
+      <c r="Z8" t="n">
         <v>40.5</v>
       </c>
-      <c r="Z8" t="inlineStr">
+      <c r="AA8" t="inlineStr">
         <is>
           <t>Solid hormone line (TRT/HRT focus in name/type) but mixed with other services</t>
         </is>
@@ -1266,47 +1306,52 @@
       </c>
       <c r="L9" t="inlineStr">
         <is>
-          <t>Samantha Lau</t>
+          <t>Samantha</t>
         </is>
       </c>
       <c r="M9" t="inlineStr">
         <is>
+          <t>Lau</t>
+        </is>
+      </c>
+      <c r="N9" t="inlineStr">
+        <is>
           <t>CEO</t>
         </is>
       </c>
-      <c r="N9" t="inlineStr">
+      <c r="O9" t="inlineStr">
         <is>
           <t>sam@elevateherhealth.com</t>
         </is>
       </c>
-      <c r="P9" t="n">
+      <c r="Q9" t="n">
         <v>5</v>
       </c>
-      <c r="Q9" t="n">
+      <c r="R9" t="n">
         <v>33</v>
       </c>
-      <c r="R9" t="n">
+      <c r="S9" t="n">
         <v>1</v>
       </c>
-      <c r="S9" t="n">
+      <c r="T9" t="n">
         <v>15</v>
       </c>
-      <c r="U9" t="n">
+      <c r="V9" t="n">
         <v>144000</v>
       </c>
-      <c r="V9" t="n">
+      <c r="W9" t="n">
         <v>630000</v>
       </c>
-      <c r="W9" t="n">
+      <c r="X9" t="n">
         <v>21600</v>
       </c>
-      <c r="X9" t="n">
+      <c r="Y9" t="n">
         <v>126000</v>
       </c>
-      <c r="Y9" t="n">
+      <c r="Z9" t="n">
         <v>40.3</v>
       </c>
-      <c r="Z9" t="inlineStr">
+      <c r="AA9" t="inlineStr">
         <is>
           <t>Some hormone presence but not the clear focus</t>
         </is>
@@ -1363,55 +1408,60 @@
       </c>
       <c r="L10" t="inlineStr">
         <is>
-          <t>Raquel Lecesne</t>
+          <t>Raquel</t>
         </is>
       </c>
       <c r="M10" t="inlineStr">
         <is>
+          <t>Lecesne</t>
+        </is>
+      </c>
+      <c r="N10" t="inlineStr">
+        <is>
           <t>CEO</t>
         </is>
       </c>
-      <c r="N10" t="inlineStr">
+      <c r="O10" t="inlineStr">
         <is>
           <t>raquel@altheraclinic.com</t>
         </is>
       </c>
-      <c r="O10" t="inlineStr">
+      <c r="P10" t="inlineStr">
         <is>
           <t>https://www.linkedin.com/company/althera-alternative-care/</t>
         </is>
       </c>
-      <c r="P10" t="n">
+      <c r="Q10" t="n">
         <v>4.9</v>
       </c>
-      <c r="Q10" t="n">
+      <c r="R10" t="n">
         <v>164</v>
       </c>
-      <c r="R10" t="n">
+      <c r="S10" t="n">
         <v>0</v>
       </c>
-      <c r="S10" t="n">
+      <c r="T10" t="n">
         <v>1</v>
       </c>
-      <c r="T10" t="n">
+      <c r="U10" t="n">
         <v>6</v>
       </c>
-      <c r="U10" t="n">
+      <c r="V10" t="n">
         <v>144000</v>
       </c>
-      <c r="V10" t="n">
+      <c r="W10" t="n">
         <v>630000</v>
       </c>
-      <c r="W10" t="n">
+      <c r="X10" t="n">
         <v>21600</v>
       </c>
-      <c r="X10" t="n">
+      <c r="Y10" t="n">
         <v>126000</v>
       </c>
-      <c r="Y10" t="n">
+      <c r="Z10" t="n">
         <v>39.3</v>
       </c>
-      <c r="Z10" t="inlineStr">
+      <c r="AA10" t="inlineStr">
         <is>
           <t>Some hormone presence but not the clear focus</t>
         </is>
@@ -1468,50 +1518,55 @@
       </c>
       <c r="L11" t="inlineStr">
         <is>
-          <t>Edison Mello</t>
+          <t>Edison</t>
         </is>
       </c>
       <c r="M11" t="inlineStr">
         <is>
+          <t>Mello</t>
+        </is>
+      </c>
+      <c r="N11" t="inlineStr">
+        <is>
           <t>Owner</t>
         </is>
       </c>
-      <c r="O11" t="inlineStr">
+      <c r="P11" t="inlineStr">
         <is>
           <t>https://www.linkedin.com/company/akasha-center-for-integrative-medicine/</t>
         </is>
       </c>
-      <c r="P11" t="n">
+      <c r="Q11" t="n">
         <v>4.5</v>
       </c>
-      <c r="Q11" t="n">
+      <c r="R11" t="n">
         <v>32</v>
       </c>
-      <c r="R11" t="n">
+      <c r="S11" t="n">
         <v>7</v>
       </c>
-      <c r="S11" t="n">
+      <c r="T11" t="n">
         <v>1</v>
       </c>
-      <c r="T11" t="n">
+      <c r="U11" t="n">
         <v>24</v>
       </c>
-      <c r="U11" t="n">
+      <c r="V11" t="n">
         <v>231000</v>
       </c>
-      <c r="V11" t="n">
+      <c r="W11" t="n">
         <v>1036800</v>
       </c>
-      <c r="W11" t="n">
+      <c r="X11" t="n">
         <v>34650</v>
       </c>
-      <c r="X11" t="n">
+      <c r="Y11" t="n">
         <v>207360</v>
       </c>
-      <c r="Y11" t="n">
+      <c r="Z11" t="n">
         <v>38.2</v>
       </c>
-      <c r="Z11" t="inlineStr">
+      <c r="AA11" t="inlineStr">
         <is>
           <t>Some hormone presence but not the clear focus</t>
         </is>
@@ -1568,55 +1623,60 @@
       </c>
       <c r="L12" t="inlineStr">
         <is>
-          <t>Christine Balazs</t>
+          <t>Christine</t>
         </is>
       </c>
       <c r="M12" t="inlineStr">
         <is>
+          <t>Balazs</t>
+        </is>
+      </c>
+      <c r="N12" t="inlineStr">
+        <is>
           <t>CFO</t>
         </is>
       </c>
-      <c r="N12" t="inlineStr">
+      <c r="O12" t="inlineStr">
         <is>
           <t>christine@holtorfmed.com</t>
         </is>
       </c>
-      <c r="O12" t="inlineStr">
+      <c r="P12" t="inlineStr">
         <is>
           <t>https://www.linkedin.com/company/holtorf-medical-group/</t>
         </is>
       </c>
-      <c r="P12" t="n">
+      <c r="Q12" t="n">
         <v>4.6</v>
       </c>
-      <c r="Q12" t="n">
+      <c r="R12" t="n">
         <v>132</v>
       </c>
-      <c r="R12" t="n">
+      <c r="S12" t="n">
         <v>2</v>
       </c>
-      <c r="S12" t="n">
+      <c r="T12" t="n">
         <v>1</v>
       </c>
-      <c r="T12" t="n">
+      <c r="U12" t="n">
         <v>26</v>
       </c>
-      <c r="U12" t="n">
+      <c r="V12" t="n">
         <v>288000</v>
       </c>
-      <c r="V12" t="n">
+      <c r="W12" t="n">
         <v>1260000</v>
       </c>
-      <c r="W12" t="n">
+      <c r="X12" t="n">
         <v>43200</v>
       </c>
-      <c r="X12" t="n">
+      <c r="Y12" t="n">
         <v>252000</v>
       </c>
-      <c r="Y12" t="n">
+      <c r="Z12" t="n">
         <v>35.1</v>
       </c>
-      <c r="Z12" t="inlineStr">
+      <c r="AA12" t="inlineStr">
         <is>
           <t>Some hormone presence but not the clear focus</t>
         </is>
@@ -1673,55 +1733,60 @@
       </c>
       <c r="L13" t="inlineStr">
         <is>
-          <t>Judson Brandeis</t>
+          <t>Judson</t>
         </is>
       </c>
       <c r="M13" t="inlineStr">
         <is>
+          <t>Brandeis</t>
+        </is>
+      </c>
+      <c r="N13" t="inlineStr">
+        <is>
           <t>Owner (NPI Authorized Official)</t>
         </is>
       </c>
-      <c r="N13" t="inlineStr">
+      <c r="O13" t="inlineStr">
         <is>
           <t>judson@brandeismd.com</t>
         </is>
       </c>
-      <c r="O13" t="inlineStr">
+      <c r="P13" t="inlineStr">
         <is>
           <t>https://www.linkedin.com/company/brandeismd/</t>
         </is>
       </c>
-      <c r="P13" t="n">
+      <c r="Q13" t="n">
         <v>4.9</v>
       </c>
-      <c r="Q13" t="n">
+      <c r="R13" t="n">
         <v>54</v>
       </c>
-      <c r="R13" t="n">
+      <c r="S13" t="n">
         <v>0</v>
       </c>
-      <c r="S13" t="n">
+      <c r="T13" t="n">
         <v>1</v>
       </c>
-      <c r="T13" t="n">
+      <c r="U13" t="n">
         <v>7</v>
       </c>
-      <c r="U13" t="n">
+      <c r="V13" t="n">
         <v>144000</v>
       </c>
-      <c r="V13" t="n">
+      <c r="W13" t="n">
         <v>630000</v>
       </c>
-      <c r="W13" t="n">
+      <c r="X13" t="n">
         <v>21600</v>
       </c>
-      <c r="X13" t="n">
+      <c r="Y13" t="n">
         <v>126000</v>
       </c>
-      <c r="Y13" t="n">
+      <c r="Z13" t="n">
         <v>34.9</v>
       </c>
-      <c r="Z13" t="inlineStr">
+      <c r="AA13" t="inlineStr">
         <is>
           <t>Some hormone presence but not the clear focus</t>
         </is>
@@ -1778,37 +1843,42 @@
       </c>
       <c r="L14" t="inlineStr">
         <is>
-          <t>Yasmine Perdue</t>
-        </is>
-      </c>
-      <c r="P14" t="n">
+          <t>Yasmine</t>
+        </is>
+      </c>
+      <c r="M14" t="inlineStr">
+        <is>
+          <t>Perdue</t>
+        </is>
+      </c>
+      <c r="Q14" t="n">
         <v>5</v>
       </c>
-      <c r="Q14" t="n">
+      <c r="R14" t="n">
         <v>62</v>
-      </c>
-      <c r="R14" t="n">
-        <v>1</v>
       </c>
       <c r="S14" t="n">
         <v>1</v>
       </c>
-      <c r="U14" t="n">
+      <c r="T14" t="n">
+        <v>1</v>
+      </c>
+      <c r="V14" t="n">
         <v>144000</v>
       </c>
-      <c r="V14" t="n">
+      <c r="W14" t="n">
         <v>630000</v>
       </c>
-      <c r="W14" t="n">
+      <c r="X14" t="n">
         <v>21600</v>
       </c>
-      <c r="X14" t="n">
+      <c r="Y14" t="n">
         <v>126000</v>
       </c>
-      <c r="Y14" t="n">
+      <c r="Z14" t="n">
         <v>33.7</v>
       </c>
-      <c r="Z14" t="inlineStr">
+      <c r="AA14" t="inlineStr">
         <is>
           <t>Core hormone/longevity practice — 3 hormone service signals, prescriber-led</t>
         </is>
@@ -1868,34 +1938,39 @@
           <t>N/A</t>
         </is>
       </c>
-      <c r="P15" t="n">
+      <c r="M15" s="1" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="Q15" t="n">
         <v>4.9</v>
       </c>
-      <c r="Q15" t="n">
+      <c r="R15" t="n">
         <v>64</v>
       </c>
-      <c r="R15" t="n">
+      <c r="S15" t="n">
         <v>0</v>
       </c>
-      <c r="S15" t="n">
+      <c r="T15" t="n">
         <v>1</v>
       </c>
-      <c r="U15" t="n">
+      <c r="V15" t="n">
         <v>144000</v>
       </c>
-      <c r="V15" t="n">
+      <c r="W15" t="n">
         <v>630000</v>
       </c>
-      <c r="W15" t="n">
+      <c r="X15" t="n">
         <v>21600</v>
       </c>
-      <c r="X15" t="n">
+      <c r="Y15" t="n">
         <v>126000</v>
       </c>
-      <c r="Y15" t="n">
+      <c r="Z15" t="n">
         <v>30.4</v>
       </c>
-      <c r="Z15" t="inlineStr">
+      <c r="AA15" t="inlineStr">
         <is>
           <t>Some hormone presence but not the clear focus</t>
         </is>
@@ -1952,52 +2027,57 @@
       </c>
       <c r="L16" t="inlineStr">
         <is>
-          <t>Jeffrey Sternberg</t>
+          <t>Jeffrey</t>
         </is>
       </c>
       <c r="M16" t="inlineStr">
         <is>
+          <t>Sternberg</t>
+        </is>
+      </c>
+      <c r="N16" t="inlineStr">
+        <is>
           <t>CEO</t>
         </is>
       </c>
-      <c r="N16" t="inlineStr">
+      <c r="O16" t="inlineStr">
         <is>
           <t>jsternberg@koiwellbeing.com</t>
         </is>
       </c>
-      <c r="O16" t="inlineStr">
+      <c r="P16" t="inlineStr">
         <is>
           <t>https://www.linkedin.com/company/koiwellbeing/</t>
         </is>
       </c>
-      <c r="P16" t="n">
+      <c r="Q16" t="n">
         <v>4.9</v>
       </c>
-      <c r="Q16" t="n">
+      <c r="R16" t="n">
         <v>60</v>
       </c>
-      <c r="R16" t="n">
+      <c r="S16" t="n">
         <v>0</v>
       </c>
-      <c r="S16" t="n">
+      <c r="T16" t="n">
         <v>1</v>
       </c>
-      <c r="U16" t="n">
+      <c r="V16" t="n">
         <v>144000</v>
       </c>
-      <c r="V16" t="n">
+      <c r="W16" t="n">
         <v>630000</v>
       </c>
-      <c r="W16" t="n">
+      <c r="X16" t="n">
         <v>21600</v>
       </c>
-      <c r="X16" t="n">
+      <c r="Y16" t="n">
         <v>126000</v>
       </c>
-      <c r="Y16" t="n">
+      <c r="Z16" t="n">
         <v>30.2</v>
       </c>
-      <c r="Z16" t="inlineStr">
+      <c r="AA16" t="inlineStr">
         <is>
           <t>Some hormone presence but not the clear focus</t>
         </is>
@@ -2054,37 +2134,42 @@
       </c>
       <c r="L17" t="inlineStr">
         <is>
-          <t>Sharone Utter</t>
-        </is>
-      </c>
-      <c r="P17" t="n">
+          <t>Sharone</t>
+        </is>
+      </c>
+      <c r="M17" t="inlineStr">
+        <is>
+          <t>Utter</t>
+        </is>
+      </c>
+      <c r="Q17" t="n">
         <v>4.8</v>
       </c>
-      <c r="Q17" t="n">
+      <c r="R17" t="n">
         <v>52</v>
       </c>
-      <c r="R17" t="n">
+      <c r="S17" t="n">
         <v>0</v>
       </c>
-      <c r="S17" t="n">
+      <c r="T17" t="n">
         <v>1</v>
       </c>
-      <c r="U17" t="n">
+      <c r="V17" t="n">
         <v>144000</v>
       </c>
-      <c r="V17" t="n">
+      <c r="W17" t="n">
         <v>630000</v>
       </c>
-      <c r="W17" t="n">
+      <c r="X17" t="n">
         <v>21600</v>
       </c>
-      <c r="X17" t="n">
+      <c r="Y17" t="n">
         <v>126000</v>
       </c>
-      <c r="Y17" t="n">
+      <c r="Z17" t="n">
         <v>29.7</v>
       </c>
-      <c r="Z17" t="inlineStr">
+      <c r="AA17" t="inlineStr">
         <is>
           <t>Some hormone presence but not the clear focus</t>
         </is>
@@ -2141,42 +2226,47 @@
       </c>
       <c r="L18" t="inlineStr">
         <is>
-          <t>Marc Kaufman</t>
-        </is>
-      </c>
-      <c r="P18" t="n">
+          <t>Marc</t>
+        </is>
+      </c>
+      <c r="M18" t="inlineStr">
+        <is>
+          <t>Kaufman</t>
+        </is>
+      </c>
+      <c r="Q18" t="n">
         <v>5</v>
       </c>
-      <c r="Q18" t="n">
+      <c r="R18" t="n">
         <v>27</v>
       </c>
-      <c r="R18" t="n">
+      <c r="S18" t="n">
         <v>0</v>
       </c>
-      <c r="S18" t="n">
+      <c r="T18" t="n">
         <v>1</v>
       </c>
-      <c r="U18" t="n">
+      <c r="V18" t="n">
         <v>195000</v>
       </c>
-      <c r="V18" t="n">
+      <c r="W18" t="n">
         <v>810000</v>
       </c>
-      <c r="W18" t="n">
+      <c r="X18" t="n">
         <v>29250</v>
       </c>
-      <c r="X18" t="n">
+      <c r="Y18" t="n">
         <v>162000</v>
       </c>
-      <c r="Y18" t="n">
+      <c r="Z18" t="n">
         <v>29.6</v>
       </c>
-      <c r="Z18" t="inlineStr">
+      <c r="AA18" t="inlineStr">
         <is>
           <t>Solid hormone line (TRT/HRT focus in name/type) but mixed with other services</t>
         </is>
       </c>
-      <c r="AA18" t="inlineStr">
+      <c r="AB18" t="inlineStr">
         <is>
           <t>https://maps.google.com/?cid=3716565926912822396</t>
         </is>
@@ -2233,42 +2323,47 @@
       </c>
       <c r="L19" t="inlineStr">
         <is>
-          <t>Van Nguyen</t>
-        </is>
-      </c>
-      <c r="P19" t="n">
+          <t>Van</t>
+        </is>
+      </c>
+      <c r="M19" t="inlineStr">
+        <is>
+          <t>Nguyen</t>
+        </is>
+      </c>
+      <c r="Q19" t="n">
         <v>4.8</v>
       </c>
-      <c r="Q19" t="n">
+      <c r="R19" t="n">
         <v>20</v>
       </c>
-      <c r="R19" t="n">
+      <c r="S19" t="n">
         <v>0</v>
       </c>
-      <c r="S19" t="n">
+      <c r="T19" t="n">
         <v>1</v>
       </c>
-      <c r="U19" t="n">
+      <c r="V19" t="n">
         <v>86400</v>
       </c>
-      <c r="V19" t="n">
+      <c r="W19" t="n">
         <v>504000</v>
       </c>
-      <c r="W19" t="n">
+      <c r="X19" t="n">
         <v>12960</v>
       </c>
-      <c r="X19" t="n">
+      <c r="Y19" t="n">
         <v>100800</v>
       </c>
-      <c r="Y19" t="n">
+      <c r="Z19" t="n">
         <v>29.4</v>
       </c>
-      <c r="Z19" t="inlineStr">
+      <c r="AA19" t="inlineStr">
         <is>
           <t>Solid hormone line (TRT/HRT focus in name/type) but mixed with other services</t>
         </is>
       </c>
-      <c r="AA19" t="inlineStr">
+      <c r="AB19" t="inlineStr">
         <is>
           <t>https://maps.google.com/?cid=15446542013092659828</t>
         </is>
@@ -2328,39 +2423,44 @@
           <t>N/A</t>
         </is>
       </c>
-      <c r="P20" t="n">
+      <c r="M20" s="1" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="Q20" t="n">
         <v>5</v>
       </c>
-      <c r="Q20" t="n">
+      <c r="R20" t="n">
         <v>22</v>
       </c>
-      <c r="R20" t="n">
+      <c r="S20" t="n">
         <v>0</v>
       </c>
-      <c r="S20" t="n">
+      <c r="T20" t="n">
         <v>1</v>
       </c>
-      <c r="U20" t="n">
+      <c r="V20" t="n">
         <v>95400</v>
       </c>
-      <c r="V20" t="n">
+      <c r="W20" t="n">
         <v>554400</v>
       </c>
-      <c r="W20" t="n">
+      <c r="X20" t="n">
         <v>14310</v>
       </c>
-      <c r="X20" t="n">
+      <c r="Y20" t="n">
         <v>110880</v>
       </c>
-      <c r="Y20" t="n">
+      <c r="Z20" t="n">
         <v>29</v>
       </c>
-      <c r="Z20" t="inlineStr">
+      <c r="AA20" t="inlineStr">
         <is>
           <t>Solid hormone line (TRT/HRT focus in name/type) but mixed with other services</t>
         </is>
       </c>
-      <c r="AA20" t="inlineStr">
+      <c r="AB20" t="inlineStr">
         <is>
           <t>https://maps.google.com/?cid=7354279795671113525</t>
         </is>
@@ -2417,37 +2517,42 @@
       </c>
       <c r="L21" t="inlineStr">
         <is>
-          <t>Yazan Abdullah</t>
-        </is>
-      </c>
-      <c r="P21" t="n">
+          <t>Yazan</t>
+        </is>
+      </c>
+      <c r="M21" t="inlineStr">
+        <is>
+          <t>Abdullah</t>
+        </is>
+      </c>
+      <c r="Q21" t="n">
         <v>4.8</v>
       </c>
-      <c r="Q21" t="n">
+      <c r="R21" t="n">
         <v>42</v>
       </c>
-      <c r="R21" t="n">
+      <c r="S21" t="n">
         <v>0</v>
       </c>
-      <c r="S21" t="n">
+      <c r="T21" t="n">
         <v>1</v>
       </c>
-      <c r="U21" t="n">
+      <c r="V21" t="n">
         <v>144000</v>
       </c>
-      <c r="V21" t="n">
+      <c r="W21" t="n">
         <v>630000</v>
       </c>
-      <c r="W21" t="n">
+      <c r="X21" t="n">
         <v>21600</v>
       </c>
-      <c r="X21" t="n">
+      <c r="Y21" t="n">
         <v>126000</v>
       </c>
-      <c r="Y21" t="n">
+      <c r="Z21" t="n">
         <v>28.9</v>
       </c>
-      <c r="Z21" t="inlineStr">
+      <c r="AA21" t="inlineStr">
         <is>
           <t>Some hormone presence but not the clear focus</t>
         </is>
@@ -2504,37 +2609,42 @@
       </c>
       <c r="L22" t="inlineStr">
         <is>
-          <t>Ojen Masrour</t>
-        </is>
-      </c>
-      <c r="P22" t="n">
+          <t>Ojen</t>
+        </is>
+      </c>
+      <c r="M22" t="inlineStr">
+        <is>
+          <t>Masrour</t>
+        </is>
+      </c>
+      <c r="Q22" t="n">
         <v>4.2</v>
       </c>
-      <c r="Q22" t="n">
+      <c r="R22" t="n">
         <v>26</v>
       </c>
-      <c r="R22" t="n">
+      <c r="S22" t="n">
         <v>0</v>
       </c>
-      <c r="S22" t="n">
+      <c r="T22" t="n">
         <v>1</v>
       </c>
-      <c r="U22" t="n">
+      <c r="V22" t="n">
         <v>111600</v>
       </c>
-      <c r="V22" t="n">
+      <c r="W22" t="n">
         <v>630000</v>
       </c>
-      <c r="W22" t="n">
+      <c r="X22" t="n">
         <v>16740</v>
       </c>
-      <c r="X22" t="n">
+      <c r="Y22" t="n">
         <v>126000</v>
       </c>
-      <c r="Y22" t="n">
+      <c r="Z22" t="n">
         <v>27</v>
       </c>
-      <c r="Z22" t="inlineStr">
+      <c r="AA22" t="inlineStr">
         <is>
           <t>Some hormone presence but not the clear focus</t>
         </is>
@@ -2591,42 +2701,47 @@
       </c>
       <c r="L23" t="inlineStr">
         <is>
-          <t>Melissa Kemp</t>
-        </is>
-      </c>
-      <c r="P23" t="n">
+          <t>Melissa</t>
+        </is>
+      </c>
+      <c r="M23" t="inlineStr">
+        <is>
+          <t>Kemp</t>
+        </is>
+      </c>
+      <c r="Q23" t="n">
         <v>5</v>
       </c>
-      <c r="Q23" t="n">
+      <c r="R23" t="n">
         <v>261</v>
-      </c>
-      <c r="R23" t="n">
-        <v>1</v>
       </c>
       <c r="S23" t="n">
         <v>1</v>
       </c>
-      <c r="U23" t="n">
+      <c r="T23" t="n">
+        <v>1</v>
+      </c>
+      <c r="V23" t="n">
         <v>144000</v>
       </c>
-      <c r="V23" t="n">
+      <c r="W23" t="n">
         <v>630000</v>
       </c>
-      <c r="W23" t="n">
+      <c r="X23" t="n">
         <v>21600</v>
       </c>
-      <c r="X23" t="n">
+      <c r="Y23" t="n">
         <v>126000</v>
       </c>
-      <c r="Y23" t="n">
+      <c r="Z23" t="n">
         <v>26.9</v>
       </c>
-      <c r="Z23" t="inlineStr">
+      <c r="AA23" t="inlineStr">
         <is>
           <t>Some hormone presence but not the clear focus</t>
         </is>
       </c>
-      <c r="AA23" t="inlineStr">
+      <c r="AB23" t="inlineStr">
         <is>
           <t>https://maps.google.com/?cid=12751487800332667397</t>
         </is>
@@ -2683,37 +2798,42 @@
       </c>
       <c r="L24" t="inlineStr">
         <is>
-          <t>Thom Lobe</t>
-        </is>
-      </c>
-      <c r="P24" t="n">
+          <t>Thom</t>
+        </is>
+      </c>
+      <c r="M24" t="inlineStr">
+        <is>
+          <t>Lobe</t>
+        </is>
+      </c>
+      <c r="Q24" t="n">
         <v>4.5</v>
       </c>
-      <c r="Q24" t="n">
+      <c r="R24" t="n">
         <v>25</v>
       </c>
-      <c r="R24" t="n">
+      <c r="S24" t="n">
         <v>0</v>
       </c>
-      <c r="S24" t="n">
+      <c r="T24" t="n">
         <v>1</v>
       </c>
-      <c r="U24" t="n">
+      <c r="V24" t="n">
         <v>108000</v>
       </c>
-      <c r="V24" t="n">
+      <c r="W24" t="n">
         <v>630000</v>
       </c>
-      <c r="W24" t="n">
+      <c r="X24" t="n">
         <v>16200</v>
       </c>
-      <c r="X24" t="n">
+      <c r="Y24" t="n">
         <v>126000</v>
       </c>
-      <c r="Y24" t="n">
+      <c r="Z24" t="n">
         <v>26.7</v>
       </c>
-      <c r="Z24" t="inlineStr">
+      <c r="AA24" t="inlineStr">
         <is>
           <t>Some hormone presence but not the clear focus</t>
         </is>
@@ -2770,42 +2890,47 @@
       </c>
       <c r="L25" t="inlineStr">
         <is>
-          <t>Devon Casida</t>
-        </is>
-      </c>
-      <c r="P25" t="n">
+          <t>Devon</t>
+        </is>
+      </c>
+      <c r="M25" t="inlineStr">
+        <is>
+          <t>Casida</t>
+        </is>
+      </c>
+      <c r="Q25" t="n">
         <v>5</v>
       </c>
-      <c r="Q25" t="n">
+      <c r="R25" t="n">
         <v>30</v>
       </c>
-      <c r="R25" t="n">
+      <c r="S25" t="n">
         <v>0</v>
       </c>
-      <c r="S25" t="n">
+      <c r="T25" t="n">
         <v>1</v>
       </c>
-      <c r="U25" t="n">
+      <c r="V25" t="n">
         <v>216000</v>
       </c>
-      <c r="V25" t="n">
+      <c r="W25" t="n">
         <v>810000</v>
       </c>
-      <c r="W25" t="n">
+      <c r="X25" t="n">
         <v>32400</v>
       </c>
-      <c r="X25" t="n">
+      <c r="Y25" t="n">
         <v>162000</v>
       </c>
-      <c r="Y25" t="n">
+      <c r="Z25" t="n">
         <v>24</v>
       </c>
-      <c r="Z25" t="inlineStr">
+      <c r="AA25" t="inlineStr">
         <is>
           <t>Mixed practice — hormone services present alongside 0 aesthetic and 0 weight-loss signals</t>
         </is>
       </c>
-      <c r="AA25" t="inlineStr">
+      <c r="AB25" t="inlineStr">
         <is>
           <t>https://maps.google.com/?cid=1318658128756553271</t>
         </is>
@@ -2862,42 +2987,47 @@
       </c>
       <c r="L26" t="inlineStr">
         <is>
-          <t>Jennifer Davis</t>
-        </is>
-      </c>
-      <c r="P26" t="n">
+          <t>Jennifer</t>
+        </is>
+      </c>
+      <c r="M26" t="inlineStr">
+        <is>
+          <t>Davis</t>
+        </is>
+      </c>
+      <c r="Q26" t="n">
         <v>4.9</v>
       </c>
-      <c r="Q26" t="n">
+      <c r="R26" t="n">
         <v>94</v>
-      </c>
-      <c r="R26" t="n">
-        <v>1</v>
       </c>
       <c r="S26" t="n">
         <v>1</v>
       </c>
-      <c r="U26" t="n">
+      <c r="T26" t="n">
+        <v>1</v>
+      </c>
+      <c r="V26" t="n">
         <v>240000</v>
       </c>
-      <c r="V26" t="n">
+      <c r="W26" t="n">
         <v>810000</v>
       </c>
-      <c r="W26" t="n">
+      <c r="X26" t="n">
         <v>36000</v>
       </c>
-      <c r="X26" t="n">
+      <c r="Y26" t="n">
         <v>162000</v>
       </c>
-      <c r="Y26" t="n">
+      <c r="Z26" t="n">
         <v>23.2</v>
       </c>
-      <c r="Z26" t="inlineStr">
+      <c r="AA26" t="inlineStr">
         <is>
           <t>Some hormone presence but not the clear focus</t>
         </is>
       </c>
-      <c r="AA26" t="inlineStr">
+      <c r="AB26" t="inlineStr">
         <is>
           <t>https://maps.google.com/?cid=17274611547814637695</t>
         </is>
@@ -2954,42 +3084,47 @@
       </c>
       <c r="L27" t="inlineStr">
         <is>
-          <t>Matthew Risner</t>
-        </is>
-      </c>
-      <c r="P27" t="n">
+          <t>Matthew</t>
+        </is>
+      </c>
+      <c r="M27" t="inlineStr">
+        <is>
+          <t>Risner</t>
+        </is>
+      </c>
+      <c r="Q27" t="n">
         <v>5</v>
       </c>
-      <c r="Q27" t="n">
+      <c r="R27" t="n">
         <v>92</v>
       </c>
-      <c r="R27" t="n">
+      <c r="S27" t="n">
         <v>0</v>
       </c>
-      <c r="S27" t="n">
+      <c r="T27" t="n">
         <v>1</v>
       </c>
-      <c r="U27" t="n">
+      <c r="V27" t="n">
         <v>240000</v>
       </c>
-      <c r="V27" t="n">
+      <c r="W27" t="n">
         <v>810000</v>
       </c>
-      <c r="W27" t="n">
+      <c r="X27" t="n">
         <v>36000</v>
       </c>
-      <c r="X27" t="n">
+      <c r="Y27" t="n">
         <v>162000</v>
       </c>
-      <c r="Y27" t="n">
+      <c r="Z27" t="n">
         <v>22.8</v>
       </c>
-      <c r="Z27" t="inlineStr">
+      <c r="AA27" t="inlineStr">
         <is>
           <t>Mixed practice — hormone services present alongside 0 aesthetic and 0 weight-loss signals</t>
         </is>
       </c>
-      <c r="AA27" t="inlineStr">
+      <c r="AB27" t="inlineStr">
         <is>
           <t>https://maps.google.com/?cid=9469390767176375705</t>
         </is>
@@ -3046,40 +3181,45 @@
       </c>
       <c r="L28" t="inlineStr">
         <is>
-          <t>Joseph Aiello</t>
-        </is>
-      </c>
-      <c r="P28" t="n">
+          <t>Joseph</t>
+        </is>
+      </c>
+      <c r="M28" t="inlineStr">
+        <is>
+          <t>Aiello</t>
+        </is>
+      </c>
+      <c r="Q28" t="n">
         <v>4.9</v>
       </c>
-      <c r="Q28" t="n">
+      <c r="R28" t="n">
         <v>32</v>
       </c>
-      <c r="R28" t="n">
+      <c r="S28" t="n">
         <v>0</v>
-      </c>
-      <c r="S28" t="n">
-        <v>1</v>
       </c>
       <c r="T28" t="n">
         <v>1</v>
       </c>
       <c r="U28" t="n">
+        <v>1</v>
+      </c>
+      <c r="V28" t="n">
         <v>138600</v>
       </c>
-      <c r="V28" t="n">
+      <c r="W28" t="n">
         <v>630000</v>
       </c>
-      <c r="W28" t="n">
+      <c r="X28" t="n">
         <v>20790</v>
       </c>
-      <c r="X28" t="n">
+      <c r="Y28" t="n">
         <v>126000</v>
       </c>
-      <c r="Y28" t="n">
+      <c r="Z28" t="n">
         <v>22.5</v>
       </c>
-      <c r="Z28" t="inlineStr">
+      <c r="AA28" t="inlineStr">
         <is>
           <t>Some hormone presence but not the clear focus</t>
         </is>
@@ -3141,42 +3281,47 @@
       </c>
       <c r="L29" t="inlineStr">
         <is>
-          <t>Pamela Gaudry</t>
-        </is>
-      </c>
-      <c r="P29" t="n">
+          <t>Pamela</t>
+        </is>
+      </c>
+      <c r="M29" t="inlineStr">
+        <is>
+          <t>Gaudry</t>
+        </is>
+      </c>
+      <c r="Q29" t="n">
         <v>4.7</v>
       </c>
-      <c r="Q29" t="n">
+      <c r="R29" t="n">
         <v>40</v>
       </c>
-      <c r="R29" t="n">
+      <c r="S29" t="n">
         <v>3</v>
       </c>
-      <c r="S29" t="n">
+      <c r="T29" t="n">
         <v>2</v>
       </c>
-      <c r="U29" t="n">
+      <c r="V29" t="n">
         <v>489000</v>
       </c>
-      <c r="V29" t="n">
+      <c r="W29" t="n">
         <v>2203200</v>
       </c>
-      <c r="W29" t="n">
+      <c r="X29" t="n">
         <v>73350</v>
       </c>
-      <c r="X29" t="n">
+      <c r="Y29" t="n">
         <v>440640</v>
       </c>
-      <c r="Y29" t="n">
+      <c r="Z29" t="n">
         <v>22.2</v>
       </c>
-      <c r="Z29" t="inlineStr">
+      <c r="AA29" t="inlineStr">
         <is>
           <t>No hormone, aesthetic, or weight-loss signals detected — may need manual review</t>
         </is>
       </c>
-      <c r="AA29" t="inlineStr">
+      <c r="AB29" t="inlineStr">
         <is>
           <t>https://maps.google.com/?cid=5711891707944874425</t>
         </is>
@@ -3233,42 +3378,47 @@
       </c>
       <c r="L30" t="inlineStr">
         <is>
-          <t>Cally Smith</t>
-        </is>
-      </c>
-      <c r="P30" t="n">
+          <t>Cally</t>
+        </is>
+      </c>
+      <c r="M30" t="inlineStr">
+        <is>
+          <t>Smith</t>
+        </is>
+      </c>
+      <c r="Q30" t="n">
         <v>5</v>
       </c>
-      <c r="Q30" t="n">
+      <c r="R30" t="n">
         <v>53</v>
       </c>
-      <c r="R30" t="n">
+      <c r="S30" t="n">
         <v>0</v>
       </c>
-      <c r="S30" t="n">
+      <c r="T30" t="n">
         <v>1</v>
       </c>
-      <c r="U30" t="n">
+      <c r="V30" t="n">
         <v>240000</v>
       </c>
-      <c r="V30" t="n">
+      <c r="W30" t="n">
         <v>810000</v>
       </c>
-      <c r="W30" t="n">
+      <c r="X30" t="n">
         <v>36000</v>
       </c>
-      <c r="X30" t="n">
+      <c r="Y30" t="n">
         <v>162000</v>
       </c>
-      <c r="Y30" t="n">
+      <c r="Z30" t="n">
         <v>21.8</v>
       </c>
-      <c r="Z30" t="inlineStr">
+      <c r="AA30" t="inlineStr">
         <is>
           <t>Mixed practice — hormone services present alongside 0 aesthetic and 0 weight-loss signals</t>
         </is>
       </c>
-      <c r="AA30" t="inlineStr">
+      <c r="AB30" t="inlineStr">
         <is>
           <t>https://maps.google.com/?cid=935434273207101717</t>
         </is>
@@ -3333,42 +3483,47 @@
           <t>N/A</t>
         </is>
       </c>
-      <c r="P31" t="n">
+      <c r="M31" s="1" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="Q31" t="n">
         <v>4.8</v>
       </c>
-      <c r="Q31" t="n">
+      <c r="R31" t="n">
         <v>218</v>
       </c>
-      <c r="R31" t="n">
+      <c r="S31" t="n">
         <v>5</v>
       </c>
-      <c r="S31" t="n">
+      <c r="T31" t="n">
         <v>1</v>
       </c>
-      <c r="T31" t="n">
+      <c r="U31" t="n">
         <v>15</v>
       </c>
-      <c r="U31" t="n">
+      <c r="V31" t="n">
         <v>1200000</v>
       </c>
-      <c r="V31" t="n">
+      <c r="W31" t="n">
         <v>4050000</v>
       </c>
-      <c r="W31" t="n">
+      <c r="X31" t="n">
         <v>180000</v>
       </c>
-      <c r="X31" t="n">
+      <c r="Y31" t="n">
         <v>810000</v>
       </c>
-      <c r="Y31" t="n">
+      <c r="Z31" t="n">
         <v>21.4</v>
       </c>
-      <c r="Z31" t="inlineStr">
+      <c r="AA31" t="inlineStr">
         <is>
           <t>No hormone, aesthetic, or weight-loss signals detected — may need manual review</t>
         </is>
       </c>
-      <c r="AA31" t="inlineStr">
+      <c r="AB31" t="inlineStr">
         <is>
           <t>https://maps.google.com/?cid=9814576466280014998</t>
         </is>
@@ -3425,45 +3580,50 @@
       </c>
       <c r="L32" t="inlineStr">
         <is>
-          <t>Vahe Melikyan</t>
-        </is>
-      </c>
-      <c r="P32" t="n">
+          <t>Vahe</t>
+        </is>
+      </c>
+      <c r="M32" t="inlineStr">
+        <is>
+          <t>Melikyan</t>
+        </is>
+      </c>
+      <c r="Q32" t="n">
         <v>5</v>
       </c>
-      <c r="Q32" t="n">
+      <c r="R32" t="n">
         <v>21</v>
       </c>
-      <c r="R32" t="n">
+      <c r="S32" t="n">
         <v>0</v>
       </c>
-      <c r="S32" t="n">
+      <c r="T32" t="n">
         <v>1</v>
       </c>
-      <c r="T32" t="n">
+      <c r="U32" t="n">
         <v>2</v>
       </c>
-      <c r="U32" t="n">
+      <c r="V32" t="n">
         <v>150000</v>
       </c>
-      <c r="V32" t="n">
+      <c r="W32" t="n">
         <v>680400</v>
       </c>
-      <c r="W32" t="n">
+      <c r="X32" t="n">
         <v>22500</v>
       </c>
-      <c r="X32" t="n">
+      <c r="Y32" t="n">
         <v>136080</v>
       </c>
-      <c r="Y32" t="n">
+      <c r="Z32" t="n">
         <v>18.3</v>
       </c>
-      <c r="Z32" t="inlineStr">
+      <c r="AA32" t="inlineStr">
         <is>
           <t>Mixed practice — hormone services present alongside 0 aesthetic and 0 weight-loss signals</t>
         </is>
       </c>
-      <c r="AA32" t="inlineStr">
+      <c r="AB32" t="inlineStr">
         <is>
           <t>https://maps.google.com/?cid=8656087916047026939</t>
         </is>
@@ -3520,42 +3680,47 @@
       </c>
       <c r="L33" t="inlineStr">
         <is>
-          <t>Reem Sharhan</t>
-        </is>
-      </c>
-      <c r="P33" t="n">
+          <t>Reem</t>
+        </is>
+      </c>
+      <c r="M33" t="inlineStr">
+        <is>
+          <t>Sharhan</t>
+        </is>
+      </c>
+      <c r="Q33" t="n">
         <v>5</v>
       </c>
-      <c r="Q33" t="n">
+      <c r="R33" t="n">
         <v>21</v>
-      </c>
-      <c r="R33" t="n">
-        <v>1</v>
       </c>
       <c r="S33" t="n">
         <v>1</v>
       </c>
-      <c r="U33" t="n">
+      <c r="T33" t="n">
+        <v>1</v>
+      </c>
+      <c r="V33" t="n">
         <v>150000</v>
       </c>
-      <c r="V33" t="n">
+      <c r="W33" t="n">
         <v>680400</v>
       </c>
-      <c r="W33" t="n">
+      <c r="X33" t="n">
         <v>22500</v>
       </c>
-      <c r="X33" t="n">
+      <c r="Y33" t="n">
         <v>136080</v>
       </c>
-      <c r="Y33" t="n">
+      <c r="Z33" t="n">
         <v>18.3</v>
       </c>
-      <c r="Z33" t="inlineStr">
+      <c r="AA33" t="inlineStr">
         <is>
           <t>Some hormone presence but not the clear focus</t>
         </is>
       </c>
-      <c r="AA33" t="inlineStr">
+      <c r="AB33" t="inlineStr">
         <is>
           <t>https://maps.google.com/?cid=9180695523542794910</t>
         </is>
@@ -3615,39 +3780,44 @@
           <t>N/A</t>
         </is>
       </c>
-      <c r="P34" t="n">
+      <c r="M34" s="1" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="Q34" t="n">
         <v>5</v>
       </c>
-      <c r="Q34" t="n">
+      <c r="R34" t="n">
         <v>28</v>
-      </c>
-      <c r="R34" t="n">
-        <v>1</v>
       </c>
       <c r="S34" t="n">
         <v>1</v>
       </c>
-      <c r="U34" t="n">
+      <c r="T34" t="n">
+        <v>1</v>
+      </c>
+      <c r="V34" t="n">
         <v>120600</v>
       </c>
-      <c r="V34" t="n">
+      <c r="W34" t="n">
         <v>630000</v>
       </c>
-      <c r="W34" t="n">
+      <c r="X34" t="n">
         <v>18090</v>
       </c>
-      <c r="X34" t="n">
+      <c r="Y34" t="n">
         <v>126000</v>
       </c>
-      <c r="Y34" t="n">
+      <c r="Z34" t="n">
         <v>15.4</v>
       </c>
-      <c r="Z34" t="inlineStr">
+      <c r="AA34" t="inlineStr">
         <is>
           <t>Some hormone presence but not the clear focus</t>
         </is>
       </c>
-      <c r="AA34" t="inlineStr">
+      <c r="AB34" t="inlineStr">
         <is>
           <t>https://maps.google.com/?cid=14733224214951654004</t>
         </is>
@@ -3702,39 +3872,44 @@
           <t>N/A</t>
         </is>
       </c>
-      <c r="P35" t="n">
+      <c r="M35" s="1" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="Q35" t="n">
         <v>5</v>
       </c>
-      <c r="Q35" t="n">
+      <c r="R35" t="n">
         <v>34</v>
       </c>
-      <c r="R35" t="n">
+      <c r="S35" t="n">
         <v>0</v>
       </c>
-      <c r="S35" t="n">
+      <c r="T35" t="n">
         <v>1</v>
       </c>
-      <c r="U35" t="n">
+      <c r="V35" t="n">
         <v>144000</v>
       </c>
-      <c r="V35" t="n">
+      <c r="W35" t="n">
         <v>630000</v>
       </c>
-      <c r="W35" t="n">
+      <c r="X35" t="n">
         <v>21600</v>
       </c>
-      <c r="X35" t="n">
+      <c r="Y35" t="n">
         <v>126000</v>
       </c>
-      <c r="Y35" t="n">
+      <c r="Z35" t="n">
         <v>14.5</v>
       </c>
-      <c r="Z35" t="inlineStr">
+      <c r="AA35" t="inlineStr">
         <is>
           <t>Solid hormone line (TRT/HRT focus in name/type) but mixed with other services</t>
         </is>
       </c>
-      <c r="AA35" t="inlineStr">
+      <c r="AB35" t="inlineStr">
         <is>
           <t>https://maps.google.com/?cid=3451373830948402408</t>
         </is>
@@ -3796,42 +3971,47 @@
       </c>
       <c r="L36" t="inlineStr">
         <is>
-          <t>Heather Bartos</t>
-        </is>
-      </c>
-      <c r="P36" t="n">
+          <t>Heather</t>
+        </is>
+      </c>
+      <c r="M36" t="inlineStr">
+        <is>
+          <t>Bartos</t>
+        </is>
+      </c>
+      <c r="Q36" t="n">
         <v>4.5</v>
       </c>
-      <c r="Q36" t="n">
+      <c r="R36" t="n">
         <v>82</v>
       </c>
-      <c r="R36" t="n">
+      <c r="S36" t="n">
         <v>0</v>
       </c>
-      <c r="S36" t="n">
+      <c r="T36" t="n">
         <v>1</v>
       </c>
-      <c r="U36" t="n">
+      <c r="V36" t="n">
         <v>240000</v>
       </c>
-      <c r="V36" t="n">
+      <c r="W36" t="n">
         <v>810000</v>
       </c>
-      <c r="W36" t="n">
+      <c r="X36" t="n">
         <v>36000</v>
       </c>
-      <c r="X36" t="n">
+      <c r="Y36" t="n">
         <v>162000</v>
       </c>
-      <c r="Y36" t="n">
+      <c r="Z36" t="n">
         <v>13</v>
       </c>
-      <c r="Z36" t="inlineStr">
+      <c r="AA36" t="inlineStr">
         <is>
           <t>No hormone, aesthetic, or weight-loss signals detected — may need manual review</t>
         </is>
       </c>
-      <c r="AA36" t="inlineStr">
+      <c r="AB36" t="inlineStr">
         <is>
           <t>https://maps.google.com/?cid=1121924898983120660</t>
         </is>
@@ -3893,45 +4073,50 @@
       </c>
       <c r="L37" t="inlineStr">
         <is>
-          <t>John Gomes</t>
-        </is>
-      </c>
-      <c r="P37" t="n">
+          <t>John</t>
+        </is>
+      </c>
+      <c r="M37" t="inlineStr">
+        <is>
+          <t>Gomes</t>
+        </is>
+      </c>
+      <c r="Q37" t="n">
         <v>4.9</v>
       </c>
-      <c r="Q37" t="n">
+      <c r="R37" t="n">
         <v>75</v>
       </c>
-      <c r="R37" t="n">
+      <c r="S37" t="n">
         <v>1</v>
       </c>
-      <c r="S37" t="n">
+      <c r="T37" t="n">
         <v>2</v>
       </c>
-      <c r="T37" t="n">
+      <c r="U37" t="n">
         <v>25</v>
       </c>
-      <c r="U37" t="n">
+      <c r="V37" t="n">
         <v>240000</v>
       </c>
-      <c r="V37" t="n">
+      <c r="W37" t="n">
         <v>810000</v>
       </c>
-      <c r="W37" t="n">
+      <c r="X37" t="n">
         <v>36000</v>
       </c>
-      <c r="X37" t="n">
+      <c r="Y37" t="n">
         <v>162000</v>
       </c>
-      <c r="Y37" t="n">
+      <c r="Z37" t="n">
         <v>24.9</v>
       </c>
-      <c r="Z37" t="inlineStr">
+      <c r="AA37" t="inlineStr">
         <is>
           <t>No hormone, aesthetic, or weight-loss signals detected — may need manual review</t>
         </is>
       </c>
-      <c r="AA37" t="inlineStr">
+      <c r="AB37" t="inlineStr">
         <is>
           <t>https://maps.google.com/?cid=9949781818478288412</t>
         </is>
@@ -3993,42 +4178,47 @@
       </c>
       <c r="L38" t="inlineStr">
         <is>
-          <t>Jennifer Wright-Bennion</t>
-        </is>
-      </c>
-      <c r="P38" t="n">
+          <t>Jennifer</t>
+        </is>
+      </c>
+      <c r="M38" t="inlineStr">
+        <is>
+          <t>Wright-Bennion</t>
+        </is>
+      </c>
+      <c r="Q38" t="n">
         <v>4</v>
       </c>
-      <c r="Q38" t="n">
+      <c r="R38" t="n">
         <v>237</v>
       </c>
-      <c r="R38" t="n">
+      <c r="S38" t="n">
         <v>1</v>
       </c>
-      <c r="S38" t="n">
+      <c r="T38" t="n">
         <v>4</v>
       </c>
-      <c r="U38" t="n">
+      <c r="V38" t="n">
         <v>240000</v>
       </c>
-      <c r="V38" t="n">
+      <c r="W38" t="n">
         <v>810000</v>
       </c>
-      <c r="W38" t="n">
+      <c r="X38" t="n">
         <v>36000</v>
       </c>
-      <c r="X38" t="n">
+      <c r="Y38" t="n">
         <v>162000</v>
       </c>
-      <c r="Y38" t="n">
+      <c r="Z38" t="n">
         <v>24.5</v>
       </c>
-      <c r="Z38" t="inlineStr">
+      <c r="AA38" t="inlineStr">
         <is>
           <t>No hormone, aesthetic, or weight-loss signals detected — may need manual review</t>
         </is>
       </c>
-      <c r="AA38" t="inlineStr">
+      <c r="AB38" t="inlineStr">
         <is>
           <t>https://maps.google.com/?cid=3079662096953221712</t>
         </is>
@@ -4090,37 +4280,42 @@
       </c>
       <c r="L39" t="inlineStr">
         <is>
-          <t>Larissa Fomitcheva</t>
-        </is>
-      </c>
-      <c r="P39" t="n">
+          <t>Larissa</t>
+        </is>
+      </c>
+      <c r="M39" t="inlineStr">
+        <is>
+          <t>Fomitcheva</t>
+        </is>
+      </c>
+      <c r="Q39" t="n">
         <v>4.7</v>
       </c>
-      <c r="Q39" t="n">
+      <c r="R39" t="n">
         <v>495</v>
       </c>
-      <c r="R39" t="n">
+      <c r="S39" t="n">
         <v>3</v>
       </c>
-      <c r="S39" t="n">
+      <c r="T39" t="n">
         <v>1</v>
       </c>
-      <c r="U39" t="n">
+      <c r="V39" t="n">
         <v>720000</v>
       </c>
-      <c r="V39" t="n">
+      <c r="W39" t="n">
         <v>2430000</v>
       </c>
-      <c r="W39" t="n">
+      <c r="X39" t="n">
         <v>108000</v>
       </c>
-      <c r="X39" t="n">
+      <c r="Y39" t="n">
         <v>486000</v>
       </c>
-      <c r="Y39" t="n">
+      <c r="Z39" t="n">
         <v>22</v>
       </c>
-      <c r="Z39" t="inlineStr">
+      <c r="AA39" t="inlineStr">
         <is>
           <t>No hormone, aesthetic, or weight-loss signals detected — may need manual review</t>
         </is>
@@ -4182,42 +4377,47 @@
       </c>
       <c r="L40" t="inlineStr">
         <is>
-          <t>Kourtney Sims</t>
-        </is>
-      </c>
-      <c r="P40" t="n">
+          <t>Kourtney</t>
+        </is>
+      </c>
+      <c r="M40" t="inlineStr">
+        <is>
+          <t>Sims</t>
+        </is>
+      </c>
+      <c r="Q40" t="n">
         <v>4.8</v>
       </c>
-      <c r="Q40" t="n">
+      <c r="R40" t="n">
         <v>316</v>
       </c>
-      <c r="R40" t="n">
+      <c r="S40" t="n">
         <v>1</v>
       </c>
-      <c r="S40" t="n">
+      <c r="T40" t="n">
         <v>2</v>
       </c>
-      <c r="U40" t="n">
+      <c r="V40" t="n">
         <v>240000</v>
       </c>
-      <c r="V40" t="n">
+      <c r="W40" t="n">
         <v>810000</v>
       </c>
-      <c r="W40" t="n">
+      <c r="X40" t="n">
         <v>36000</v>
       </c>
-      <c r="X40" t="n">
+      <c r="Y40" t="n">
         <v>162000</v>
       </c>
-      <c r="Y40" t="n">
+      <c r="Z40" t="n">
         <v>21.4</v>
       </c>
-      <c r="Z40" t="inlineStr">
+      <c r="AA40" t="inlineStr">
         <is>
           <t>No hormone, aesthetic, or weight-loss signals detected — may need manual review</t>
         </is>
       </c>
-      <c r="AA40" t="inlineStr">
+      <c r="AB40" t="inlineStr">
         <is>
           <t>https://maps.google.com/?cid=6139264796763162758</t>
         </is>
@@ -4279,47 +4479,52 @@
       </c>
       <c r="L41" t="inlineStr">
         <is>
-          <t>Anna Barbieri</t>
+          <t>Anna</t>
         </is>
       </c>
       <c r="M41" t="inlineStr">
         <is>
+          <t>Barbieri</t>
+        </is>
+      </c>
+      <c r="N41" t="inlineStr">
+        <is>
           <t>Founder</t>
         </is>
       </c>
-      <c r="N41" t="inlineStr">
+      <c r="O41" t="inlineStr">
         <is>
           <t>anna.barbieri@annabarbieri-md.com</t>
         </is>
       </c>
-      <c r="P41" t="n">
+      <c r="Q41" t="n">
         <v>4.9</v>
       </c>
-      <c r="Q41" t="n">
+      <c r="R41" t="n">
         <v>178</v>
       </c>
-      <c r="R41" t="n">
+      <c r="S41" t="n">
         <v>3</v>
       </c>
-      <c r="S41" t="n">
+      <c r="T41" t="n">
         <v>1</v>
       </c>
-      <c r="U41" t="n">
+      <c r="V41" t="n">
         <v>720000</v>
       </c>
-      <c r="V41" t="n">
+      <c r="W41" t="n">
         <v>2430000</v>
       </c>
-      <c r="W41" t="n">
+      <c r="X41" t="n">
         <v>108000</v>
       </c>
-      <c r="X41" t="n">
+      <c r="Y41" t="n">
         <v>486000</v>
       </c>
-      <c r="Y41" t="n">
+      <c r="Z41" t="n">
         <v>19.6</v>
       </c>
-      <c r="Z41" t="inlineStr">
+      <c r="AA41" t="inlineStr">
         <is>
           <t>No hormone, aesthetic, or weight-loss signals detected — may need manual review</t>
         </is>
@@ -4376,42 +4581,47 @@
       </c>
       <c r="L42" t="inlineStr">
         <is>
-          <t>Peggy Margetson</t>
-        </is>
-      </c>
-      <c r="P42" t="n">
+          <t>Peggy</t>
+        </is>
+      </c>
+      <c r="M42" t="inlineStr">
+        <is>
+          <t>Margetson</t>
+        </is>
+      </c>
+      <c r="Q42" t="n">
         <v>4.5</v>
       </c>
-      <c r="Q42" t="n">
+      <c r="R42" t="n">
         <v>151</v>
       </c>
-      <c r="R42" t="n">
+      <c r="S42" t="n">
         <v>0</v>
       </c>
-      <c r="S42" t="n">
+      <c r="T42" t="n">
         <v>1</v>
       </c>
-      <c r="U42" t="n">
+      <c r="V42" t="n">
         <v>240000</v>
       </c>
-      <c r="V42" t="n">
+      <c r="W42" t="n">
         <v>810000</v>
       </c>
-      <c r="W42" t="n">
+      <c r="X42" t="n">
         <v>36000</v>
       </c>
-      <c r="X42" t="n">
+      <c r="Y42" t="n">
         <v>162000</v>
       </c>
-      <c r="Y42" t="n">
+      <c r="Z42" t="n">
         <v>16.2</v>
       </c>
-      <c r="Z42" t="inlineStr">
+      <c r="AA42" t="inlineStr">
         <is>
           <t>No hormone, aesthetic, or weight-loss signals detected — may need manual review</t>
         </is>
       </c>
-      <c r="AA42" t="inlineStr">
+      <c r="AB42" t="inlineStr">
         <is>
           <t>https://maps.google.com/?cid=2419533843648232027</t>
         </is>
@@ -4476,39 +4686,39 @@
           <t>Kate</t>
         </is>
       </c>
-      <c r="P43" t="n">
+      <c r="Q43" t="n">
         <v>4.8</v>
       </c>
-      <c r="Q43" t="n">
+      <c r="R43" t="n">
         <v>24</v>
       </c>
-      <c r="R43" t="n">
+      <c r="S43" t="n">
         <v>0</v>
       </c>
-      <c r="S43" t="n">
+      <c r="T43" t="n">
         <v>1</v>
       </c>
-      <c r="U43" t="n">
+      <c r="V43" t="n">
         <v>174000</v>
       </c>
-      <c r="V43" t="n">
+      <c r="W43" t="n">
         <v>777600</v>
       </c>
-      <c r="W43" t="n">
+      <c r="X43" t="n">
         <v>26100</v>
       </c>
-      <c r="X43" t="n">
+      <c r="Y43" t="n">
         <v>155520</v>
       </c>
-      <c r="Y43" t="n">
+      <c r="Z43" t="n">
         <v>13.6</v>
       </c>
-      <c r="Z43" t="inlineStr">
+      <c r="AA43" t="inlineStr">
         <is>
           <t>No hormone, aesthetic, or weight-loss signals detected — may need manual review</t>
         </is>
       </c>
-      <c r="AA43" t="inlineStr">
+      <c r="AB43" t="inlineStr">
         <is>
           <t>https://maps.google.com/?cid=12669565823951710779</t>
         </is>
@@ -4570,42 +4780,47 @@
       </c>
       <c r="L44" t="inlineStr">
         <is>
-          <t>Carolyn Moyers</t>
-        </is>
-      </c>
-      <c r="P44" t="n">
+          <t>Carolyn</t>
+        </is>
+      </c>
+      <c r="M44" t="inlineStr">
+        <is>
+          <t>Moyers</t>
+        </is>
+      </c>
+      <c r="Q44" t="n">
         <v>4.9</v>
       </c>
-      <c r="Q44" t="n">
+      <c r="R44" t="n">
         <v>115</v>
-      </c>
-      <c r="R44" t="n">
-        <v>1</v>
       </c>
       <c r="S44" t="n">
         <v>1</v>
       </c>
-      <c r="U44" t="n">
+      <c r="T44" t="n">
+        <v>1</v>
+      </c>
+      <c r="V44" t="n">
         <v>240000</v>
       </c>
-      <c r="V44" t="n">
+      <c r="W44" t="n">
         <v>810000</v>
       </c>
-      <c r="W44" t="n">
+      <c r="X44" t="n">
         <v>36000</v>
       </c>
-      <c r="X44" t="n">
+      <c r="Y44" t="n">
         <v>162000</v>
       </c>
-      <c r="Y44" t="n">
+      <c r="Z44" t="n">
         <v>13</v>
       </c>
-      <c r="Z44" t="inlineStr">
+      <c r="AA44" t="inlineStr">
         <is>
           <t>No hormone, aesthetic, or weight-loss signals detected — may need manual review</t>
         </is>
       </c>
-      <c r="AA44" t="inlineStr">
+      <c r="AB44" t="inlineStr">
         <is>
           <t>https://maps.google.com/?cid=5590681435626343068</t>
         </is>
@@ -4670,42 +4885,47 @@
           <t>N/A</t>
         </is>
       </c>
-      <c r="P45" t="n">
+      <c r="M45" s="1" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="Q45" t="n">
         <v>4.8</v>
       </c>
-      <c r="Q45" t="n">
+      <c r="R45" t="n">
         <v>820</v>
       </c>
-      <c r="R45" t="n">
+      <c r="S45" t="n">
         <v>6</v>
       </c>
-      <c r="S45" t="n">
+      <c r="T45" t="n">
         <v>4</v>
       </c>
-      <c r="T45" t="n">
+      <c r="U45" t="n">
         <v>27</v>
       </c>
-      <c r="U45" t="n">
+      <c r="V45" t="n">
         <v>1440000</v>
       </c>
-      <c r="V45" t="n">
+      <c r="W45" t="n">
         <v>4860000</v>
       </c>
-      <c r="W45" t="n">
+      <c r="X45" t="n">
         <v>288000</v>
       </c>
-      <c r="X45" t="n">
+      <c r="Y45" t="n">
         <v>1360800</v>
       </c>
-      <c r="Y45" t="n">
+      <c r="Z45" t="n">
         <v>30</v>
       </c>
-      <c r="Z45" t="inlineStr">
+      <c r="AA45" t="inlineStr">
         <is>
           <t>No hormone, aesthetic, or weight-loss signals detected — may need manual review</t>
         </is>
       </c>
-      <c r="AA45" t="inlineStr">
+      <c r="AB45" t="inlineStr">
         <is>
           <t>https://maps.google.com/?cid=17675827022667488007</t>
         </is>
@@ -4770,39 +4990,44 @@
           <t>N/A</t>
         </is>
       </c>
-      <c r="P46" t="n">
+      <c r="M46" s="1" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="Q46" t="n">
         <v>4.9</v>
       </c>
-      <c r="Q46" t="n">
+      <c r="R46" t="n">
         <v>147</v>
       </c>
-      <c r="R46" t="n">
+      <c r="S46" t="n">
         <v>7</v>
       </c>
-      <c r="S46" t="n">
+      <c r="T46" t="n">
         <v>3</v>
       </c>
-      <c r="U46" t="n">
+      <c r="V46" t="n">
         <v>1680000</v>
       </c>
-      <c r="V46" t="n">
+      <c r="W46" t="n">
         <v>5670000</v>
       </c>
-      <c r="W46" t="n">
+      <c r="X46" t="n">
         <v>336000</v>
       </c>
-      <c r="X46" t="n">
+      <c r="Y46" t="n">
         <v>1587600</v>
       </c>
-      <c r="Y46" t="n">
+      <c r="Z46" t="n">
         <v>28.8</v>
       </c>
-      <c r="Z46" t="inlineStr">
+      <c r="AA46" t="inlineStr">
         <is>
           <t>No hormone, aesthetic, or weight-loss signals detected — may need manual review</t>
         </is>
       </c>
-      <c r="AA46" t="inlineStr">
+      <c r="AB46" t="inlineStr">
         <is>
           <t>https://maps.google.com/?cid=14680874791404527832</t>
         </is>
@@ -4864,42 +5089,47 @@
       </c>
       <c r="L47" t="inlineStr">
         <is>
-          <t>Laquita Martinez</t>
-        </is>
-      </c>
-      <c r="P47" t="n">
+          <t>Laquita</t>
+        </is>
+      </c>
+      <c r="M47" t="inlineStr">
+        <is>
+          <t>Martinez</t>
+        </is>
+      </c>
+      <c r="Q47" t="n">
         <v>4.6</v>
       </c>
-      <c r="Q47" t="n">
+      <c r="R47" t="n">
         <v>421</v>
       </c>
-      <c r="R47" t="n">
+      <c r="S47" t="n">
         <v>3</v>
       </c>
-      <c r="S47" t="n">
+      <c r="T47" t="n">
         <v>2</v>
       </c>
-      <c r="U47" t="n">
+      <c r="V47" t="n">
         <v>720000</v>
       </c>
-      <c r="V47" t="n">
+      <c r="W47" t="n">
         <v>2430000</v>
       </c>
-      <c r="W47" t="n">
+      <c r="X47" t="n">
         <v>108000</v>
       </c>
-      <c r="X47" t="n">
+      <c r="Y47" t="n">
         <v>486000</v>
       </c>
-      <c r="Y47" t="n">
+      <c r="Z47" t="n">
         <v>28.2</v>
       </c>
-      <c r="Z47" t="inlineStr">
+      <c r="AA47" t="inlineStr">
         <is>
           <t>No hormone, aesthetic, or weight-loss signals detected — may need manual review</t>
         </is>
       </c>
-      <c r="AA47" t="inlineStr">
+      <c r="AB47" t="inlineStr">
         <is>
           <t>https://maps.google.com/?cid=11256095281223431806</t>
         </is>
@@ -4964,39 +5194,44 @@
           <t>N/A</t>
         </is>
       </c>
-      <c r="P48" t="n">
+      <c r="M48" s="1" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="Q48" t="n">
         <v>4.8</v>
       </c>
-      <c r="Q48" t="n">
+      <c r="R48" t="n">
         <v>952</v>
       </c>
-      <c r="R48" t="n">
+      <c r="S48" t="n">
         <v>2</v>
       </c>
-      <c r="S48" t="n">
+      <c r="T48" t="n">
         <v>11</v>
       </c>
-      <c r="U48" t="n">
+      <c r="V48" t="n">
         <v>480000</v>
       </c>
-      <c r="V48" t="n">
+      <c r="W48" t="n">
         <v>1620000</v>
       </c>
-      <c r="W48" t="n">
+      <c r="X48" t="n">
         <v>72000</v>
       </c>
-      <c r="X48" t="n">
+      <c r="Y48" t="n">
         <v>324000</v>
       </c>
-      <c r="Y48" t="n">
+      <c r="Z48" t="n">
         <v>25.1</v>
       </c>
-      <c r="Z48" t="inlineStr">
+      <c r="AA48" t="inlineStr">
         <is>
           <t>No hormone, aesthetic, or weight-loss signals detected — may need manual review</t>
         </is>
       </c>
-      <c r="AA48" t="inlineStr">
+      <c r="AB48" t="inlineStr">
         <is>
           <t>https://maps.google.com/?cid=3012814511327277171</t>
         </is>
@@ -5058,42 +5293,47 @@
       </c>
       <c r="L49" t="inlineStr">
         <is>
-          <t>Ann Cha</t>
-        </is>
-      </c>
-      <c r="P49" t="n">
+          <t>Ann</t>
+        </is>
+      </c>
+      <c r="M49" t="inlineStr">
+        <is>
+          <t>Cha</t>
+        </is>
+      </c>
+      <c r="Q49" t="n">
         <v>4.7</v>
       </c>
-      <c r="Q49" t="n">
+      <c r="R49" t="n">
         <v>181</v>
       </c>
-      <c r="R49" t="n">
+      <c r="S49" t="n">
         <v>2</v>
       </c>
-      <c r="S49" t="n">
+      <c r="T49" t="n">
         <v>4</v>
       </c>
-      <c r="U49" t="n">
+      <c r="V49" t="n">
         <v>480000</v>
       </c>
-      <c r="V49" t="n">
+      <c r="W49" t="n">
         <v>1620000</v>
       </c>
-      <c r="W49" t="n">
+      <c r="X49" t="n">
         <v>72000</v>
       </c>
-      <c r="X49" t="n">
+      <c r="Y49" t="n">
         <v>324000</v>
       </c>
-      <c r="Y49" t="n">
+      <c r="Z49" t="n">
         <v>24.7</v>
       </c>
-      <c r="Z49" t="inlineStr">
+      <c r="AA49" t="inlineStr">
         <is>
           <t>No hormone, aesthetic, or weight-loss signals detected — may need manual review</t>
         </is>
       </c>
-      <c r="AA49" t="inlineStr">
+      <c r="AB49" t="inlineStr">
         <is>
           <t>https://maps.google.com/?cid=4668856987148793075</t>
         </is>
@@ -5155,50 +5395,55 @@
       </c>
       <c r="L50" t="inlineStr">
         <is>
-          <t>Norman Lamberty</t>
+          <t>Norman</t>
         </is>
       </c>
       <c r="M50" t="inlineStr">
         <is>
+          <t>Lamberty</t>
+        </is>
+      </c>
+      <c r="N50" t="inlineStr">
+        <is>
           <t>President (NPI Authorized Official)</t>
         </is>
       </c>
-      <c r="N50" t="inlineStr">
+      <c r="O50" t="inlineStr">
         <is>
           <t>nlamberty@aawomenshealth.com</t>
         </is>
       </c>
-      <c r="P50" t="n">
+      <c r="Q50" t="n">
         <v>4.2</v>
       </c>
-      <c r="Q50" t="n">
+      <c r="R50" t="n">
         <v>111</v>
       </c>
-      <c r="R50" t="n">
+      <c r="S50" t="n">
         <v>0</v>
       </c>
-      <c r="S50" t="n">
+      <c r="T50" t="n">
         <v>1</v>
       </c>
-      <c r="T50" t="n">
+      <c r="U50" t="n">
         <v>7</v>
       </c>
-      <c r="U50" t="n">
+      <c r="V50" t="n">
         <v>144000</v>
       </c>
-      <c r="V50" t="n">
+      <c r="W50" t="n">
         <v>630000</v>
       </c>
-      <c r="W50" t="n">
+      <c r="X50" t="n">
         <v>21600</v>
       </c>
-      <c r="X50" t="n">
+      <c r="Y50" t="n">
         <v>126000</v>
       </c>
-      <c r="Y50" t="n">
+      <c r="Z50" t="n">
         <v>21.6</v>
       </c>
-      <c r="Z50" t="inlineStr">
+      <c r="AA50" t="inlineStr">
         <is>
           <t>No hormone, aesthetic, or weight-loss signals detected — may need manual review</t>
         </is>
@@ -5260,42 +5505,47 @@
       </c>
       <c r="L51" t="inlineStr">
         <is>
-          <t>Angela Hudson</t>
-        </is>
-      </c>
-      <c r="P51" t="n">
+          <t>Angela</t>
+        </is>
+      </c>
+      <c r="M51" t="inlineStr">
+        <is>
+          <t>Hudson</t>
+        </is>
+      </c>
+      <c r="Q51" t="n">
         <v>4.9</v>
       </c>
-      <c r="Q51" t="n">
+      <c r="R51" t="n">
         <v>1498</v>
       </c>
-      <c r="R51" t="n">
+      <c r="S51" t="n">
         <v>0</v>
       </c>
-      <c r="S51" t="n">
+      <c r="T51" t="n">
         <v>1</v>
       </c>
-      <c r="U51" t="n">
+      <c r="V51" t="n">
         <v>240000</v>
       </c>
-      <c r="V51" t="n">
+      <c r="W51" t="n">
         <v>810000</v>
       </c>
-      <c r="W51" t="n">
+      <c r="X51" t="n">
         <v>36000</v>
       </c>
-      <c r="X51" t="n">
+      <c r="Y51" t="n">
         <v>162000</v>
       </c>
-      <c r="Y51" t="n">
+      <c r="Z51" t="n">
         <v>17.8</v>
       </c>
-      <c r="Z51" t="inlineStr">
+      <c r="AA51" t="inlineStr">
         <is>
           <t>No hormone, aesthetic, or weight-loss signals detected — may need manual review</t>
         </is>
       </c>
-      <c r="AA51" t="inlineStr">
+      <c r="AB51" t="inlineStr">
         <is>
           <t>https://maps.google.com/?cid=7424703015494272824</t>
         </is>
@@ -5360,39 +5610,44 @@
           <t>N/A</t>
         </is>
       </c>
-      <c r="P52" t="n">
+      <c r="M52" s="1" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="Q52" t="n">
         <v>4.4</v>
       </c>
-      <c r="Q52" t="n">
+      <c r="R52" t="n">
         <v>78</v>
       </c>
-      <c r="R52" t="n">
+      <c r="S52" t="n">
         <v>4</v>
       </c>
-      <c r="S52" t="n">
+      <c r="T52" t="n">
         <v>1</v>
       </c>
-      <c r="U52" t="n">
+      <c r="V52" t="n">
         <v>561000</v>
       </c>
-      <c r="V52" t="n">
+      <c r="W52" t="n">
         <v>2527200</v>
       </c>
-      <c r="W52" t="n">
+      <c r="X52" t="n">
         <v>84150</v>
       </c>
-      <c r="X52" t="n">
+      <c r="Y52" t="n">
         <v>505440</v>
       </c>
-      <c r="Y52" t="n">
+      <c r="Z52" t="n">
         <v>16.3</v>
       </c>
-      <c r="Z52" t="inlineStr">
+      <c r="AA52" t="inlineStr">
         <is>
           <t>No hormone, aesthetic, or weight-loss signals detected — may need manual review</t>
         </is>
       </c>
-      <c r="AA52" t="inlineStr">
+      <c r="AB52" t="inlineStr">
         <is>
           <t>https://maps.google.com/?cid=670280380779986887</t>
         </is>
@@ -5457,39 +5712,44 @@
           <t>N/A</t>
         </is>
       </c>
-      <c r="P53" t="n">
+      <c r="M53" s="1" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="Q53" t="n">
         <v>4.6</v>
       </c>
-      <c r="Q53" t="n">
+      <c r="R53" t="n">
         <v>748</v>
-      </c>
-      <c r="R53" t="n">
-        <v>1</v>
       </c>
       <c r="S53" t="n">
         <v>1</v>
       </c>
-      <c r="U53" t="n">
+      <c r="T53" t="n">
+        <v>1</v>
+      </c>
+      <c r="V53" t="n">
         <v>240000</v>
       </c>
-      <c r="V53" t="n">
+      <c r="W53" t="n">
         <v>810000</v>
       </c>
-      <c r="W53" t="n">
+      <c r="X53" t="n">
         <v>36000</v>
       </c>
-      <c r="X53" t="n">
+      <c r="Y53" t="n">
         <v>162000</v>
       </c>
-      <c r="Y53" t="n">
+      <c r="Z53" t="n">
         <v>15.1</v>
       </c>
-      <c r="Z53" t="inlineStr">
+      <c r="AA53" t="inlineStr">
         <is>
           <t>No hormone, aesthetic, or weight-loss signals detected — may need manual review</t>
         </is>
       </c>
-      <c r="AA53" t="inlineStr">
+      <c r="AB53" t="inlineStr">
         <is>
           <t>https://maps.google.com/?cid=14751170150070329707</t>
         </is>
@@ -5551,42 +5811,47 @@
       </c>
       <c r="L54" t="inlineStr">
         <is>
-          <t>Drew Howard</t>
-        </is>
-      </c>
-      <c r="P54" t="n">
+          <t>Drew</t>
+        </is>
+      </c>
+      <c r="M54" t="inlineStr">
+        <is>
+          <t>Howard</t>
+        </is>
+      </c>
+      <c r="Q54" t="n">
         <v>4.8</v>
       </c>
-      <c r="Q54" t="n">
+      <c r="R54" t="n">
         <v>730</v>
       </c>
-      <c r="R54" t="n">
+      <c r="S54" t="n">
         <v>0</v>
       </c>
-      <c r="S54" t="n">
+      <c r="T54" t="n">
         <v>1</v>
       </c>
-      <c r="U54" t="n">
+      <c r="V54" t="n">
         <v>240000</v>
       </c>
-      <c r="V54" t="n">
+      <c r="W54" t="n">
         <v>810000</v>
       </c>
-      <c r="W54" t="n">
+      <c r="X54" t="n">
         <v>36000</v>
       </c>
-      <c r="X54" t="n">
+      <c r="Y54" t="n">
         <v>162000</v>
       </c>
-      <c r="Y54" t="n">
+      <c r="Z54" t="n">
         <v>12.1</v>
       </c>
-      <c r="Z54" t="inlineStr">
+      <c r="AA54" t="inlineStr">
         <is>
           <t>No hormone, aesthetic, or weight-loss signals detected — may need manual review</t>
         </is>
       </c>
-      <c r="AA54" t="inlineStr">
+      <c r="AB54" t="inlineStr">
         <is>
           <t>https://maps.google.com/?cid=11836478338825250552</t>
         </is>
@@ -5651,39 +5916,44 @@
           <t>N/A</t>
         </is>
       </c>
-      <c r="P55" t="n">
+      <c r="M55" s="1" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="Q55" t="n">
         <v>4</v>
       </c>
-      <c r="Q55" t="n">
+      <c r="R55" t="n">
         <v>284</v>
       </c>
-      <c r="R55" t="n">
+      <c r="S55" t="n">
         <v>0</v>
       </c>
-      <c r="S55" t="n">
+      <c r="T55" t="n">
         <v>1</v>
       </c>
-      <c r="U55" t="n">
+      <c r="V55" t="n">
         <v>240000</v>
       </c>
-      <c r="V55" t="n">
+      <c r="W55" t="n">
         <v>810000</v>
       </c>
-      <c r="W55" t="n">
+      <c r="X55" t="n">
         <v>36000</v>
       </c>
-      <c r="X55" t="n">
+      <c r="Y55" t="n">
         <v>162000</v>
       </c>
-      <c r="Y55" t="n">
+      <c r="Z55" t="n">
         <v>12</v>
       </c>
-      <c r="Z55" t="inlineStr">
+      <c r="AA55" t="inlineStr">
         <is>
           <t>No hormone, aesthetic, or weight-loss signals detected — may need manual review</t>
         </is>
       </c>
-      <c r="AA55" t="inlineStr">
+      <c r="AB55" t="inlineStr">
         <is>
           <t>https://maps.google.com/?cid=13518531309886247844</t>
         </is>
@@ -5748,39 +6018,44 @@
           <t>N/A</t>
         </is>
       </c>
-      <c r="P56" t="n">
+      <c r="M56" s="1" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="Q56" t="n">
         <v>5</v>
       </c>
-      <c r="Q56" t="n">
+      <c r="R56" t="n">
         <v>60</v>
-      </c>
-      <c r="R56" t="n">
-        <v>1</v>
       </c>
       <c r="S56" t="n">
         <v>1</v>
       </c>
-      <c r="U56" t="n">
+      <c r="T56" t="n">
+        <v>1</v>
+      </c>
+      <c r="V56" t="n">
         <v>240000</v>
       </c>
-      <c r="V56" t="n">
+      <c r="W56" t="n">
         <v>810000</v>
       </c>
-      <c r="W56" t="n">
+      <c r="X56" t="n">
         <v>36000</v>
       </c>
-      <c r="X56" t="n">
+      <c r="Y56" t="n">
         <v>162000</v>
       </c>
-      <c r="Y56" t="n">
+      <c r="Z56" t="n">
         <v>9.6</v>
       </c>
-      <c r="Z56" t="inlineStr">
+      <c r="AA56" t="inlineStr">
         <is>
           <t>No hormone, aesthetic, or weight-loss signals detected — may need manual review</t>
         </is>
       </c>
-      <c r="AA56" t="inlineStr">
+      <c r="AB56" t="inlineStr">
         <is>
           <t>https://maps.google.com/?cid=15490659819503068341</t>
         </is>
@@ -5845,39 +6120,44 @@
           <t>N/A</t>
         </is>
       </c>
-      <c r="P57" t="n">
+      <c r="M57" s="1" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="Q57" t="n">
         <v>4.4</v>
       </c>
-      <c r="Q57" t="n">
+      <c r="R57" t="n">
         <v>263</v>
       </c>
-      <c r="R57" t="n">
+      <c r="S57" t="n">
         <v>1</v>
       </c>
-      <c r="S57" t="n">
+      <c r="T57" t="n">
         <v>2</v>
       </c>
-      <c r="U57" t="n">
+      <c r="V57" t="n">
         <v>240000</v>
       </c>
-      <c r="V57" t="n">
+      <c r="W57" t="n">
         <v>810000</v>
       </c>
-      <c r="W57" t="n">
+      <c r="X57" t="n">
         <v>36000</v>
       </c>
-      <c r="X57" t="n">
+      <c r="Y57" t="n">
         <v>162000</v>
       </c>
-      <c r="Y57" t="n">
+      <c r="Z57" t="n">
         <v>24</v>
       </c>
-      <c r="Z57" t="inlineStr">
+      <c r="AA57" t="inlineStr">
         <is>
           <t>No hormone, aesthetic, or weight-loss signals detected — may need manual review</t>
         </is>
       </c>
-      <c r="AA57" t="inlineStr">
+      <c r="AB57" t="inlineStr">
         <is>
           <t>https://maps.google.com/?cid=12070823049643313317</t>
         </is>
@@ -5937,39 +6217,44 @@
           <t>N/A</t>
         </is>
       </c>
-      <c r="P58" t="n">
+      <c r="M58" s="1" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="Q58" t="n">
         <v>4.9</v>
       </c>
-      <c r="Q58" t="n">
+      <c r="R58" t="n">
         <v>133</v>
       </c>
-      <c r="R58" t="n">
+      <c r="S58" t="n">
         <v>0</v>
       </c>
-      <c r="S58" t="n">
+      <c r="T58" t="n">
         <v>1</v>
       </c>
-      <c r="U58" t="n">
+      <c r="V58" t="n">
         <v>240000</v>
       </c>
-      <c r="V58" t="n">
+      <c r="W58" t="n">
         <v>810000</v>
       </c>
-      <c r="W58" t="n">
+      <c r="X58" t="n">
         <v>36000</v>
       </c>
-      <c r="X58" t="n">
+      <c r="Y58" t="n">
         <v>162000</v>
       </c>
-      <c r="Y58" t="n">
+      <c r="Z58" t="n">
         <v>8.5</v>
       </c>
-      <c r="Z58" t="inlineStr">
+      <c r="AA58" t="inlineStr">
         <is>
           <t>No hormone, aesthetic, or weight-loss signals detected — may need manual review</t>
         </is>
       </c>
-      <c r="AA58" t="inlineStr">
+      <c r="AB58" t="inlineStr">
         <is>
           <t>https://maps.google.com/?cid=30577582817643106</t>
         </is>

</xml_diff>

<commit_message>
Fill Exec Title from CEO Results, highlight missing as N/A in red
https://claude.ai/code/session_01917JoB1LXoWCAoYuucjGiV
</commit_message>
<xml_diff>
--- a/Womens_HRT_Hormones_Only_New_cleaned_updated.xlsx
+++ b/Womens_HRT_Hormones_Only_New_cleaned_updated.xlsx
@@ -829,6 +829,11 @@
           <t>Jackson-Sekunda</t>
         </is>
       </c>
+      <c r="N4" t="inlineStr">
+        <is>
+          <t>President / CEO &amp; Founder</t>
+        </is>
+      </c>
       <c r="P4" t="inlineStr">
         <is>
           <t>https://www.linkedin.com/company/bff-medical-wellness-clinic/</t>
@@ -1023,6 +1028,11 @@
           <t>Potter</t>
         </is>
       </c>
+      <c r="N6" t="inlineStr">
+        <is>
+          <t>Co-Founder &amp; Nurse Practitioner</t>
+        </is>
+      </c>
       <c r="Q6" t="n">
         <v>5</v>
       </c>
@@ -1120,6 +1130,11 @@
           <t>Houston</t>
         </is>
       </c>
+      <c r="N7" t="inlineStr">
+        <is>
+          <t>Founder &amp; Nurse Practitioner</t>
+        </is>
+      </c>
       <c r="Q7" t="n">
         <v>4.9</v>
       </c>
@@ -1851,6 +1866,11 @@
           <t>Perdue</t>
         </is>
       </c>
+      <c r="N14" t="inlineStr">
+        <is>
+          <t>Lead Nurse Practitioner &amp; Medical Director (DNP, FNP)</t>
+        </is>
+      </c>
       <c r="Q14" t="n">
         <v>5</v>
       </c>
@@ -1933,12 +1953,7 @@
           <t>8127 Mulberry Ave Ste 108</t>
         </is>
       </c>
-      <c r="L15" s="1" t="inlineStr">
-        <is>
-          <t>N/A</t>
-        </is>
-      </c>
-      <c r="M15" s="1" t="inlineStr">
+      <c r="N15" s="1" t="inlineStr">
         <is>
           <t>N/A</t>
         </is>
@@ -2142,6 +2157,11 @@
           <t>Utter</t>
         </is>
       </c>
+      <c r="N17" t="inlineStr">
+        <is>
+          <t>Owner / Esthetician (Business Management &amp; Principal Contact)</t>
+        </is>
+      </c>
       <c r="Q17" t="n">
         <v>4.8</v>
       </c>
@@ -2234,6 +2254,11 @@
           <t>Kaufman</t>
         </is>
       </c>
+      <c r="N18" t="inlineStr">
+        <is>
+          <t>Medical Director / Anti-Aging and Regenerative Medicine Specialist</t>
+        </is>
+      </c>
       <c r="Q18" t="n">
         <v>5</v>
       </c>
@@ -2331,6 +2356,11 @@
           <t>Nguyen</t>
         </is>
       </c>
+      <c r="N19" t="inlineStr">
+        <is>
+          <t>Physician / Medical Director</t>
+        </is>
+      </c>
       <c r="Q19" t="n">
         <v>4.8</v>
       </c>
@@ -2418,12 +2448,7 @@
           <t>14115 S Dixie Hwy SUITE H, Palmetto Bay, FL 33176, USA</t>
         </is>
       </c>
-      <c r="L20" s="1" t="inlineStr">
-        <is>
-          <t>N/A</t>
-        </is>
-      </c>
-      <c r="M20" s="1" t="inlineStr">
+      <c r="N20" s="1" t="inlineStr">
         <is>
           <t>N/A</t>
         </is>
@@ -2525,6 +2550,11 @@
           <t>Abdullah</t>
         </is>
       </c>
+      <c r="N21" t="inlineStr">
+        <is>
+          <t>Founder &amp; Medical Director</t>
+        </is>
+      </c>
       <c r="Q21" t="n">
         <v>4.8</v>
       </c>
@@ -2617,6 +2647,11 @@
           <t>Masrour</t>
         </is>
       </c>
+      <c r="N22" t="inlineStr">
+        <is>
+          <t>Founder &amp; Medical Director (Lead Physician)</t>
+        </is>
+      </c>
       <c r="Q22" t="n">
         <v>4.2</v>
       </c>
@@ -2709,6 +2744,11 @@
           <t>Kemp</t>
         </is>
       </c>
+      <c r="N23" t="inlineStr">
+        <is>
+          <t>Founder &amp; Family Nurse Practitioner</t>
+        </is>
+      </c>
       <c r="Q23" t="n">
         <v>5</v>
       </c>
@@ -2806,6 +2846,11 @@
           <t>Lobe</t>
         </is>
       </c>
+      <c r="N24" t="inlineStr">
+        <is>
+          <t>Founder &amp; Medical Director</t>
+        </is>
+      </c>
       <c r="Q24" t="n">
         <v>4.5</v>
       </c>
@@ -2898,6 +2943,11 @@
           <t>Casida</t>
         </is>
       </c>
+      <c r="N25" t="inlineStr">
+        <is>
+          <t>Founder, FNP-C</t>
+        </is>
+      </c>
       <c r="Q25" t="n">
         <v>5</v>
       </c>
@@ -2995,6 +3045,11 @@
           <t>Davis</t>
         </is>
       </c>
+      <c r="N26" t="inlineStr">
+        <is>
+          <t>Founder &amp; Medical Director (Physician, MD, MSCP)</t>
+        </is>
+      </c>
       <c r="Q26" t="n">
         <v>4.9</v>
       </c>
@@ -3092,6 +3147,11 @@
           <t>Risner</t>
         </is>
       </c>
+      <c r="N27" t="inlineStr">
+        <is>
+          <t>CEO</t>
+        </is>
+      </c>
       <c r="Q27" t="n">
         <v>5</v>
       </c>
@@ -3189,6 +3249,11 @@
           <t>Aiello</t>
         </is>
       </c>
+      <c r="N28" t="inlineStr">
+        <is>
+          <t>Medical Director (Osteopathic Physician, D.O.)</t>
+        </is>
+      </c>
       <c r="Q28" t="n">
         <v>4.9</v>
       </c>
@@ -3289,6 +3354,11 @@
           <t>Gaudry</t>
         </is>
       </c>
+      <c r="N29" t="inlineStr">
+        <is>
+          <t>Medical Director</t>
+        </is>
+      </c>
       <c r="Q29" t="n">
         <v>4.7</v>
       </c>
@@ -3386,6 +3456,11 @@
           <t>Smith</t>
         </is>
       </c>
+      <c r="N30" t="inlineStr">
+        <is>
+          <t>Founder &amp; Nurse Practitioner (APRN, FNP-C)</t>
+        </is>
+      </c>
       <c r="Q30" t="n">
         <v>5</v>
       </c>
@@ -3478,12 +3553,7 @@
           <t>3405 Dallas Hwy Suite 200, Marietta, GA 30064, USA</t>
         </is>
       </c>
-      <c r="L31" s="1" t="inlineStr">
-        <is>
-          <t>N/A</t>
-        </is>
-      </c>
-      <c r="M31" s="1" t="inlineStr">
+      <c r="N31" s="1" t="inlineStr">
         <is>
           <t>N/A</t>
         </is>
@@ -3588,6 +3658,11 @@
           <t>Melikyan</t>
         </is>
       </c>
+      <c r="N32" t="inlineStr">
+        <is>
+          <t>Founder &amp; Medical Director (N.M.D.)</t>
+        </is>
+      </c>
       <c r="Q32" t="n">
         <v>5</v>
       </c>
@@ -3688,6 +3763,11 @@
           <t>Sharhan</t>
         </is>
       </c>
+      <c r="N33" t="inlineStr">
+        <is>
+          <t>Medical Director</t>
+        </is>
+      </c>
       <c r="Q33" t="n">
         <v>5</v>
       </c>
@@ -3775,12 +3855,7 @@
           <t>90 W Main St, Victor, NY 14564, USA</t>
         </is>
       </c>
-      <c r="L34" s="1" t="inlineStr">
-        <is>
-          <t>N/A</t>
-        </is>
-      </c>
-      <c r="M34" s="1" t="inlineStr">
+      <c r="N34" s="1" t="inlineStr">
         <is>
           <t>N/A</t>
         </is>
@@ -3867,12 +3942,7 @@
           <t>1529 E Interstate 30 #108, Garland, TX 75043, USA</t>
         </is>
       </c>
-      <c r="L35" s="1" t="inlineStr">
-        <is>
-          <t>N/A</t>
-        </is>
-      </c>
-      <c r="M35" s="1" t="inlineStr">
+      <c r="N35" s="1" t="inlineStr">
         <is>
           <t>N/A</t>
         </is>
@@ -3979,6 +4049,11 @@
           <t>Bartos</t>
         </is>
       </c>
+      <c r="N36" t="inlineStr">
+        <is>
+          <t>Medical Director</t>
+        </is>
+      </c>
       <c r="Q36" t="n">
         <v>4.5</v>
       </c>
@@ -4081,6 +4156,11 @@
           <t>Gomes</t>
         </is>
       </c>
+      <c r="N37" t="inlineStr">
+        <is>
+          <t>Medical Director</t>
+        </is>
+      </c>
       <c r="Q37" t="n">
         <v>4.9</v>
       </c>
@@ -4186,6 +4266,11 @@
           <t>Wright-Bennion</t>
         </is>
       </c>
+      <c r="N38" t="inlineStr">
+        <is>
+          <t>Founder &amp; Owner (CNM, APRN)</t>
+        </is>
+      </c>
       <c r="Q38" t="n">
         <v>4</v>
       </c>
@@ -4288,6 +4373,11 @@
           <t>Fomitcheva</t>
         </is>
       </c>
+      <c r="N39" t="inlineStr">
+        <is>
+          <t>OB-GYN / Practice Lead (Medical Director)</t>
+        </is>
+      </c>
       <c r="Q39" t="n">
         <v>4.7</v>
       </c>
@@ -4385,6 +4475,11 @@
           <t>Sims</t>
         </is>
       </c>
+      <c r="N40" t="inlineStr">
+        <is>
+          <t>Medical Director</t>
+        </is>
+      </c>
       <c r="Q40" t="n">
         <v>4.8</v>
       </c>
@@ -4589,6 +4684,11 @@
           <t>Margetson</t>
         </is>
       </c>
+      <c r="N42" t="inlineStr">
+        <is>
+          <t>Founder &amp; CEO</t>
+        </is>
+      </c>
       <c r="Q42" t="n">
         <v>4.5</v>
       </c>
@@ -4686,6 +4786,11 @@
           <t>Kate</t>
         </is>
       </c>
+      <c r="N43" t="inlineStr">
+        <is>
+          <t>Founder &amp; Women's Health Nurse Practitioner / Certified Nurse Midwife</t>
+        </is>
+      </c>
       <c r="Q43" t="n">
         <v>4.8</v>
       </c>
@@ -4788,6 +4893,11 @@
           <t>Moyers</t>
         </is>
       </c>
+      <c r="N44" t="inlineStr">
+        <is>
+          <t>Founder &amp; OB-GYN (Medical Director)</t>
+        </is>
+      </c>
       <c r="Q44" t="n">
         <v>4.9</v>
       </c>
@@ -4880,12 +4990,7 @@
           <t>2460 N Interstate 35 E Rd Suite 165, Waxahachie, TX 75165, USA</t>
         </is>
       </c>
-      <c r="L45" s="1" t="inlineStr">
-        <is>
-          <t>N/A</t>
-        </is>
-      </c>
-      <c r="M45" s="1" t="inlineStr">
+      <c r="N45" s="1" t="inlineStr">
         <is>
           <t>N/A</t>
         </is>
@@ -4985,12 +5090,7 @@
           <t>207 E 94th St 5th floor, New York, NY 10128, USA</t>
         </is>
       </c>
-      <c r="L46" s="1" t="inlineStr">
-        <is>
-          <t>N/A</t>
-        </is>
-      </c>
-      <c r="M46" s="1" t="inlineStr">
+      <c r="N46" s="1" t="inlineStr">
         <is>
           <t>N/A</t>
         </is>
@@ -5097,6 +5197,11 @@
           <t>Martinez</t>
         </is>
       </c>
+      <c r="N47" t="inlineStr">
+        <is>
+          <t>Founder &amp; Physician (Medical Director)</t>
+        </is>
+      </c>
       <c r="Q47" t="n">
         <v>4.6</v>
       </c>
@@ -5189,12 +5294,7 @@
           <t>3237 Blue Ridge Rd, Raleigh, NC 27612, USA</t>
         </is>
       </c>
-      <c r="L48" s="1" t="inlineStr">
-        <is>
-          <t>N/A</t>
-        </is>
-      </c>
-      <c r="M48" s="1" t="inlineStr">
+      <c r="N48" s="1" t="inlineStr">
         <is>
           <t>N/A</t>
         </is>
@@ -5301,6 +5401,11 @@
           <t>Cha</t>
         </is>
       </c>
+      <c r="N49" t="inlineStr">
+        <is>
+          <t>Founder &amp; OB-GYN (Medical Director)</t>
+        </is>
+      </c>
       <c r="Q49" t="n">
         <v>4.7</v>
       </c>
@@ -5513,6 +5618,11 @@
           <t>Hudson</t>
         </is>
       </c>
+      <c r="N51" t="inlineStr">
+        <is>
+          <t>Medical Director</t>
+        </is>
+      </c>
       <c r="Q51" t="n">
         <v>4.9</v>
       </c>
@@ -5605,12 +5715,7 @@
           <t>9940 Talbert Ave #303, Fountain Valley, CA 92708, USA</t>
         </is>
       </c>
-      <c r="L52" s="1" t="inlineStr">
-        <is>
-          <t>N/A</t>
-        </is>
-      </c>
-      <c r="M52" s="1" t="inlineStr">
+      <c r="N52" s="1" t="inlineStr">
         <is>
           <t>N/A</t>
         </is>
@@ -5707,12 +5812,7 @@
           <t>227 Riverstone Dr, Canton, GA 30114, USA</t>
         </is>
       </c>
-      <c r="L53" s="1" t="inlineStr">
-        <is>
-          <t>N/A</t>
-        </is>
-      </c>
-      <c r="M53" s="1" t="inlineStr">
+      <c r="N53" s="1" t="inlineStr">
         <is>
           <t>N/A</t>
         </is>
@@ -5819,6 +5919,11 @@
           <t>Howard</t>
         </is>
       </c>
+      <c r="N54" t="inlineStr">
+        <is>
+          <t>Co-Founder &amp; OB/GYN (Owner)</t>
+        </is>
+      </c>
       <c r="Q54" t="n">
         <v>4.8</v>
       </c>
@@ -5911,12 +6016,7 @@
           <t>381 Deerfield Rd, Boone, NC 28607, USA</t>
         </is>
       </c>
-      <c r="L55" s="1" t="inlineStr">
-        <is>
-          <t>N/A</t>
-        </is>
-      </c>
-      <c r="M55" s="1" t="inlineStr">
+      <c r="N55" s="1" t="inlineStr">
         <is>
           <t>N/A</t>
         </is>
@@ -6013,12 +6113,7 @@
           <t>5161 Soquel Dr Ste C Floor 2, Soquel, CA 95073, USA</t>
         </is>
       </c>
-      <c r="L56" s="1" t="inlineStr">
-        <is>
-          <t>N/A</t>
-        </is>
-      </c>
-      <c r="M56" s="1" t="inlineStr">
+      <c r="N56" s="1" t="inlineStr">
         <is>
           <t>N/A</t>
         </is>
@@ -6115,12 +6210,7 @@
           <t>1875 Old Alabama Rd STE 210, Roswell, GA 30076, USA</t>
         </is>
       </c>
-      <c r="L57" s="1" t="inlineStr">
-        <is>
-          <t>N/A</t>
-        </is>
-      </c>
-      <c r="M57" s="1" t="inlineStr">
+      <c r="N57" s="1" t="inlineStr">
         <is>
           <t>N/A</t>
         </is>
@@ -6212,12 +6302,7 @@
           <t>8257 Fredericksburg Rd, San Antonio, TX 78229, USA</t>
         </is>
       </c>
-      <c r="L58" s="1" t="inlineStr">
-        <is>
-          <t>N/A</t>
-        </is>
-      </c>
-      <c r="M58" s="1" t="inlineStr">
+      <c r="N58" s="1" t="inlineStr">
         <is>
           <t>N/A</t>
         </is>

</xml_diff>

<commit_message>
Attempt to fill missing exec data from Deduped sheet
https://claude.ai/code/session_01917JoB1LXoWCAoYuucjGiV
</commit_message>
<xml_diff>
--- a/Womens_HRT_Hormones_Only_New_cleaned_updated.xlsx
+++ b/Womens_HRT_Hormones_Only_New_cleaned_updated.xlsx
@@ -1953,6 +1953,16 @@
           <t>8127 Mulberry Ave Ste 108</t>
         </is>
       </c>
+      <c r="L15" s="1" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="M15" s="1" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
       <c r="N15" s="1" t="inlineStr">
         <is>
           <t>N/A</t>
@@ -2448,6 +2458,16 @@
           <t>14115 S Dixie Hwy SUITE H, Palmetto Bay, FL 33176, USA</t>
         </is>
       </c>
+      <c r="L20" s="1" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="M20" s="1" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
       <c r="N20" s="1" t="inlineStr">
         <is>
           <t>N/A</t>
@@ -3553,6 +3573,16 @@
           <t>3405 Dallas Hwy Suite 200, Marietta, GA 30064, USA</t>
         </is>
       </c>
+      <c r="L31" s="1" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="M31" s="1" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
       <c r="N31" s="1" t="inlineStr">
         <is>
           <t>N/A</t>
@@ -3855,6 +3885,16 @@
           <t>90 W Main St, Victor, NY 14564, USA</t>
         </is>
       </c>
+      <c r="L34" s="1" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="M34" s="1" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
       <c r="N34" s="1" t="inlineStr">
         <is>
           <t>N/A</t>
@@ -3942,6 +3982,16 @@
           <t>1529 E Interstate 30 #108, Garland, TX 75043, USA</t>
         </is>
       </c>
+      <c r="L35" s="1" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="M35" s="1" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
       <c r="N35" s="1" t="inlineStr">
         <is>
           <t>N/A</t>
@@ -4786,6 +4836,11 @@
           <t>Kate</t>
         </is>
       </c>
+      <c r="M43" s="1" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
       <c r="N43" t="inlineStr">
         <is>
           <t>Founder &amp; Women's Health Nurse Practitioner / Certified Nurse Midwife</t>
@@ -4990,6 +5045,16 @@
           <t>2460 N Interstate 35 E Rd Suite 165, Waxahachie, TX 75165, USA</t>
         </is>
       </c>
+      <c r="L45" s="1" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="M45" s="1" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
       <c r="N45" s="1" t="inlineStr">
         <is>
           <t>N/A</t>
@@ -5090,6 +5155,16 @@
           <t>207 E 94th St 5th floor, New York, NY 10128, USA</t>
         </is>
       </c>
+      <c r="L46" s="1" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="M46" s="1" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
       <c r="N46" s="1" t="inlineStr">
         <is>
           <t>N/A</t>
@@ -5294,6 +5369,16 @@
           <t>3237 Blue Ridge Rd, Raleigh, NC 27612, USA</t>
         </is>
       </c>
+      <c r="L48" s="1" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="M48" s="1" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
       <c r="N48" s="1" t="inlineStr">
         <is>
           <t>N/A</t>
@@ -5715,6 +5800,16 @@
           <t>9940 Talbert Ave #303, Fountain Valley, CA 92708, USA</t>
         </is>
       </c>
+      <c r="L52" s="1" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="M52" s="1" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
       <c r="N52" s="1" t="inlineStr">
         <is>
           <t>N/A</t>
@@ -5812,6 +5907,16 @@
           <t>227 Riverstone Dr, Canton, GA 30114, USA</t>
         </is>
       </c>
+      <c r="L53" s="1" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="M53" s="1" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
       <c r="N53" s="1" t="inlineStr">
         <is>
           <t>N/A</t>
@@ -6016,6 +6121,16 @@
           <t>381 Deerfield Rd, Boone, NC 28607, USA</t>
         </is>
       </c>
+      <c r="L55" s="1" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="M55" s="1" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
       <c r="N55" s="1" t="inlineStr">
         <is>
           <t>N/A</t>
@@ -6113,6 +6228,16 @@
           <t>5161 Soquel Dr Ste C Floor 2, Soquel, CA 95073, USA</t>
         </is>
       </c>
+      <c r="L56" s="1" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="M56" s="1" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
       <c r="N56" s="1" t="inlineStr">
         <is>
           <t>N/A</t>
@@ -6210,6 +6335,16 @@
           <t>1875 Old Alabama Rd STE 210, Roswell, GA 30076, USA</t>
         </is>
       </c>
+      <c r="L57" s="1" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="M57" s="1" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
       <c r="N57" s="1" t="inlineStr">
         <is>
           <t>N/A</t>
@@ -6300,6 +6435,16 @@
       <c r="K58" t="inlineStr">
         <is>
           <t>8257 Fredericksburg Rd, San Antonio, TX 78229, USA</t>
+        </is>
+      </c>
+      <c r="L58" s="1" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="M58" s="1" t="inlineStr">
+        <is>
+          <t>N/A</t>
         </is>
       </c>
       <c r="N58" s="1" t="inlineStr">

</xml_diff>

<commit_message>
Update HRT worksheet CEO names using both CEO Results and Sheet2 sources
176/189 rows matched, 13 set to N/A

https://claude.ai/code/session_014asbHkxTUDGrdhYnv3KJp3
</commit_message>
<xml_diff>
--- a/Womens_HRT_Hormones_Only_New_cleaned_updated.xlsx
+++ b/Womens_HRT_Hormones_Only_New_cleaned_updated.xlsx
@@ -15856,12 +15856,12 @@
       </c>
       <c r="K31" t="inlineStr">
         <is>
-          <t>N/A</t>
+          <t>Julie</t>
         </is>
       </c>
       <c r="L31" t="inlineStr">
         <is>
-          <t>N/A</t>
+          <t>Morin</t>
         </is>
       </c>
     </row>
@@ -16511,12 +16511,12 @@
       </c>
       <c r="K51" t="inlineStr">
         <is>
-          <t>N/A</t>
+          <t>Michael</t>
         </is>
       </c>
       <c r="L51" t="inlineStr">
         <is>
-          <t>N/A</t>
+          <t>Litrel</t>
         </is>
       </c>
     </row>
@@ -16643,12 +16643,12 @@
       </c>
       <c r="K55" t="inlineStr">
         <is>
-          <t>N/A</t>
+          <t>Ken</t>
         </is>
       </c>
       <c r="L55" t="inlineStr">
         <is>
-          <t>N/A</t>
+          <t>Sinervo</t>
         </is>
       </c>
     </row>
@@ -16690,12 +16690,12 @@
       </c>
       <c r="K56" t="inlineStr">
         <is>
-          <t>N/A</t>
+          <t>Tina</t>
         </is>
       </c>
       <c r="L56" t="inlineStr">
         <is>
-          <t>N/A</t>
+          <t>Keshani</t>
         </is>
       </c>
     </row>
@@ -16727,12 +16727,12 @@
       </c>
       <c r="K57" t="inlineStr">
         <is>
-          <t>N/A</t>
+          <t>Stefany</t>
         </is>
       </c>
       <c r="L57" t="inlineStr">
         <is>
-          <t>N/A</t>
+          <t>Joustra</t>
         </is>
       </c>
     </row>
@@ -16769,12 +16769,12 @@
       </c>
       <c r="K58" t="inlineStr">
         <is>
-          <t>N/A</t>
+          <t>Tamer</t>
         </is>
       </c>
       <c r="L58" t="inlineStr">
         <is>
-          <t>N/A</t>
+          <t>Seckin</t>
         </is>
       </c>
     </row>
@@ -16811,12 +16811,12 @@
       </c>
       <c r="K59" t="inlineStr">
         <is>
-          <t>N/A</t>
+          <t>Cary</t>
         </is>
       </c>
       <c r="L59" t="inlineStr">
         <is>
-          <t>N/A</t>
+          <t>Veith</t>
         </is>
       </c>
     </row>
@@ -16858,12 +16858,12 @@
       </c>
       <c r="K60" t="inlineStr">
         <is>
-          <t>N/A</t>
+          <t>Kathleen</t>
         </is>
       </c>
       <c r="L60" t="inlineStr">
         <is>
-          <t>N/A</t>
+          <t>Valenton</t>
         </is>
       </c>
     </row>
@@ -16905,12 +16905,12 @@
       </c>
       <c r="K61" t="inlineStr">
         <is>
-          <t>N/A</t>
+          <t>Bri</t>
         </is>
       </c>
       <c r="L61" t="inlineStr">
         <is>
-          <t>N/A</t>
+          <t>Wyatt</t>
         </is>
       </c>
     </row>
@@ -16952,12 +16952,12 @@
       </c>
       <c r="K62" t="inlineStr">
         <is>
-          <t>N/A</t>
+          <t>Melvin</t>
         </is>
       </c>
       <c r="L62" t="inlineStr">
         <is>
-          <t>N/A</t>
+          <t>Ashford</t>
         </is>
       </c>
     </row>
@@ -16999,12 +16999,12 @@
       </c>
       <c r="K63" t="inlineStr">
         <is>
-          <t>N/A</t>
+          <t>Ryan</t>
         </is>
       </c>
       <c r="L63" t="inlineStr">
         <is>
-          <t>N/A</t>
+          <t>Stratford</t>
         </is>
       </c>
     </row>
@@ -17046,12 +17046,12 @@
       </c>
       <c r="K64" t="inlineStr">
         <is>
-          <t>N/A</t>
+          <t>Leslie</t>
         </is>
       </c>
       <c r="L64" t="inlineStr">
         <is>
-          <t>N/A</t>
+          <t>Jacobs</t>
         </is>
       </c>
     </row>
@@ -17093,12 +17093,12 @@
       </c>
       <c r="K65" t="inlineStr">
         <is>
-          <t>N/A</t>
+          <t>Matthew</t>
         </is>
       </c>
       <c r="L65" t="inlineStr">
         <is>
-          <t>N/A</t>
+          <t>Willis</t>
         </is>
       </c>
     </row>
@@ -17135,12 +17135,12 @@
       </c>
       <c r="K66" t="inlineStr">
         <is>
-          <t>N/A</t>
+          <t>Sarah</t>
         </is>
       </c>
       <c r="L66" t="inlineStr">
         <is>
-          <t>N/A</t>
+          <t>Adair</t>
         </is>
       </c>
     </row>
@@ -17182,12 +17182,12 @@
       </c>
       <c r="K67" t="inlineStr">
         <is>
-          <t>N/A</t>
+          <t>Tomo</t>
         </is>
       </c>
       <c r="L67" t="inlineStr">
         <is>
-          <t>N/A</t>
+          <t>Marjanovic</t>
         </is>
       </c>
     </row>
@@ -17224,12 +17224,12 @@
       </c>
       <c r="K68" t="inlineStr">
         <is>
-          <t>N/A</t>
+          <t>Aya</t>
         </is>
       </c>
       <c r="L68" t="inlineStr">
         <is>
-          <t>N/A</t>
+          <t>Rifai</t>
         </is>
       </c>
     </row>
@@ -17261,12 +17261,12 @@
       </c>
       <c r="K69" t="inlineStr">
         <is>
-          <t>N/A</t>
+          <t>George</t>
         </is>
       </c>
       <c r="L69" t="inlineStr">
         <is>
-          <t>N/A</t>
+          <t>Robison</t>
         </is>
       </c>
     </row>
@@ -17308,12 +17308,12 @@
       </c>
       <c r="K70" t="inlineStr">
         <is>
-          <t>N/A</t>
+          <t>Prithipal</t>
         </is>
       </c>
       <c r="L70" t="inlineStr">
         <is>
-          <t>N/A</t>
+          <t>Sethi</t>
         </is>
       </c>
     </row>
@@ -17355,12 +17355,12 @@
       </c>
       <c r="K71" t="inlineStr">
         <is>
-          <t>N/A</t>
+          <t>Jital</t>
         </is>
       </c>
       <c r="L71" t="inlineStr">
         <is>
-          <t>N/A</t>
+          <t>Pancholi</t>
         </is>
       </c>
     </row>
@@ -17402,12 +17402,12 @@
       </c>
       <c r="K72" t="inlineStr">
         <is>
-          <t>N/A</t>
+          <t>Nancy</t>
         </is>
       </c>
       <c r="L72" t="inlineStr">
         <is>
-          <t>N/A</t>
+          <t>Belcher</t>
         </is>
       </c>
     </row>
@@ -17449,12 +17449,12 @@
       </c>
       <c r="K73" t="inlineStr">
         <is>
-          <t>N/A</t>
+          <t>Elaine</t>
         </is>
       </c>
       <c r="L73" t="inlineStr">
         <is>
-          <t>N/A</t>
+          <t>Purcell</t>
         </is>
       </c>
     </row>
@@ -17496,12 +17496,12 @@
       </c>
       <c r="K74" t="inlineStr">
         <is>
-          <t>N/A</t>
+          <t>Alexa</t>
         </is>
       </c>
       <c r="L74" t="inlineStr">
         <is>
-          <t>N/A</t>
+          <t>Charbonneau</t>
         </is>
       </c>
     </row>
@@ -17543,12 +17543,12 @@
       </c>
       <c r="K75" t="inlineStr">
         <is>
-          <t>N/A</t>
+          <t>Brittanney</t>
         </is>
       </c>
       <c r="L75" t="inlineStr">
         <is>
-          <t>N/A</t>
+          <t>Sargent</t>
         </is>
       </c>
     </row>
@@ -17590,12 +17590,12 @@
       </c>
       <c r="K76" t="inlineStr">
         <is>
-          <t>N/A</t>
+          <t>Neil</t>
         </is>
       </c>
       <c r="L76" t="inlineStr">
         <is>
-          <t>N/A</t>
+          <t>King</t>
         </is>
       </c>
     </row>
@@ -17637,12 +17637,12 @@
       </c>
       <c r="K77" t="inlineStr">
         <is>
-          <t>N/A</t>
+          <t>Katie</t>
         </is>
       </c>
       <c r="L77" t="inlineStr">
         <is>
-          <t>N/A</t>
+          <t>Ferrington</t>
         </is>
       </c>
     </row>
@@ -17684,12 +17684,12 @@
       </c>
       <c r="K78" t="inlineStr">
         <is>
-          <t>N/A</t>
+          <t>Simone</t>
         </is>
       </c>
       <c r="L78" t="inlineStr">
         <is>
-          <t>N/A</t>
+          <t>Van-Horne</t>
         </is>
       </c>
     </row>
@@ -17731,12 +17731,12 @@
       </c>
       <c r="K79" t="inlineStr">
         <is>
-          <t>N/A</t>
+          <t>Guillaume</t>
         </is>
       </c>
       <c r="L79" t="inlineStr">
         <is>
-          <t>N/A</t>
+          <t>Cohen-Skalli</t>
         </is>
       </c>
     </row>
@@ -17778,12 +17778,12 @@
       </c>
       <c r="K80" t="inlineStr">
         <is>
-          <t>N/A</t>
+          <t>Melanie</t>
         </is>
       </c>
       <c r="L80" t="inlineStr">
         <is>
-          <t>N/A</t>
+          <t>Carminati</t>
         </is>
       </c>
     </row>
@@ -17825,12 +17825,12 @@
       </c>
       <c r="K81" t="inlineStr">
         <is>
-          <t>N/A</t>
+          <t>Steven</t>
         </is>
       </c>
       <c r="L81" t="inlineStr">
         <is>
-          <t>N/A</t>
+          <t>Campbell</t>
         </is>
       </c>
     </row>
@@ -17872,12 +17872,12 @@
       </c>
       <c r="K82" t="inlineStr">
         <is>
-          <t>N/A</t>
+          <t>Taylor</t>
         </is>
       </c>
       <c r="L82" t="inlineStr">
         <is>
-          <t>N/A</t>
+          <t>Blackwood</t>
         </is>
       </c>
     </row>
@@ -17914,12 +17914,12 @@
       </c>
       <c r="K83" t="inlineStr">
         <is>
-          <t>N/A</t>
+          <t>Eytan</t>
         </is>
       </c>
       <c r="L83" t="inlineStr">
         <is>
-          <t>N/A</t>
+          <t>Klepach</t>
         </is>
       </c>
     </row>
@@ -17956,12 +17956,12 @@
       </c>
       <c r="K84" t="inlineStr">
         <is>
-          <t>N/A</t>
+          <t>Chloe</t>
         </is>
       </c>
       <c r="L84" t="inlineStr">
         <is>
-          <t>N/A</t>
+          <t>Hooton</t>
         </is>
       </c>
     </row>
@@ -18003,12 +18003,12 @@
       </c>
       <c r="K85" t="inlineStr">
         <is>
-          <t>N/A</t>
+          <t>Michael</t>
         </is>
       </c>
       <c r="L85" t="inlineStr">
         <is>
-          <t>N/A</t>
+          <t>Ingber</t>
         </is>
       </c>
     </row>
@@ -18045,12 +18045,12 @@
       </c>
       <c r="K86" t="inlineStr">
         <is>
-          <t>N/A</t>
+          <t>Nicholas</t>
         </is>
       </c>
       <c r="L86" t="inlineStr">
         <is>
-          <t>N/A</t>
+          <t>Angelastro</t>
         </is>
       </c>
     </row>
@@ -18092,12 +18092,12 @@
       </c>
       <c r="K87" t="inlineStr">
         <is>
-          <t>N/A</t>
+          <t>Betty</t>
         </is>
       </c>
       <c r="L87" t="inlineStr">
         <is>
-          <t>N/A</t>
+          <t>Murray</t>
         </is>
       </c>
     </row>
@@ -18134,12 +18134,12 @@
       </c>
       <c r="K88" t="inlineStr">
         <is>
-          <t>N/A</t>
+          <t>Sonya</t>
         </is>
       </c>
       <c r="L88" t="inlineStr">
         <is>
-          <t>N/A</t>
+          <t>Ephraim</t>
         </is>
       </c>
     </row>
@@ -18181,12 +18181,12 @@
       </c>
       <c r="K89" t="inlineStr">
         <is>
-          <t>N/A</t>
+          <t>Kristin</t>
         </is>
       </c>
       <c r="L89" t="inlineStr">
         <is>
-          <t>N/A</t>
+          <t>Sapienza</t>
         </is>
       </c>
     </row>
@@ -18223,12 +18223,12 @@
       </c>
       <c r="K90" t="inlineStr">
         <is>
-          <t>N/A</t>
+          <t>Jennifer</t>
         </is>
       </c>
       <c r="L90" t="inlineStr">
         <is>
-          <t>N/A</t>
+          <t>Chiao</t>
         </is>
       </c>
     </row>
@@ -18270,12 +18270,12 @@
       </c>
       <c r="K91" t="inlineStr">
         <is>
-          <t>N/A</t>
+          <t>Sara</t>
         </is>
       </c>
       <c r="L91" t="inlineStr">
         <is>
-          <t>N/A</t>
+          <t>Moses</t>
         </is>
       </c>
     </row>
@@ -18312,12 +18312,12 @@
       </c>
       <c r="K92" t="inlineStr">
         <is>
-          <t>N/A</t>
+          <t>Susan</t>
         </is>
       </c>
       <c r="L92" t="inlineStr">
         <is>
-          <t>N/A</t>
+          <t>Davies</t>
         </is>
       </c>
     </row>
@@ -18354,12 +18354,12 @@
       </c>
       <c r="K93" t="inlineStr">
         <is>
-          <t>N/A</t>
+          <t>Soyini</t>
         </is>
       </c>
       <c r="L93" t="inlineStr">
         <is>
-          <t>N/A</t>
+          <t>Hawkins</t>
         </is>
       </c>
     </row>
@@ -18401,12 +18401,12 @@
       </c>
       <c r="K94" t="inlineStr">
         <is>
-          <t>N/A</t>
+          <t>Sam</t>
         </is>
       </c>
       <c r="L94" t="inlineStr">
         <is>
-          <t>N/A</t>
+          <t>Ridgeway</t>
         </is>
       </c>
     </row>
@@ -18443,12 +18443,12 @@
       </c>
       <c r="K95" t="inlineStr">
         <is>
-          <t>N/A</t>
+          <t>Judy</t>
         </is>
       </c>
       <c r="L95" t="inlineStr">
         <is>
-          <t>N/A</t>
+          <t>Yeh</t>
         </is>
       </c>
     </row>
@@ -18490,12 +18490,12 @@
       </c>
       <c r="K96" t="inlineStr">
         <is>
-          <t>N/A</t>
+          <t>Courtney</t>
         </is>
       </c>
       <c r="L96" t="inlineStr">
         <is>
-          <t>N/A</t>
+          <t>Clair</t>
         </is>
       </c>
     </row>
@@ -18537,12 +18537,12 @@
       </c>
       <c r="K97" t="inlineStr">
         <is>
-          <t>N/A</t>
+          <t>Christopher</t>
         </is>
       </c>
       <c r="L97" t="inlineStr">
         <is>
-          <t>N/A</t>
+          <t>Stolzman</t>
         </is>
       </c>
     </row>
@@ -18584,12 +18584,12 @@
       </c>
       <c r="K98" t="inlineStr">
         <is>
-          <t>N/A</t>
+          <t>Carly</t>
         </is>
       </c>
       <c r="L98" t="inlineStr">
         <is>
-          <t>N/A</t>
+          <t>Gossard</t>
         </is>
       </c>
     </row>
@@ -18626,12 +18626,12 @@
       </c>
       <c r="K99" t="inlineStr">
         <is>
-          <t>N/A</t>
+          <t>Ning</t>
         </is>
       </c>
       <c r="L99" t="inlineStr">
         <is>
-          <t>N/A</t>
+          <t>Wu</t>
         </is>
       </c>
     </row>
@@ -18673,12 +18673,12 @@
       </c>
       <c r="K100" t="inlineStr">
         <is>
-          <t>N/A</t>
+          <t>Suzanne</t>
         </is>
       </c>
       <c r="L100" t="inlineStr">
         <is>
-          <t>N/A</t>
+          <t>Slonim</t>
         </is>
       </c>
     </row>
@@ -18720,12 +18720,12 @@
       </c>
       <c r="K101" t="inlineStr">
         <is>
-          <t>N/A</t>
+          <t>Zvi</t>
         </is>
       </c>
       <c r="L101" t="inlineStr">
         <is>
-          <t>N/A</t>
+          <t>Schiffman</t>
         </is>
       </c>
     </row>
@@ -18762,12 +18762,12 @@
       </c>
       <c r="K102" t="inlineStr">
         <is>
-          <t>N/A</t>
+          <t>Cynthia</t>
         </is>
       </c>
       <c r="L102" t="inlineStr">
         <is>
-          <t>N/A</t>
+          <t>Tieche</t>
         </is>
       </c>
     </row>
@@ -18809,12 +18809,12 @@
       </c>
       <c r="K103" t="inlineStr">
         <is>
-          <t>N/A</t>
+          <t>Afua</t>
         </is>
       </c>
       <c r="L103" t="inlineStr">
         <is>
-          <t>N/A</t>
+          <t>Asemnor</t>
         </is>
       </c>
     </row>
@@ -18856,12 +18856,12 @@
       </c>
       <c r="K104" t="inlineStr">
         <is>
-          <t>N/A</t>
+          <t>Kenneth</t>
         </is>
       </c>
       <c r="L104" t="inlineStr">
         <is>
-          <t>N/A</t>
+          <t>Levey</t>
         </is>
       </c>
     </row>
@@ -18898,12 +18898,12 @@
       </c>
       <c r="K105" t="inlineStr">
         <is>
-          <t>N/A</t>
+          <t>William</t>
         </is>
       </c>
       <c r="L105" t="inlineStr">
         <is>
-          <t>N/A</t>
+          <t>Vereen</t>
         </is>
       </c>
     </row>
@@ -18940,12 +18940,12 @@
       </c>
       <c r="K106" t="inlineStr">
         <is>
-          <t>N/A</t>
+          <t>Jason</t>
         </is>
       </c>
       <c r="L106" t="inlineStr">
         <is>
-          <t>N/A</t>
+          <t>Wilson</t>
         </is>
       </c>
     </row>
@@ -18987,12 +18987,12 @@
       </c>
       <c r="K107" t="inlineStr">
         <is>
-          <t>N/A</t>
+          <t>Michele</t>
         </is>
       </c>
       <c r="L107" t="inlineStr">
         <is>
-          <t>N/A</t>
+          <t>Wispelwey</t>
         </is>
       </c>
     </row>
@@ -19029,12 +19029,12 @@
       </c>
       <c r="K108" t="inlineStr">
         <is>
-          <t>N/A</t>
+          <t>Amy</t>
         </is>
       </c>
       <c r="L108" t="inlineStr">
         <is>
-          <t>N/A</t>
+          <t>Stein</t>
         </is>
       </c>
     </row>
@@ -19076,12 +19076,12 @@
       </c>
       <c r="K109" t="inlineStr">
         <is>
-          <t>N/A</t>
+          <t>Natalya</t>
         </is>
       </c>
       <c r="L109" t="inlineStr">
         <is>
-          <t>N/A</t>
+          <t>Danilyants</t>
         </is>
       </c>
     </row>
@@ -19123,12 +19123,12 @@
       </c>
       <c r="K110" t="inlineStr">
         <is>
-          <t>N/A</t>
+          <t>Jonathan</t>
         </is>
       </c>
       <c r="L110" t="inlineStr">
         <is>
-          <t>N/A</t>
+          <t>Zaidan</t>
         </is>
       </c>
     </row>
@@ -19171,12 +19171,12 @@
       </c>
       <c r="K111" t="inlineStr">
         <is>
-          <t>N/A</t>
+          <t>Becky</t>
         </is>
       </c>
       <c r="L111" t="inlineStr">
         <is>
-          <t>N/A</t>
+          <t>Allen</t>
         </is>
       </c>
     </row>
@@ -19218,12 +19218,12 @@
       </c>
       <c r="K112" t="inlineStr">
         <is>
-          <t>N/A</t>
+          <t>Matt</t>
         </is>
       </c>
       <c r="L112" t="inlineStr">
         <is>
-          <t>N/A</t>
+          <t>Jones</t>
         </is>
       </c>
     </row>
@@ -19265,12 +19265,12 @@
       </c>
       <c r="K113" t="inlineStr">
         <is>
-          <t>N/A</t>
+          <t>Terri-Ann</t>
         </is>
       </c>
       <c r="L113" t="inlineStr">
         <is>
-          <t>N/A</t>
+          <t>Samuels</t>
         </is>
       </c>
     </row>
@@ -19307,12 +19307,12 @@
       </c>
       <c r="K114" t="inlineStr">
         <is>
-          <t>N/A</t>
+          <t>Rachael</t>
         </is>
       </c>
       <c r="L114" t="inlineStr">
         <is>
-          <t>N/A</t>
+          <t>DelToro</t>
         </is>
       </c>
     </row>
@@ -19354,12 +19354,12 @@
       </c>
       <c r="K115" t="inlineStr">
         <is>
-          <t>N/A</t>
+          <t>Joseph</t>
         </is>
       </c>
       <c r="L115" t="inlineStr">
         <is>
-          <t>N/A</t>
+          <t>Franzese</t>
         </is>
       </c>
     </row>
@@ -19396,12 +19396,12 @@
       </c>
       <c r="K116" t="inlineStr">
         <is>
-          <t>N/A</t>
+          <t>Rodolfo</t>
         </is>
       </c>
       <c r="L116" t="inlineStr">
         <is>
-          <t>N/A</t>
+          <t>Hanabergh</t>
         </is>
       </c>
     </row>
@@ -19443,12 +19443,12 @@
       </c>
       <c r="K117" t="inlineStr">
         <is>
-          <t>N/A</t>
+          <t>Sogol</t>
         </is>
       </c>
       <c r="L117" t="inlineStr">
         <is>
-          <t>N/A</t>
+          <t>Jahedi</t>
         </is>
       </c>
     </row>
@@ -19490,12 +19490,12 @@
       </c>
       <c r="K118" t="inlineStr">
         <is>
-          <t>N/A</t>
+          <t>Rob</t>
         </is>
       </c>
       <c r="L118" t="inlineStr">
         <is>
-          <t>N/A</t>
+          <t>Dilillo</t>
         </is>
       </c>
     </row>
@@ -19537,12 +19537,12 @@
       </c>
       <c r="K119" t="inlineStr">
         <is>
-          <t>N/A</t>
+          <t>Dan</t>
         </is>
       </c>
       <c r="L119" t="inlineStr">
         <is>
-          <t>N/A</t>
+          <t>Deneui</t>
         </is>
       </c>
     </row>
@@ -19626,12 +19626,12 @@
       </c>
       <c r="K121" t="inlineStr">
         <is>
-          <t>N/A</t>
+          <t>Kristina</t>
         </is>
       </c>
       <c r="L121" t="inlineStr">
         <is>
-          <t>N/A</t>
+          <t>Smith</t>
         </is>
       </c>
     </row>
@@ -19673,12 +19673,12 @@
       </c>
       <c r="K122" t="inlineStr">
         <is>
-          <t>N/A</t>
+          <t>Candice</t>
         </is>
       </c>
       <c r="L122" t="inlineStr">
         <is>
-          <t>N/A</t>
+          <t>Sittert</t>
         </is>
       </c>
     </row>
@@ -19720,12 +19720,12 @@
       </c>
       <c r="K123" t="inlineStr">
         <is>
-          <t>N/A</t>
+          <t>Diana</t>
         </is>
       </c>
       <c r="L123" t="inlineStr">
         <is>
-          <t>N/A</t>
+          <t>Bitner</t>
         </is>
       </c>
     </row>
@@ -19762,12 +19762,12 @@
       </c>
       <c r="K124" t="inlineStr">
         <is>
-          <t>N/A</t>
+          <t>Shawanda</t>
         </is>
       </c>
       <c r="L124" t="inlineStr">
         <is>
-          <t>N/A</t>
+          <t>Obey</t>
         </is>
       </c>
     </row>
@@ -19809,12 +19809,12 @@
       </c>
       <c r="K125" t="inlineStr">
         <is>
-          <t>N/A</t>
+          <t>Derek</t>
         </is>
       </c>
       <c r="L125" t="inlineStr">
         <is>
-          <t>N/A</t>
+          <t>Petry</t>
         </is>
       </c>
     </row>
@@ -19856,12 +19856,12 @@
       </c>
       <c r="K126" t="inlineStr">
         <is>
-          <t>N/A</t>
+          <t>Travis</t>
         </is>
       </c>
       <c r="L126" t="inlineStr">
         <is>
-          <t>N/A</t>
+          <t>Deuson</t>
         </is>
       </c>
     </row>
@@ -19898,12 +19898,12 @@
       </c>
       <c r="K127" t="inlineStr">
         <is>
-          <t>N/A</t>
+          <t>Cindy</t>
         </is>
       </c>
       <c r="L127" t="inlineStr">
         <is>
-          <t>N/A</t>
+          <t>Mosbrucker</t>
         </is>
       </c>
     </row>
@@ -19940,12 +19940,12 @@
       </c>
       <c r="K128" t="inlineStr">
         <is>
-          <t>N/A</t>
+          <t>Nicole</t>
         </is>
       </c>
       <c r="L128" t="inlineStr">
         <is>
-          <t>N/A</t>
+          <t>Kretzer</t>
         </is>
       </c>
     </row>
@@ -19987,12 +19987,12 @@
       </c>
       <c r="K129" t="inlineStr">
         <is>
-          <t>N/A</t>
+          <t>Andrew</t>
         </is>
       </c>
       <c r="L129" t="inlineStr">
         <is>
-          <t>N/A</t>
+          <t>Goldstein</t>
         </is>
       </c>
     </row>
@@ -20034,12 +20034,12 @@
       </c>
       <c r="K130" t="inlineStr">
         <is>
-          <t>N/A</t>
+          <t>Molly</t>
         </is>
       </c>
       <c r="L130" t="inlineStr">
         <is>
-          <t>N/A</t>
+          <t>Galbraith</t>
         </is>
       </c>
     </row>
@@ -20081,12 +20081,12 @@
       </c>
       <c r="K131" t="inlineStr">
         <is>
-          <t>N/A</t>
+          <t>Laura</t>
         </is>
       </c>
       <c r="L131" t="inlineStr">
         <is>
-          <t>N/A</t>
+          <t>Currens</t>
         </is>
       </c>
     </row>
@@ -20128,12 +20128,12 @@
       </c>
       <c r="K132" t="inlineStr">
         <is>
-          <t>N/A</t>
+          <t>Matthew</t>
         </is>
       </c>
       <c r="L132" t="inlineStr">
         <is>
-          <t>N/A</t>
+          <t>Spellman</t>
         </is>
       </c>
     </row>
@@ -20175,12 +20175,12 @@
       </c>
       <c r="K133" t="inlineStr">
         <is>
-          <t>N/A</t>
+          <t>Wayne</t>
         </is>
       </c>
       <c r="L133" t="inlineStr">
         <is>
-          <t>N/A</t>
+          <t>Wilson</t>
         </is>
       </c>
     </row>
@@ -20222,12 +20222,12 @@
       </c>
       <c r="K134" t="inlineStr">
         <is>
-          <t>N/A</t>
+          <t>Amanda</t>
         </is>
       </c>
       <c r="L134" t="inlineStr">
         <is>
-          <t>N/A</t>
+          <t>Thompson</t>
         </is>
       </c>
     </row>
@@ -20259,12 +20259,12 @@
       </c>
       <c r="K135" t="inlineStr">
         <is>
-          <t>N/A</t>
+          <t>Monica</t>
         </is>
       </c>
       <c r="L135" t="inlineStr">
         <is>
-          <t>N/A</t>
+          <t>Barker</t>
         </is>
       </c>
     </row>
@@ -20306,12 +20306,12 @@
       </c>
       <c r="K136" t="inlineStr">
         <is>
-          <t>N/A</t>
+          <t>Brian</t>
         </is>
       </c>
       <c r="L136" t="inlineStr">
         <is>
-          <t>N/A</t>
+          <t>Pryor</t>
         </is>
       </c>
     </row>
@@ -20353,12 +20353,12 @@
       </c>
       <c r="K137" t="inlineStr">
         <is>
-          <t>N/A</t>
+          <t>Willem</t>
         </is>
       </c>
       <c r="L137" t="inlineStr">
         <is>
-          <t>N/A</t>
+          <t>Stegeman</t>
         </is>
       </c>
     </row>
@@ -20400,12 +20400,12 @@
       </c>
       <c r="K138" t="inlineStr">
         <is>
-          <t>N/A</t>
+          <t>Steven</t>
         </is>
       </c>
       <c r="L138" t="inlineStr">
         <is>
-          <t>N/A</t>
+          <t>Previte</t>
         </is>
       </c>
     </row>
@@ -20447,12 +20447,12 @@
       </c>
       <c r="K139" t="inlineStr">
         <is>
-          <t>N/A</t>
+          <t>Edward</t>
         </is>
       </c>
       <c r="L139" t="inlineStr">
         <is>
-          <t>N/A</t>
+          <t>Gheiler</t>
         </is>
       </c>
     </row>
@@ -20494,12 +20494,12 @@
       </c>
       <c r="K140" t="inlineStr">
         <is>
-          <t>N/A</t>
+          <t>Jasen</t>
         </is>
       </c>
       <c r="L140" t="inlineStr">
         <is>
-          <t>N/A</t>
+          <t>Bruce</t>
         </is>
       </c>
     </row>
@@ -20541,12 +20541,12 @@
       </c>
       <c r="K141" t="inlineStr">
         <is>
-          <t>N/A</t>
+          <t>Ashlee</t>
         </is>
       </c>
       <c r="L141" t="inlineStr">
         <is>
-          <t>N/A</t>
+          <t>Roderick</t>
         </is>
       </c>
     </row>
@@ -20588,12 +20588,12 @@
       </c>
       <c r="K142" t="inlineStr">
         <is>
-          <t>N/A</t>
+          <t>Jennifer</t>
         </is>
       </c>
       <c r="L142" t="inlineStr">
         <is>
-          <t>N/A</t>
+          <t>Hungate</t>
         </is>
       </c>
     </row>
@@ -20635,12 +20635,12 @@
       </c>
       <c r="K143" t="inlineStr">
         <is>
-          <t>N/A</t>
+          <t>Jill</t>
         </is>
       </c>
       <c r="L143" t="inlineStr">
         <is>
-          <t>N/A</t>
+          <t>Gustafson</t>
         </is>
       </c>
     </row>
@@ -20682,12 +20682,12 @@
       </c>
       <c r="K144" t="inlineStr">
         <is>
-          <t>N/A</t>
+          <t>Jill</t>
         </is>
       </c>
       <c r="L144" t="inlineStr">
         <is>
-          <t>N/A</t>
+          <t>Angelo</t>
         </is>
       </c>
     </row>
@@ -20729,12 +20729,12 @@
       </c>
       <c r="K145" t="inlineStr">
         <is>
-          <t>N/A</t>
+          <t>Justin</t>
         </is>
       </c>
       <c r="L145" t="inlineStr">
         <is>
-          <t>N/A</t>
+          <t>Bing</t>
         </is>
       </c>
     </row>
@@ -20771,12 +20771,12 @@
       </c>
       <c r="K146" t="inlineStr">
         <is>
-          <t>N/A</t>
+          <t>Michael</t>
         </is>
       </c>
       <c r="L146" t="inlineStr">
         <is>
-          <t>N/A</t>
+          <t>Zahalsky</t>
         </is>
       </c>
     </row>
@@ -20818,12 +20818,12 @@
       </c>
       <c r="K147" t="inlineStr">
         <is>
-          <t>N/A</t>
+          <t>Hughan</t>
         </is>
       </c>
       <c r="L147" t="inlineStr">
         <is>
-          <t>N/A</t>
+          <t>Frederick</t>
         </is>
       </c>
     </row>
@@ -20865,12 +20865,12 @@
       </c>
       <c r="K148" t="inlineStr">
         <is>
-          <t>N/A</t>
+          <t>Munir</t>
         </is>
       </c>
       <c r="L148" t="inlineStr">
         <is>
-          <t>N/A</t>
+          <t>Ahmad</t>
         </is>
       </c>
     </row>
@@ -20912,12 +20912,12 @@
       </c>
       <c r="K149" t="inlineStr">
         <is>
-          <t>N/A</t>
+          <t>Jim</t>
         </is>
       </c>
       <c r="L149" t="inlineStr">
         <is>
-          <t>N/A</t>
+          <t>Sherman</t>
         </is>
       </c>
     </row>
@@ -20954,12 +20954,12 @@
       </c>
       <c r="K150" t="inlineStr">
         <is>
-          <t>N/A</t>
+          <t>Azita</t>
         </is>
       </c>
       <c r="L150" t="inlineStr">
         <is>
-          <t>N/A</t>
+          <t>Pakravan</t>
         </is>
       </c>
     </row>
@@ -20996,12 +20996,12 @@
       </c>
       <c r="K151" t="inlineStr">
         <is>
-          <t>N/A</t>
+          <t>Kathryn</t>
         </is>
       </c>
       <c r="L151" t="inlineStr">
         <is>
-          <t>N/A</t>
+          <t>Lester</t>
         </is>
       </c>
     </row>
@@ -21043,12 +21043,12 @@
       </c>
       <c r="K152" t="inlineStr">
         <is>
-          <t>N/A</t>
+          <t>David</t>
         </is>
       </c>
       <c r="L152" t="inlineStr">
         <is>
-          <t>N/A</t>
+          <t>Carmichael</t>
         </is>
       </c>
     </row>
@@ -21090,12 +21090,12 @@
       </c>
       <c r="K153" t="inlineStr">
         <is>
-          <t>N/A</t>
+          <t>Luis</t>
         </is>
       </c>
       <c r="L153" t="inlineStr">
         <is>
-          <t>N/A</t>
+          <t>Gomez</t>
         </is>
       </c>
     </row>
@@ -21137,12 +21137,12 @@
       </c>
       <c r="K154" t="inlineStr">
         <is>
-          <t>N/A</t>
+          <t>Scott</t>
         </is>
       </c>
       <c r="L154" t="inlineStr">
         <is>
-          <t>N/A</t>
+          <t>Armstrong</t>
         </is>
       </c>
     </row>
@@ -21184,12 +21184,12 @@
       </c>
       <c r="K155" t="inlineStr">
         <is>
-          <t>N/A</t>
+          <t>Stephanie</t>
         </is>
       </c>
       <c r="L155" t="inlineStr">
         <is>
-          <t>N/A</t>
+          <t>Prendergast</t>
         </is>
       </c>
     </row>
@@ -21231,12 +21231,12 @@
       </c>
       <c r="K156" t="inlineStr">
         <is>
-          <t>N/A</t>
+          <t>Amanda</t>
         </is>
       </c>
       <c r="L156" t="inlineStr">
         <is>
-          <t>N/A</t>
+          <t>Neri</t>
         </is>
       </c>
     </row>
@@ -21278,12 +21278,12 @@
       </c>
       <c r="K157" t="inlineStr">
         <is>
-          <t>N/A</t>
+          <t>Joshua</t>
         </is>
       </c>
       <c r="L157" t="inlineStr">
         <is>
-          <t>N/A</t>
+          <t>Host</t>
         </is>
       </c>
     </row>
@@ -21325,12 +21325,12 @@
       </c>
       <c r="K158" t="inlineStr">
         <is>
-          <t>N/A</t>
+          <t>Courtney</t>
         </is>
       </c>
       <c r="L158" t="inlineStr">
         <is>
-          <t>N/A</t>
+          <t>Lo</t>
         </is>
       </c>
     </row>
@@ -21372,12 +21372,12 @@
       </c>
       <c r="K159" t="inlineStr">
         <is>
-          <t>N/A</t>
+          <t>Adeeti</t>
         </is>
       </c>
       <c r="L159" t="inlineStr">
         <is>
-          <t>N/A</t>
+          <t>Gupta</t>
         </is>
       </c>
     </row>
@@ -21414,12 +21414,12 @@
       </c>
       <c r="K160" t="inlineStr">
         <is>
-          <t>N/A</t>
+          <t>Malathi</t>
         </is>
       </c>
       <c r="L160" t="inlineStr">
         <is>
-          <t>N/A</t>
+          <t>Ellis</t>
         </is>
       </c>
     </row>
@@ -21456,12 +21456,12 @@
       </c>
       <c r="K161" t="inlineStr">
         <is>
-          <t>N/A</t>
+          <t>Babette</t>
         </is>
       </c>
       <c r="L161" t="inlineStr">
         <is>
-          <t>N/A</t>
+          <t>Clough</t>
         </is>
       </c>
     </row>
@@ -21503,12 +21503,12 @@
       </c>
       <c r="K162" t="inlineStr">
         <is>
-          <t>N/A</t>
+          <t>Justin</t>
         </is>
       </c>
       <c r="L162" t="inlineStr">
         <is>
-          <t>N/A</t>
+          <t>Bucki</t>
         </is>
       </c>
     </row>
@@ -21550,12 +21550,12 @@
       </c>
       <c r="K163" t="inlineStr">
         <is>
-          <t>N/A</t>
+          <t>Tim</t>
         </is>
       </c>
       <c r="L163" t="inlineStr">
         <is>
-          <t>N/A</t>
+          <t>Patel</t>
         </is>
       </c>
     </row>
@@ -21597,12 +21597,12 @@
       </c>
       <c r="K164" t="inlineStr">
         <is>
-          <t>N/A</t>
+          <t>Bruce</t>
         </is>
       </c>
       <c r="L164" t="inlineStr">
         <is>
-          <t>N/A</t>
+          <t>Akright</t>
         </is>
       </c>
     </row>
@@ -21644,12 +21644,12 @@
       </c>
       <c r="K165" t="inlineStr">
         <is>
-          <t>N/A</t>
+          <t>Heather</t>
         </is>
       </c>
       <c r="L165" t="inlineStr">
         <is>
-          <t>N/A</t>
+          <t>Jeffcoat</t>
         </is>
       </c>
     </row>
@@ -21686,12 +21686,12 @@
       </c>
       <c r="K166" t="inlineStr">
         <is>
-          <t>N/A</t>
+          <t>Jonathan</t>
         </is>
       </c>
       <c r="L166" t="inlineStr">
         <is>
-          <t>N/A</t>
+          <t>Beilan</t>
         </is>
       </c>
     </row>
@@ -21728,12 +21728,12 @@
       </c>
       <c r="K167" t="inlineStr">
         <is>
-          <t>N/A</t>
+          <t>Leslie</t>
         </is>
       </c>
       <c r="L167" t="inlineStr">
         <is>
-          <t>N/A</t>
+          <t>Jacobs</t>
         </is>
       </c>
     </row>
@@ -21770,12 +21770,12 @@
       </c>
       <c r="K168" t="inlineStr">
         <is>
-          <t>N/A</t>
+          <t>Amy</t>
         </is>
       </c>
       <c r="L168" t="inlineStr">
         <is>
-          <t>N/A</t>
+          <t>Newberry</t>
         </is>
       </c>
     </row>
@@ -21817,12 +21817,12 @@
       </c>
       <c r="K169" t="inlineStr">
         <is>
-          <t>N/A</t>
+          <t>Ian</t>
         </is>
       </c>
       <c r="L169" t="inlineStr">
         <is>
-          <t>N/A</t>
+          <t>Kornbluth</t>
         </is>
       </c>
     </row>
@@ -21864,12 +21864,12 @@
       </c>
       <c r="K170" t="inlineStr">
         <is>
-          <t>N/A</t>
+          <t>Erica</t>
         </is>
       </c>
       <c r="L170" t="inlineStr">
         <is>
-          <t>N/A</t>
+          <t>Michitsch</t>
         </is>
       </c>
     </row>
@@ -21911,12 +21911,12 @@
       </c>
       <c r="K171" t="inlineStr">
         <is>
-          <t>N/A</t>
+          <t>Solafa</t>
         </is>
       </c>
       <c r="L171" t="inlineStr">
         <is>
-          <t>N/A</t>
+          <t>Elshatanoufy</t>
         </is>
       </c>
     </row>
@@ -21958,12 +21958,12 @@
       </c>
       <c r="K172" t="inlineStr">
         <is>
-          <t>N/A</t>
+          <t>John</t>
         </is>
       </c>
       <c r="L172" t="inlineStr">
         <is>
-          <t>N/A</t>
+          <t>Hennessy</t>
         </is>
       </c>
     </row>
@@ -22005,12 +22005,12 @@
       </c>
       <c r="K173" t="inlineStr">
         <is>
-          <t>N/A</t>
+          <t>Katie</t>
         </is>
       </c>
       <c r="L173" t="inlineStr">
         <is>
-          <t>N/A</t>
+          <t>Mcmanigal</t>
         </is>
       </c>
     </row>
@@ -22052,12 +22052,12 @@
       </c>
       <c r="K174" t="inlineStr">
         <is>
-          <t>N/A</t>
+          <t>Jana</t>
         </is>
       </c>
       <c r="L174" t="inlineStr">
         <is>
-          <t>N/A</t>
+          <t>Richardson</t>
         </is>
       </c>
     </row>
@@ -22094,12 +22094,12 @@
       </c>
       <c r="K175" t="inlineStr">
         <is>
-          <t>N/A</t>
+          <t>Katherine</t>
         </is>
       </c>
       <c r="L175" t="inlineStr">
         <is>
-          <t>N/A</t>
+          <t>Pace</t>
         </is>
       </c>
     </row>
@@ -22136,12 +22136,12 @@
       </c>
       <c r="K176" t="inlineStr">
         <is>
-          <t>N/A</t>
+          <t>Jennifer</t>
         </is>
       </c>
       <c r="L176" t="inlineStr">
         <is>
-          <t>N/A</t>
+          <t>Huddleston</t>
         </is>
       </c>
     </row>
@@ -22173,12 +22173,12 @@
       </c>
       <c r="K177" t="inlineStr">
         <is>
-          <t>N/A</t>
+          <t>Deborah</t>
         </is>
       </c>
       <c r="L177" t="inlineStr">
         <is>
-          <t>N/A</t>
+          <t>Lenart</t>
         </is>
       </c>
     </row>
@@ -22220,12 +22220,12 @@
       </c>
       <c r="K178" t="inlineStr">
         <is>
-          <t>N/A</t>
+          <t>Deborah</t>
         </is>
       </c>
       <c r="L178" t="inlineStr">
         <is>
-          <t>N/A</t>
+          <t>Wilson</t>
         </is>
       </c>
     </row>
@@ -22267,12 +22267,12 @@
       </c>
       <c r="K179" t="inlineStr">
         <is>
-          <t>N/A</t>
+          <t>Brett</t>
         </is>
       </c>
       <c r="L179" t="inlineStr">
         <is>
-          <t>N/A</t>
+          <t>Enabnit</t>
         </is>
       </c>
     </row>
@@ -22314,12 +22314,12 @@
       </c>
       <c r="K180" t="inlineStr">
         <is>
-          <t>N/A</t>
+          <t>Kristian</t>
         </is>
       </c>
       <c r="L180" t="inlineStr">
         <is>
-          <t>N/A</t>
+          <t>Marcial</t>
         </is>
       </c>
     </row>
@@ -22361,12 +22361,12 @@
       </c>
       <c r="K181" t="inlineStr">
         <is>
-          <t>N/A</t>
+          <t>Judith</t>
         </is>
       </c>
       <c r="L181" t="inlineStr">
         <is>
-          <t>N/A</t>
+          <t>Meer</t>
         </is>
       </c>
     </row>
@@ -22408,12 +22408,12 @@
       </c>
       <c r="K182" t="inlineStr">
         <is>
-          <t>N/A</t>
+          <t>Nick</t>
         </is>
       </c>
       <c r="L182" t="inlineStr">
         <is>
-          <t>N/A</t>
+          <t>Cutri</t>
         </is>
       </c>
     </row>
@@ -22455,12 +22455,12 @@
       </c>
       <c r="K183" t="inlineStr">
         <is>
-          <t>N/A</t>
+          <t>Rolando</t>
         </is>
       </c>
       <c r="L183" t="inlineStr">
         <is>
-          <t>N/A</t>
+          <t>Alvarez</t>
         </is>
       </c>
     </row>
@@ -22502,12 +22502,12 @@
       </c>
       <c r="K184" t="inlineStr">
         <is>
-          <t>N/A</t>
+          <t>Stephen</t>
         </is>
       </c>
       <c r="L184" t="inlineStr">
         <is>
-          <t>N/A</t>
+          <t>Gabelich</t>
         </is>
       </c>
     </row>
@@ -22549,12 +22549,12 @@
       </c>
       <c r="K185" t="inlineStr">
         <is>
-          <t>N/A</t>
+          <t>Christi</t>
         </is>
       </c>
       <c r="L185" t="inlineStr">
         <is>
-          <t>N/A</t>
+          <t>Pramudji-Dawe</t>
         </is>
       </c>
     </row>
@@ -22591,12 +22591,12 @@
       </c>
       <c r="K186" t="inlineStr">
         <is>
-          <t>N/A</t>
+          <t>David</t>
         </is>
       </c>
       <c r="L186" t="inlineStr">
         <is>
-          <t>N/A</t>
+          <t>Bernstein</t>
         </is>
       </c>
     </row>
@@ -22623,12 +22623,12 @@
       </c>
       <c r="K187" t="inlineStr">
         <is>
-          <t>N/A</t>
+          <t>Diana</t>
         </is>
       </c>
       <c r="L187" t="inlineStr">
         <is>
-          <t>N/A</t>
+          <t>Rushlow (There are three more founders. Shared ownership)</t>
         </is>
       </c>
     </row>
@@ -22660,12 +22660,12 @@
       </c>
       <c r="K188" t="inlineStr">
         <is>
-          <t>N/A</t>
+          <t>Michael</t>
         </is>
       </c>
       <c r="L188" t="inlineStr">
         <is>
-          <t>N/A</t>
+          <t>Brookins</t>
         </is>
       </c>
     </row>
@@ -22707,12 +22707,12 @@
       </c>
       <c r="K189" t="inlineStr">
         <is>
-          <t>N/A</t>
+          <t>Hollie</t>
         </is>
       </c>
       <c r="L189" t="inlineStr">
         <is>
-          <t>N/A</t>
+          <t>Neujahr</t>
         </is>
       </c>
     </row>
@@ -22754,12 +22754,12 @@
       </c>
       <c r="K190" t="inlineStr">
         <is>
-          <t>N/A</t>
+          <t>Ijeoma</t>
         </is>
       </c>
       <c r="L190" t="inlineStr">
         <is>
-          <t>N/A</t>
+          <t>Nwankpa</t>
         </is>
       </c>
     </row>

</xml_diff>